<commit_message>
add function ramp on E4648A
</commit_message>
<xml_diff>
--- a/IVM6311_Testing_scripts.xlsx
+++ b/IVM6311_Testing_scripts.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\invlab\Documents\IVM6311ATE\IVM6311ATE\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94F37258-3DDD-4705-832D-A4E55C033317}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9AE321D6-0E39-4A77-A663-78EFD2658DA9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="693" firstSheet="1" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -29419,692 +29419,6 @@
   <si>
     <r>
       <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FFFF3399"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">Run__startup
-Run__Boost_test_default
-Run__Enable_Ana_Testpoint
-Wait__delay__0.1ms
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FFFF3399"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">
-Force__VBIAS__5V
-Force__VBSO__4.5V
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF4472C4"/>
-        <rFont val="Calibri"/>
-      </rPr>
-      <t xml:space="preserve">
-0xFE_0x00 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>"Select page 0"</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF4472C4"/>
-        <rFont val="Calibri"/>
-      </rPr>
-      <t xml:space="preserve">
-0x00_0x0F</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-      </rPr>
-      <t xml:space="preserve"> "Power-up"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF4472C4"/>
-        <rFont val="Calibri"/>
-      </rPr>
-      <t>0xB0_0x00</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-      </rPr>
-      <t xml:space="preserve"> "en 1 bst low"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF4472C4"/>
-        <rFont val="Calibri"/>
-      </rPr>
-      <t>0xB1_0x00</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-      </rPr>
-      <t xml:space="preserve"> "en 2 bst low"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF4472C4"/>
-        <rFont val="Calibri"/>
-      </rPr>
-      <t>0xB3[4:3]_0x00</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-      </rPr>
-      <t xml:space="preserve"> "en 3 bst low"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF4472C4"/>
-        <rFont val="Calibri"/>
-      </rPr>
-      <t xml:space="preserve">
-0xFE_0x01</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-      </rPr>
-      <t xml:space="preserve"> "Select page 1"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF4472C4"/>
-        <rFont val="Calibri"/>
-      </rPr>
-      <t>0x2F_0xAA</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-      </rPr>
-      <t xml:space="preserve"> "Unlock test page"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF4472C4"/>
-        <rFont val="Calibri"/>
-      </rPr>
-      <t>0x2F_0xBB</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-      </rPr>
-      <t xml:space="preserve"> "Unlock test page"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF4472C4"/>
-        <rFont val="Calibri"/>
-      </rPr>
-      <t xml:space="preserve">
-0x18[6]_0x01</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-      </rPr>
-      <t xml:space="preserve"> "Enable Mirr"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF4472C4"/>
-        <rFont val="Calibri"/>
-      </rPr>
-      <t>0xFE_0x00</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-      </rPr>
-      <t xml:space="preserve"> "Select page 0"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF4472C4"/>
-        <rFont val="Calibri"/>
-      </rPr>
-      <t>0xB1[6]_0x01</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-      </rPr>
-      <t xml:space="preserve"> "Bootstrap en"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF4472C4"/>
-        <rFont val="Calibri"/>
-      </rPr>
-      <t>0xB2[1]_0x00</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-      </rPr>
-      <t xml:space="preserve"> "ls_sel off"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF4472C4"/>
-        <rFont val="Calibri"/>
-      </rPr>
-      <t>0xB4[2:0]_0x04</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-      </rPr>
-      <t xml:space="preserve"> "hsb on hsa_byp off"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF4472C4"/>
-        <rFont val="Calibri"/>
-      </rPr>
-      <t xml:space="preserve">0xB0[0]_0x01 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-      </rPr>
-      <t xml:space="preserve">"bst general en"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF4472C4"/>
-        <rFont val="Calibri"/>
-      </rPr>
-      <t>0xFE_0x01</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-      </rPr>
-      <t xml:space="preserve"> "Select page 1"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF4472C4"/>
-        <rFont val="Calibri"/>
-      </rPr>
-      <t>0x1A_0x03</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-      </rPr>
-      <t xml:space="preserve"> "ana test TSW drive"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF4472C4"/>
-        <rFont val="Calibri"/>
-      </rPr>
-      <t>0x03_0x05</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-      </rPr>
-      <t xml:space="preserve"> "FSYN and SDI TMUX"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF4472C4"/>
-        <rFont val="Calibri"/>
-      </rPr>
-      <t>0x04_0x14</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-      </rPr>
-      <t xml:space="preserve"> "dig test EN FSYN=bst_bootstrap_comp_out SDI=low_on"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF4472C4"/>
-        <rFont val="Calibri"/>
-      </rPr>
-      <t>0x17[6]_0x01</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-      </rPr>
-      <t xml:space="preserve"> "Force Mirr"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF4472C4"/>
-        <rFont val="Calibri"/>
-      </rPr>
-      <t>0x16[6]_0x01</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-      </rPr>
-      <t xml:space="preserve"> "Force Bootstrap"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF4472C4"/>
-        <rFont val="Calibri"/>
-      </rPr>
-      <t>0xFE_0x00</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-      </rPr>
-      <t xml:space="preserve"> "Select page 0"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF7030A0"/>
-        <rFont val="Calibri"/>
-      </rPr>
-      <t xml:space="preserve">
-Wait__delay__0.1ms
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF4472C4"/>
-        <rFont val="Calibri"/>
-      </rPr>
-      <t xml:space="preserve">
-0xB2[0]_0x01</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF7030A0"/>
-        <rFont val="Calibri"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-      </rPr>
-      <t xml:space="preserve">"Power Force en"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF4472C4"/>
-        <rFont val="Calibri"/>
-      </rPr>
-      <t>0xFE_0x01</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF7030A0"/>
-        <rFont val="Calibri"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-      </rPr>
-      <t xml:space="preserve">"Select page 1"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF4472C4"/>
-        <rFont val="Calibri"/>
-      </rPr>
-      <t>0x15[4]_0x01</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-      </rPr>
-      <t xml:space="preserve"> "Force bst general en"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF7030A0"/>
-        <rFont val="Calibri"/>
-      </rPr>
-      <t xml:space="preserve">
-Wait__delay__0.1ms
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF4472C4"/>
-        <rFont val="Calibri"/>
-      </rPr>
-      <t xml:space="preserve">
-0x19[1]_0x01</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-      </rPr>
-      <t xml:space="preserve"> "bst_test en"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF7030A0"/>
-        <rFont val="Calibri"/>
-      </rPr>
-      <t xml:space="preserve">
-Wait__delay__0.1ms
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FFFF33CC"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FFFF33CC"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>Force__SW__0V</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FFFF33CC"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF70AD47"/>
-        <rFont val="Calibri"/>
-      </rPr>
-      <t xml:space="preserve">
-Measure__Voltage__SDWN </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-      </rPr>
-      <t xml:space="preserve">"should be 1V more or less"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF70AD47"/>
-        <rFont val="Calibri"/>
-      </rPr>
-      <t>Measure__Voltage__FSYN</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-      </rPr>
-      <t xml:space="preserve"> "should be 0"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF70AD47"/>
-        <rFont val="Calibri"/>
-      </rPr>
-      <t xml:space="preserve">Measure__Voltage__SDI </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-      </rPr>
-      <t xml:space="preserve">"should be 0"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FFFF3399"/>
-        <rFont val="Calibri"/>
-      </rPr>
-      <t xml:space="preserve">
-Force__VBSO__Ramp</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-      </rPr>
-      <t xml:space="preserve"> "decrease VBSO from 4.5V with steps of 50mV untill FSYN and SDI toggle from Low to High"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF7030A0"/>
-        <rFont val="Calibri"/>
-      </rPr>
-      <t xml:space="preserve">
-Wait__delay__0.1ms </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-      </rPr>
-      <t xml:space="preserve">"after comparator triggers"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF70AD47"/>
-        <rFont val="Calibri"/>
-      </rPr>
-      <t xml:space="preserve">
-Measure__Voltage__SDWN </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-      </rPr>
-      <t xml:space="preserve">"should be 0"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF70AD47"/>
-        <rFont val="Calibri"/>
-      </rPr>
-      <t xml:space="preserve">Measure__Voltage__FSYN </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-      </rPr>
-      <t xml:space="preserve">"should be 1"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF70AD47"/>
-        <rFont val="Calibri"/>
-      </rPr>
-      <t>Measure__Voltage__SDI</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-      </rPr>
-      <t xml:space="preserve"> "should be 1"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF4472C4"/>
-        <rFont val="Calibri"/>
-      </rPr>
-      <t xml:space="preserve">
-0x03_0x00 
-0x04_0x00
-0x1A_0x00
-0x19_0x00</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
         <sz val="11"/>
         <color rgb="FFFF3399"/>
         <rFont val="Calibri"/>
@@ -44676,6 +43990,692 @@
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve">
+0x1A_0x00
+0x19_0x00</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FFFF3399"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Run__startup
+Run__Boost_test_default
+Run__Enable_Ana_Testpoint
+Wait__delay__0.1ms
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF3399"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+Force__VBIAS__5V
+Force__VBSO__4.5V
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF4472C4"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve">
+0xFE_0x00 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>"Select page 0"</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF4472C4"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve">
+0x00_0x0F</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve"> "Power-up"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF4472C4"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>0xB0_0x00</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve"> "en 1 bst low"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF4472C4"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>0xB1_0x00</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve"> "en 2 bst low"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF4472C4"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>0xB3[4:3]_0x00</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve"> "en 3 bst low"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF4472C4"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve">
+0xFE_0x01</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve"> "Select page 1"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF4472C4"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>0x2F_0xAA</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve"> "Unlock test page"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF4472C4"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>0x2F_0xBB</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve"> "Unlock test page"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF4472C4"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve">
+0x18[6]_0x01</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve"> "Enable Mirr"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF4472C4"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>0xFE_0x00</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve"> "Select page 0"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF4472C4"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>0xB1[6]_0x01</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve"> "Bootstrap en"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF4472C4"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>0xB2[1]_0x00</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve"> "ls_sel off"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF4472C4"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>0xB4[2:0]_0x04</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve"> "hsb on hsa_byp off"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF4472C4"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve">0xB0[0]_0x01 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve">"bst general en"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF4472C4"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>0xFE_0x01</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve"> "Select page 1"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF4472C4"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>0x1A_0x03</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve"> "ana test TSW drive"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF4472C4"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>0x03_0x05</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve"> "FSYN and SDI TMUX"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF4472C4"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>0x04_0x14</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve"> "dig test EN FSYN=bst_bootstrap_comp_out SDI=low_on"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF4472C4"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>0x17[6]_0x01</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve"> "Force Mirr"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF4472C4"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>0x16[6]_0x01</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve"> "Force Bootstrap"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF4472C4"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>0xFE_0x00</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve"> "Select page 0"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF7030A0"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve">
+Wait__delay__0.1ms
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF4472C4"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve">
+0xB2[0]_0x01</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF7030A0"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve">"Power Force en"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF4472C4"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>0xFE_0x01</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF7030A0"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve">"Select page 1"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF4472C4"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>0x15[4]_0x01</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve"> "Force bst general en"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF7030A0"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve">
+Wait__delay__0.1ms
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF4472C4"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve">
+0x19[1]_0x01</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve"> "bst_test en"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF7030A0"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve">
+Wait__delay__0.1ms
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF33CC"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FFFF33CC"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Force__SW__0V</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF33CC"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF70AD47"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve">
+Measure__Voltage__SDWN </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve">"should be 1V more or less"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF70AD47"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>Measure__Voltage__FSYN</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve"> "should be 0"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF70AD47"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve">Measure__Voltage__SDI </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve">"should be 0"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF3399"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve">
+Force__VBSO__Ramp__4.5V__0V</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve"> "decrease VBSO from 4.5V with steps of 50mV untill FSYN and SDI toggle from Low to High"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF7030A0"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve">
+Wait__delay__0.1ms </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve">"after comparator triggers"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF70AD47"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve">
+Measure__Voltage__SDWN </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve">"should be 0"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF70AD47"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve">Measure__Voltage__FSYN </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve">"should be 1"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF70AD47"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>Measure__Voltage__SDI</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve"> "should be 1"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF4472C4"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve">
+0x03_0x00 
+0x04_0x00
 0x1A_0x00
 0x19_0x00</t>
     </r>
@@ -46461,6 +46461,9 @@
     <xf numFmtId="164" fontId="27" fillId="8" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="2" fontId="27" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
@@ -46490,9 +46493,6 @@
     </xf>
     <xf numFmtId="3" fontId="26" fillId="7" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="27" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -46900,177 +46900,177 @@
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" s="26" t="s">
+        <v>334</v>
+      </c>
+      <c r="J1" s="26" t="s">
         <v>335</v>
-      </c>
-      <c r="J1" s="26" t="s">
-        <v>336</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" s="25" t="s">
+        <v>336</v>
+      </c>
+      <c r="J2" s="25" t="s">
         <v>337</v>
-      </c>
-      <c r="J2" s="25" t="s">
-        <v>338</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" s="25" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="J3" s="25"/>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" s="25" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="J4" s="25"/>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" s="25" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="J5" s="25"/>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" s="25" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="B6" s="23"/>
       <c r="C6" s="23" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="D6" s="23"/>
       <c r="E6" s="23" t="s">
+        <v>343</v>
+      </c>
+      <c r="F6" s="23" t="s">
         <v>344</v>
       </c>
-      <c r="F6" s="23" t="s">
+      <c r="G6" s="23" t="s">
         <v>345</v>
       </c>
-      <c r="G6" s="23" t="s">
+      <c r="H6" s="24" t="s">
         <v>346</v>
       </c>
-      <c r="H6" s="24" t="s">
+      <c r="J6" s="25" t="s">
         <v>347</v>
       </c>
-      <c r="J6" s="25" t="s">
+      <c r="K6" s="58" t="s">
         <v>348</v>
-      </c>
-      <c r="K6" s="58" t="s">
-        <v>349</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" s="25" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="J7" s="25"/>
       <c r="K7" s="58" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" s="25" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="B8" s="88"/>
       <c r="C8" s="23" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="D8" s="23"/>
       <c r="E8" s="23" t="s">
+        <v>351</v>
+      </c>
+      <c r="F8" s="23" t="s">
         <v>352</v>
       </c>
-      <c r="F8" s="23" t="s">
+      <c r="G8" s="23" t="s">
         <v>353</v>
       </c>
-      <c r="G8" s="23" t="s">
+      <c r="H8" s="24" t="s">
         <v>354</v>
-      </c>
-      <c r="H8" s="24" t="s">
-        <v>355</v>
       </c>
       <c r="J8" s="25"/>
       <c r="K8" s="58"/>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" s="25" t="s">
+        <v>355</v>
+      </c>
+      <c r="J9" s="25" t="s">
         <v>356</v>
-      </c>
-      <c r="J9" s="25" t="s">
-        <v>357</v>
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" s="25" t="s">
+        <v>357</v>
+      </c>
+      <c r="J10" s="25" t="s">
         <v>358</v>
-      </c>
-      <c r="J10" s="25" t="s">
-        <v>359</v>
       </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" s="25" t="s">
+        <v>359</v>
+      </c>
+      <c r="J11" s="25" t="s">
         <v>360</v>
-      </c>
-      <c r="J11" s="25" t="s">
-        <v>361</v>
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" s="25" t="s">
+        <v>361</v>
+      </c>
+      <c r="J12" s="25" t="s">
         <v>362</v>
-      </c>
-      <c r="J12" s="25" t="s">
-        <v>363</v>
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" s="25" t="s">
+        <v>363</v>
+      </c>
+      <c r="J13" s="25" t="s">
         <v>364</v>
-      </c>
-      <c r="J13" s="25" t="s">
-        <v>365</v>
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" s="25" t="s">
+        <v>365</v>
+      </c>
+      <c r="J14" s="25" t="s">
         <v>366</v>
-      </c>
-      <c r="J14" s="25" t="s">
-        <v>367</v>
       </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" s="25" t="s">
+        <v>367</v>
+      </c>
+      <c r="J15" s="25" t="s">
         <v>368</v>
-      </c>
-      <c r="J15" s="25" t="s">
-        <v>369</v>
       </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" s="25" t="s">
+        <v>369</v>
+      </c>
+      <c r="J16" s="25" t="s">
         <v>370</v>
-      </c>
-      <c r="J16" s="25" t="s">
-        <v>371</v>
       </c>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A17" s="25" t="s">
+        <v>371</v>
+      </c>
+      <c r="J17" s="25" t="s">
         <v>372</v>
-      </c>
-      <c r="J17" s="25" t="s">
-        <v>373</v>
       </c>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A18" s="25" t="s">
+        <v>373</v>
+      </c>
+      <c r="J18" s="25" t="s">
         <v>374</v>
-      </c>
-      <c r="J18" s="25" t="s">
-        <v>375</v>
       </c>
     </row>
   </sheetData>
@@ -47966,10 +47966,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="21" x14ac:dyDescent="0.35">
-      <c r="A1" s="233" t="s">
-        <v>376</v>
-      </c>
-      <c r="B1" s="233"/>
+      <c r="A1" s="234" t="s">
+        <v>375</v>
+      </c>
+      <c r="B1" s="234"/>
       <c r="C1" s="9" t="s">
         <v>142</v>
       </c>
@@ -48000,10 +48000,10 @@
       </c>
     </row>
     <row r="3" spans="1:6" ht="21" x14ac:dyDescent="0.35">
-      <c r="A3" s="233" t="s">
+      <c r="A3" s="234" t="s">
         <v>140</v>
       </c>
-      <c r="B3" s="233"/>
+      <c r="B3" s="234"/>
       <c r="C3" s="15" t="s">
         <v>60</v>
       </c>
@@ -48018,10 +48018,10 @@
       </c>
     </row>
     <row r="4" spans="1:6" ht="21" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="233" t="s">
+      <c r="A4" s="234" t="s">
         <v>137</v>
       </c>
-      <c r="B4" s="233"/>
+      <c r="B4" s="234"/>
       <c r="C4" s="9" t="s">
         <v>142</v>
       </c>
@@ -48036,23 +48036,23 @@
       </c>
     </row>
     <row r="5" spans="1:6" ht="409.5" x14ac:dyDescent="0.25">
-      <c r="A5" s="234"/>
-      <c r="B5" s="235"/>
+      <c r="A5" s="235"/>
+      <c r="B5" s="236"/>
       <c r="C5" s="204" t="s">
+        <v>418</v>
+      </c>
+      <c r="D5" s="204" t="s">
         <v>419</v>
       </c>
-      <c r="D5" s="204" t="s">
-        <v>420</v>
-      </c>
       <c r="E5" s="204" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="F5" s="189" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="22.5" x14ac:dyDescent="0.3">
-      <c r="A6" s="236" t="s">
+      <c r="A6" s="237" t="s">
         <v>145</v>
       </c>
       <c r="B6" s="13" t="s">
@@ -48063,12 +48063,12 @@
       </c>
       <c r="D6" s="38"/>
       <c r="E6" s="38" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="F6" s="67"/>
     </row>
     <row r="7" spans="1:6" ht="22.5" x14ac:dyDescent="0.3">
-      <c r="A7" s="236"/>
+      <c r="A7" s="237"/>
       <c r="B7" s="14" t="s">
         <v>147</v>
       </c>
@@ -48080,7 +48080,7 @@
       <c r="F7" s="68"/>
     </row>
     <row r="8" spans="1:6" ht="22.5" x14ac:dyDescent="0.3">
-      <c r="A8" s="236"/>
+      <c r="A8" s="237"/>
       <c r="B8" s="10" t="s">
         <v>149</v>
       </c>
@@ -48088,15 +48088,15 @@
         <v>208</v>
       </c>
       <c r="D8" s="11" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="E8" s="11" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="F8" s="69"/>
     </row>
     <row r="9" spans="1:6" ht="22.5" x14ac:dyDescent="0.3">
-      <c r="A9" s="236"/>
+      <c r="A9" s="237"/>
       <c r="B9" s="12" t="s">
         <v>151</v>
       </c>
@@ -48108,7 +48108,7 @@
       <c r="F9" s="71"/>
     </row>
     <row r="10" spans="1:6" ht="22.5" x14ac:dyDescent="0.3">
-      <c r="A10" s="236"/>
+      <c r="A10" s="237"/>
       <c r="B10" s="14" t="s">
         <v>152</v>
       </c>
@@ -48117,7 +48117,7 @@
       </c>
       <c r="D10" s="8"/>
       <c r="E10" s="229" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="F10" s="68"/>
     </row>
@@ -49031,10 +49031,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="21" x14ac:dyDescent="0.35">
-      <c r="A1" s="233" t="s">
+      <c r="A1" s="234" t="s">
         <v>137</v>
       </c>
-      <c r="B1" s="233"/>
+      <c r="B1" s="234"/>
       <c r="C1" s="17" t="s">
         <v>138</v>
       </c>
@@ -49065,10 +49065,10 @@
       </c>
     </row>
     <row r="3" spans="1:6" ht="21" x14ac:dyDescent="0.35">
-      <c r="A3" s="233" t="s">
+      <c r="A3" s="234" t="s">
         <v>140</v>
       </c>
-      <c r="B3" s="233"/>
+      <c r="B3" s="234"/>
       <c r="C3" s="15" t="s">
         <v>79</v>
       </c>
@@ -49083,10 +49083,10 @@
       </c>
     </row>
     <row r="4" spans="1:6" ht="21" x14ac:dyDescent="0.35">
-      <c r="A4" s="233" t="s">
+      <c r="A4" s="234" t="s">
         <v>141</v>
       </c>
-      <c r="B4" s="233"/>
+      <c r="B4" s="234"/>
       <c r="C4" s="9" t="s">
         <v>200</v>
       </c>
@@ -49101,8 +49101,8 @@
       </c>
     </row>
     <row r="5" spans="1:6" ht="273" x14ac:dyDescent="0.25">
-      <c r="A5" s="234"/>
-      <c r="B5" s="235"/>
+      <c r="A5" s="235"/>
+      <c r="B5" s="236"/>
       <c r="C5" s="37" t="s">
         <v>204</v>
       </c>
@@ -49117,7 +49117,7 @@
       </c>
     </row>
     <row r="6" spans="1:6" ht="22.5" x14ac:dyDescent="0.3">
-      <c r="A6" s="237" t="s">
+      <c r="A6" s="238" t="s">
         <v>145</v>
       </c>
       <c r="B6" s="13" t="s">
@@ -49135,7 +49135,7 @@
       </c>
     </row>
     <row r="7" spans="1:6" ht="22.5" x14ac:dyDescent="0.3">
-      <c r="A7" s="237"/>
+      <c r="A7" s="238"/>
       <c r="B7" s="14" t="s">
         <v>147</v>
       </c>
@@ -49151,7 +49151,7 @@
       </c>
     </row>
     <row r="8" spans="1:6" ht="22.5" x14ac:dyDescent="0.3">
-      <c r="A8" s="237"/>
+      <c r="A8" s="238"/>
       <c r="B8" s="10" t="s">
         <v>149</v>
       </c>
@@ -49169,7 +49169,7 @@
       </c>
     </row>
     <row r="9" spans="1:6" ht="22.5" x14ac:dyDescent="0.3">
-      <c r="A9" s="237"/>
+      <c r="A9" s="238"/>
       <c r="B9" s="12" t="s">
         <v>151</v>
       </c>
@@ -49185,7 +49185,7 @@
       </c>
     </row>
     <row r="10" spans="1:6" ht="22.5" x14ac:dyDescent="0.3">
-      <c r="A10" s="237"/>
+      <c r="A10" s="238"/>
       <c r="B10" s="14" t="s">
         <v>152</v>
       </c>
@@ -49953,15 +49953,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="21" x14ac:dyDescent="0.35">
-      <c r="A1" s="233" t="s">
+      <c r="A1" s="234" t="s">
         <v>141</v>
       </c>
-      <c r="B1" s="233"/>
+      <c r="B1" s="234"/>
       <c r="C1" s="103" t="s">
         <v>211</v>
       </c>
       <c r="D1" s="116" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="E1" s="225" t="s">
         <v>212</v>
@@ -49985,10 +49985,10 @@
       </c>
     </row>
     <row r="3" spans="1:6" s="1" customFormat="1" ht="25.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="233" t="s">
+      <c r="A3" s="234" t="s">
         <v>140</v>
       </c>
-      <c r="B3" s="233"/>
+      <c r="B3" s="234"/>
       <c r="C3" s="102" t="s">
         <v>20</v>
       </c>
@@ -50003,15 +50003,15 @@
       </c>
     </row>
     <row r="4" spans="1:6" s="1" customFormat="1" ht="74.45" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="233" t="s">
+      <c r="A4" s="234" t="s">
         <v>137</v>
       </c>
-      <c r="B4" s="233"/>
+      <c r="B4" s="234"/>
       <c r="C4" s="103" t="s">
         <v>211</v>
       </c>
       <c r="D4" s="116" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="E4" s="103" t="s">
         <v>212</v>
@@ -50021,23 +50021,23 @@
       </c>
     </row>
     <row r="5" spans="1:6" s="1" customFormat="1" ht="409.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="234"/>
-      <c r="B5" s="235"/>
+      <c r="A5" s="235"/>
+      <c r="B5" s="236"/>
       <c r="C5" s="207" t="s">
         <v>214</v>
       </c>
       <c r="D5" s="216" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="E5" s="207" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="F5" s="218" t="s">
         <v>215</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="237" t="s">
+      <c r="A6" s="238" t="s">
         <v>145</v>
       </c>
       <c r="B6" s="13" t="s">
@@ -50051,7 +50051,7 @@
       </c>
     </row>
     <row r="7" spans="1:6" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="237"/>
+      <c r="A7" s="238"/>
       <c r="B7" s="14" t="s">
         <v>147</v>
       </c>
@@ -50061,12 +50061,12 @@
       <c r="F7" s="130"/>
     </row>
     <row r="8" spans="1:6" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="237"/>
+      <c r="A8" s="238"/>
       <c r="B8" s="10" t="s">
         <v>149</v>
       </c>
       <c r="C8" s="106" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="D8" s="119" t="s">
         <v>216</v>
@@ -50079,7 +50079,7 @@
       </c>
     </row>
     <row r="9" spans="1:6" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="237"/>
+      <c r="A9" s="238"/>
       <c r="B9" s="12" t="s">
         <v>151</v>
       </c>
@@ -50091,7 +50091,7 @@
       </c>
     </row>
     <row r="10" spans="1:6" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="237"/>
+      <c r="A10" s="238"/>
       <c r="B10" s="14" t="s">
         <v>152</v>
       </c>
@@ -51005,10 +51005,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:29" ht="21" x14ac:dyDescent="0.35">
-      <c r="A1" s="238" t="s">
+      <c r="A1" s="239" t="s">
         <v>137</v>
       </c>
-      <c r="B1" s="238"/>
+      <c r="B1" s="239"/>
       <c r="C1" s="65" t="s">
         <v>19</v>
       </c>
@@ -51175,10 +51175,10 @@
       </c>
     </row>
     <row r="3" spans="1:29" s="1" customFormat="1" ht="25.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="238" t="s">
+      <c r="A3" s="239" t="s">
         <v>140</v>
       </c>
-      <c r="B3" s="238"/>
+      <c r="B3" s="239"/>
       <c r="C3" s="182" t="s">
         <v>20</v>
       </c>
@@ -51262,10 +51262,10 @@
       </c>
     </row>
     <row r="4" spans="1:29" s="1" customFormat="1" ht="74.45" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="238" t="s">
+      <c r="A4" s="239" t="s">
         <v>141</v>
       </c>
-      <c r="B4" s="238"/>
+      <c r="B4" s="239"/>
       <c r="C4" s="65" t="s">
         <v>19</v>
       </c>
@@ -51349,45 +51349,45 @@
       </c>
     </row>
     <row r="5" spans="1:29" s="1" customFormat="1" ht="409.5" x14ac:dyDescent="0.25">
-      <c r="A5" s="239"/>
-      <c r="B5" s="239"/>
+      <c r="A5" s="240"/>
+      <c r="B5" s="240"/>
       <c r="C5" s="183" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="D5" s="183" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
       <c r="E5" s="183" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="F5" s="221" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
       <c r="G5" s="183" t="s">
+        <v>410</v>
+      </c>
+      <c r="H5" s="189" t="s">
+        <v>423</v>
+      </c>
+      <c r="I5" s="189" t="s">
         <v>411</v>
       </c>
-      <c r="H5" s="189" t="s">
-        <v>424</v>
-      </c>
-      <c r="I5" s="189" t="s">
+      <c r="J5" s="189" t="s">
+        <v>430</v>
+      </c>
+      <c r="K5" s="189" t="s">
+        <v>427</v>
+      </c>
+      <c r="L5" s="183" t="s">
         <v>412</v>
       </c>
-      <c r="J5" s="189" t="s">
-        <v>431</v>
-      </c>
-      <c r="K5" s="189" t="s">
-        <v>428</v>
-      </c>
-      <c r="L5" s="183" t="s">
+      <c r="M5" s="221" t="s">
         <v>413</v>
       </c>
-      <c r="M5" s="221" t="s">
-        <v>414</v>
-      </c>
       <c r="N5" s="183" t="s">
-        <v>426</v>
-      </c>
-      <c r="O5" s="183" t="s">
+        <v>425</v>
+      </c>
+      <c r="O5" s="221" t="s">
         <v>231</v>
       </c>
       <c r="P5" s="221" t="s">
@@ -51397,22 +51397,22 @@
         <v>233</v>
       </c>
       <c r="R5" s="221" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
       <c r="S5" s="188" t="s">
         <v>234</v>
       </c>
       <c r="T5" s="189" t="s">
+        <v>431</v>
+      </c>
+      <c r="U5" s="189" t="s">
         <v>432</v>
-      </c>
-      <c r="U5" s="189" t="s">
-        <v>433</v>
       </c>
       <c r="V5" s="189" t="s">
         <v>235</v>
       </c>
       <c r="W5" s="190" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
       <c r="X5" s="190" t="s">
         <v>236</v>
@@ -51421,20 +51421,20 @@
         <v>237</v>
       </c>
       <c r="Z5" s="190" t="s">
+        <v>435</v>
+      </c>
+      <c r="AA5" s="189" t="s">
+        <v>414</v>
+      </c>
+      <c r="AB5" s="189" t="s">
+        <v>415</v>
+      </c>
+      <c r="AC5" s="221" t="s">
         <v>238</v>
       </c>
-      <c r="AA5" s="189" t="s">
-        <v>415</v>
-      </c>
-      <c r="AB5" s="189" t="s">
-        <v>416</v>
-      </c>
-      <c r="AC5" s="221" t="s">
-        <v>239</v>
-      </c>
     </row>
     <row r="6" spans="1:29" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="240" t="s">
+      <c r="A6" s="241" t="s">
         <v>145</v>
       </c>
       <c r="B6" s="59" t="s">
@@ -51513,7 +51513,7 @@
       <c r="AC6" s="67"/>
     </row>
     <row r="7" spans="1:29" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="240"/>
+      <c r="A7" s="241"/>
       <c r="B7" s="60" t="s">
         <v>147</v>
       </c>
@@ -51548,15 +51548,15 @@
       <c r="AC7" s="68"/>
     </row>
     <row r="8" spans="1:29" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="240"/>
+      <c r="A8" s="241"/>
       <c r="B8" s="61" t="s">
         <v>149</v>
       </c>
       <c r="C8" s="69" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="D8" s="69" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="E8" s="69" t="s">
         <v>24</v>
@@ -51565,19 +51565,19 @@
         <v>44</v>
       </c>
       <c r="G8" s="69" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="H8" s="69" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="I8" s="69" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="J8" s="69" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="K8" s="69" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="L8" s="11" t="s">
         <v>79</v>
@@ -51592,40 +51592,40 @@
         <v>24</v>
       </c>
       <c r="P8" s="69" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="Q8" s="69" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="R8" s="153" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="S8" s="141"/>
       <c r="T8" s="119" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="U8" s="69" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="V8" s="69" t="s">
-        <v>423</v>
-      </c>
-      <c r="W8" s="243" t="s">
-        <v>423</v>
+        <v>422</v>
+      </c>
+      <c r="W8" s="233" t="s">
+        <v>422</v>
       </c>
       <c r="X8" s="69"/>
       <c r="Y8" s="69"/>
       <c r="Z8" s="69" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="AA8" s="69"/>
       <c r="AB8" s="69"/>
       <c r="AC8" s="11" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
     </row>
     <row r="9" spans="1:29" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="240"/>
+      <c r="A9" s="241"/>
       <c r="B9" s="62" t="s">
         <v>151</v>
       </c>
@@ -51650,7 +51650,7 @@
         <v>1.8</v>
       </c>
       <c r="K9" s="71" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="L9" s="71">
         <v>3</v>
@@ -51665,7 +51665,7 @@
         <v>4</v>
       </c>
       <c r="P9" s="71" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="Q9" s="70">
         <v>1.64</v>
@@ -51677,10 +51677,10 @@
       <c r="T9" s="232"/>
       <c r="U9" s="71"/>
       <c r="V9" s="71" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="W9" s="71" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="X9" s="196">
         <v>20.074999999999999</v>
@@ -51689,18 +51689,18 @@
         <v>24.2</v>
       </c>
       <c r="Z9" s="71" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="AA9" s="39" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="AB9" s="39" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="AC9" s="71"/>
     </row>
     <row r="10" spans="1:29" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="240"/>
+      <c r="A10" s="241"/>
       <c r="B10" s="60" t="s">
         <v>152</v>
       </c>
@@ -51743,10 +51743,10 @@
         <v>218</v>
       </c>
       <c r="D11" s="72" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="E11" s="72" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="F11" s="72"/>
       <c r="G11" s="72" t="s">
@@ -51814,7 +51814,7 @@
         <v>155</v>
       </c>
       <c r="AC11" s="5" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
     </row>
     <row r="12" spans="1:29" ht="20.25" customHeight="1" x14ac:dyDescent="0.35">
@@ -51952,10 +51952,10 @@
         <v>163</v>
       </c>
       <c r="D14" s="86" t="s">
+        <v>246</v>
+      </c>
+      <c r="E14" s="86" t="s">
         <v>247</v>
-      </c>
-      <c r="E14" s="86" t="s">
-        <v>248</v>
       </c>
       <c r="F14" s="85" t="s">
         <v>163</v>
@@ -52018,7 +52018,7 @@
         <v>163</v>
       </c>
       <c r="AB14" s="84" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="AC14" s="85" t="s">
         <v>163</v>
@@ -52368,7 +52368,7 @@
       <c r="N20" s="85"/>
       <c r="O20" s="85"/>
       <c r="P20" s="85" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="Q20" s="85"/>
       <c r="R20" s="155"/>
@@ -52487,7 +52487,7 @@
         <v>191</v>
       </c>
       <c r="F23" s="98" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="G23" s="84" t="s">
         <v>163</v>
@@ -52529,7 +52529,7 @@
         <v>163</v>
       </c>
       <c r="T23" s="168" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="U23" s="84" t="s">
         <v>163</v>
@@ -52616,10 +52616,10 @@
         <v>191</v>
       </c>
       <c r="T24" s="166" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="U24" s="85" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="V24" s="85" t="s">
         <v>191</v>
@@ -52711,11 +52711,11 @@
       <c r="Y26" s="85"/>
       <c r="Z26" s="85"/>
       <c r="AA26" s="84" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="AB26" s="84"/>
       <c r="AC26" s="84" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
     </row>
     <row r="27" spans="1:29" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -52750,7 +52750,7 @@
       <c r="Y27" s="85"/>
       <c r="Z27" s="85"/>
       <c r="AA27" s="84" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="AB27" s="85"/>
       <c r="AC27" s="85"/>
@@ -55237,10 +55237,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="21" x14ac:dyDescent="0.35">
-      <c r="A1" s="238" t="s">
+      <c r="A1" s="239" t="s">
         <v>137</v>
       </c>
-      <c r="B1" s="238"/>
+      <c r="B1" s="239"/>
       <c r="C1" s="17" t="s">
         <v>138</v>
       </c>
@@ -55335,10 +55335,10 @@
       </c>
     </row>
     <row r="3" spans="1:17" s="1" customFormat="1" ht="25.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="238" t="s">
+      <c r="A3" s="239" t="s">
         <v>140</v>
       </c>
-      <c r="B3" s="238"/>
+      <c r="B3" s="239"/>
       <c r="C3" s="15" t="s">
         <v>99</v>
       </c>
@@ -55386,107 +55386,107 @@
       </c>
     </row>
     <row r="4" spans="1:17" s="1" customFormat="1" ht="97.15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="238" t="s">
+      <c r="A4" s="239" t="s">
         <v>141</v>
       </c>
-      <c r="B4" s="238"/>
+      <c r="B4" s="239"/>
       <c r="C4" s="65" t="s">
+        <v>256</v>
+      </c>
+      <c r="D4" s="9" t="s">
         <v>257</v>
       </c>
-      <c r="D4" s="9" t="s">
+      <c r="E4" s="9" t="s">
         <v>258</v>
       </c>
-      <c r="E4" s="9" t="s">
+      <c r="F4" s="9" t="s">
         <v>259</v>
       </c>
-      <c r="F4" s="9" t="s">
+      <c r="G4" s="65" t="s">
         <v>260</v>
       </c>
-      <c r="G4" s="65" t="s">
+      <c r="H4" s="9" t="s">
         <v>261</v>
       </c>
-      <c r="H4" s="9" t="s">
+      <c r="I4" s="90" t="s">
         <v>262</v>
       </c>
-      <c r="I4" s="90" t="s">
+      <c r="J4" s="90" t="s">
         <v>263</v>
       </c>
-      <c r="J4" s="90" t="s">
+      <c r="K4" s="90" t="s">
         <v>264</v>
       </c>
-      <c r="K4" s="90" t="s">
+      <c r="L4" s="93" t="s">
         <v>265</v>
       </c>
-      <c r="L4" s="93" t="s">
+      <c r="M4" s="93" t="s">
         <v>266</v>
       </c>
-      <c r="M4" s="93" t="s">
+      <c r="N4" s="93" t="s">
         <v>267</v>
       </c>
-      <c r="N4" s="93" t="s">
+      <c r="O4" s="93" t="s">
         <v>268</v>
       </c>
-      <c r="O4" s="93" t="s">
+      <c r="P4" s="93" t="s">
         <v>269</v>
       </c>
-      <c r="P4" s="93" t="s">
+      <c r="Q4" s="93" t="s">
         <v>270</v>
       </c>
-      <c r="Q4" s="93" t="s">
+    </row>
+    <row r="5" spans="1:17" s="1" customFormat="1" ht="409.6" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="242"/>
+      <c r="B5" s="243"/>
+      <c r="C5" s="219" t="s">
         <v>271</v>
       </c>
-    </row>
-    <row r="5" spans="1:17" s="1" customFormat="1" ht="409.6" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="241"/>
-      <c r="B5" s="242"/>
-      <c r="C5" s="219" t="s">
+      <c r="D5" s="220" t="s">
         <v>272</v>
       </c>
-      <c r="D5" s="220" t="s">
+      <c r="E5" s="203" t="s">
+        <v>403</v>
+      </c>
+      <c r="F5" s="203" t="s">
+        <v>409</v>
+      </c>
+      <c r="G5" s="203" t="s">
+        <v>402</v>
+      </c>
+      <c r="H5" s="203" t="s">
+        <v>401</v>
+      </c>
+      <c r="I5" s="203" t="s">
+        <v>400</v>
+      </c>
+      <c r="J5" s="203" t="s">
+        <v>399</v>
+      </c>
+      <c r="K5" s="203" t="s">
+        <v>398</v>
+      </c>
+      <c r="L5" s="203" t="s">
+        <v>394</v>
+      </c>
+      <c r="M5" s="202" t="s">
         <v>273</v>
       </c>
-      <c r="E5" s="203" t="s">
-        <v>404</v>
-      </c>
-      <c r="F5" s="203" t="s">
-        <v>410</v>
-      </c>
-      <c r="G5" s="203" t="s">
-        <v>403</v>
-      </c>
-      <c r="H5" s="203" t="s">
-        <v>402</v>
-      </c>
-      <c r="I5" s="203" t="s">
-        <v>401</v>
-      </c>
-      <c r="J5" s="203" t="s">
-        <v>400</v>
-      </c>
-      <c r="K5" s="203" t="s">
-        <v>399</v>
-      </c>
-      <c r="L5" s="203" t="s">
-        <v>395</v>
-      </c>
-      <c r="M5" s="202" t="s">
+      <c r="N5" s="202" t="s">
         <v>274</v>
       </c>
-      <c r="N5" s="202" t="s">
+      <c r="O5" s="202" t="s">
         <v>275</v>
       </c>
-      <c r="O5" s="202" t="s">
+      <c r="P5" s="202" t="s">
         <v>276</v>
       </c>
-      <c r="P5" s="202" t="s">
+      <c r="Q5" s="202" t="s">
         <v>277</v>
       </c>
-      <c r="Q5" s="202" t="s">
-        <v>278</v>
-      </c>
     </row>
     <row r="6" spans="1:17" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="240" t="s">
+      <c r="A6" s="241" t="s">
         <v>145</v>
       </c>
       <c r="B6" s="59" t="s">
@@ -55509,7 +55509,7 @@
       <c r="Q6" s="38"/>
     </row>
     <row r="7" spans="1:17" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="240"/>
+      <c r="A7" s="241"/>
       <c r="B7" s="60" t="s">
         <v>147</v>
       </c>
@@ -55530,52 +55530,52 @@
       <c r="Q7" s="8"/>
     </row>
     <row r="8" spans="1:17" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="240"/>
+      <c r="A8" s="241"/>
       <c r="B8" s="61" t="s">
         <v>149</v>
       </c>
       <c r="C8" s="11"/>
       <c r="D8" s="11"/>
       <c r="E8" s="11" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="F8" s="11" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="G8" s="11" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="H8" s="11" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="I8" s="11" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="J8" s="11" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="K8" s="11" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="L8" s="11"/>
       <c r="M8" s="11" t="s">
+        <v>279</v>
+      </c>
+      <c r="N8" s="11" t="s">
         <v>280</v>
       </c>
-      <c r="N8" s="11" t="s">
+      <c r="O8" s="11" t="s">
         <v>281</v>
       </c>
-      <c r="O8" s="11" t="s">
+      <c r="P8" s="11" t="s">
         <v>282</v>
       </c>
-      <c r="P8" s="11" t="s">
+      <c r="Q8" s="11" t="s">
         <v>283</v>
       </c>
-      <c r="Q8" s="11" t="s">
-        <v>284</v>
-      </c>
     </row>
     <row r="9" spans="1:17" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="240"/>
+      <c r="A9" s="241"/>
       <c r="B9" s="62" t="s">
         <v>151</v>
       </c>
@@ -55583,7 +55583,7 @@
         <v>1</v>
       </c>
       <c r="D9" s="39" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="E9" s="71"/>
       <c r="F9" s="71"/>
@@ -55600,7 +55600,7 @@
       <c r="Q9" s="39"/>
     </row>
     <row r="10" spans="1:17" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="240"/>
+      <c r="A10" s="241"/>
       <c r="B10" s="60" t="s">
         <v>152</v>
       </c>
@@ -55626,47 +55626,47 @@
         <v>154</v>
       </c>
       <c r="C11" s="5" t="s">
+        <v>285</v>
+      </c>
+      <c r="D11" s="5" t="s">
+        <v>285</v>
+      </c>
+      <c r="E11" s="5" t="s">
         <v>286</v>
       </c>
-      <c r="D11" s="5" t="s">
+      <c r="F11" s="5" t="s">
         <v>286</v>
       </c>
-      <c r="E11" s="5" t="s">
-        <v>287</v>
-      </c>
-      <c r="F11" s="5" t="s">
-        <v>287</v>
-      </c>
       <c r="G11" s="5" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="H11" s="5" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="I11" s="5" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="J11" s="5" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="K11" s="5" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="L11" s="5"/>
       <c r="M11" s="5" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="N11" s="5" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="O11" s="5" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="P11" s="5" t="s">
         <v>155</v>
       </c>
       <c r="Q11" s="5" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="12" spans="1:17" ht="20.25" customHeight="1" x14ac:dyDescent="0.35">
@@ -55986,13 +55986,13 @@
       </c>
       <c r="C20" s="50"/>
       <c r="D20" s="50" t="s">
+        <v>289</v>
+      </c>
+      <c r="E20" s="50" t="s">
         <v>290</v>
       </c>
-      <c r="E20" s="50" t="s">
-        <v>291</v>
-      </c>
       <c r="F20" s="50" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="G20" s="89"/>
       <c r="I20" s="76"/>
@@ -56013,29 +56013,29 @@
         <v>184</v>
       </c>
       <c r="C21" s="50" t="s">
+        <v>291</v>
+      </c>
+      <c r="D21" s="50" t="s">
         <v>292</v>
       </c>
-      <c r="D21" s="50" t="s">
+      <c r="E21" s="50" t="s">
         <v>293</v>
-      </c>
-      <c r="E21" s="50" t="s">
-        <v>294</v>
       </c>
       <c r="F21" s="50"/>
       <c r="G21" s="50" t="s">
+        <v>294</v>
+      </c>
+      <c r="H21" s="50" t="s">
         <v>295</v>
       </c>
-      <c r="H21" s="50" t="s">
+      <c r="I21" s="76" t="s">
         <v>296</v>
       </c>
-      <c r="I21" s="76" t="s">
-        <v>297</v>
-      </c>
       <c r="J21" s="76" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="K21" s="76" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="L21" s="76"/>
       <c r="M21" s="50"/>
@@ -56052,31 +56052,31 @@
         <v>186</v>
       </c>
       <c r="C22" s="50" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="D22" s="50" t="s">
+        <v>297</v>
+      </c>
+      <c r="E22" s="50" t="s">
         <v>298</v>
       </c>
-      <c r="E22" s="50" t="s">
+      <c r="F22" s="50" t="s">
+        <v>298</v>
+      </c>
+      <c r="G22" s="50" t="s">
         <v>299</v>
       </c>
-      <c r="F22" s="50" t="s">
-        <v>299</v>
-      </c>
-      <c r="G22" s="50" t="s">
+      <c r="H22" s="50" t="s">
         <v>300</v>
       </c>
-      <c r="H22" s="50" t="s">
+      <c r="I22" s="76" t="s">
         <v>301</v>
       </c>
-      <c r="I22" s="76" t="s">
+      <c r="J22" s="76" t="s">
         <v>302</v>
       </c>
-      <c r="J22" s="76" t="s">
+      <c r="K22" s="76" t="s">
         <v>303</v>
-      </c>
-      <c r="K22" s="76" t="s">
-        <v>304</v>
       </c>
       <c r="L22" s="76"/>
       <c r="M22" s="50"/>
@@ -56162,31 +56162,31 @@
         <v>195</v>
       </c>
       <c r="C26" s="50" t="s">
+        <v>304</v>
+      </c>
+      <c r="D26" s="50" t="s">
+        <v>304</v>
+      </c>
+      <c r="E26" s="50" t="s">
         <v>305</v>
       </c>
-      <c r="D26" s="50" t="s">
+      <c r="F26" s="50" t="s">
         <v>305</v>
       </c>
-      <c r="E26" s="50" t="s">
-        <v>306</v>
-      </c>
-      <c r="F26" s="50" t="s">
-        <v>306</v>
-      </c>
       <c r="G26" s="50" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="H26" s="50" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="I26" s="50" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="J26" s="50" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="K26" s="50" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="L26" s="50"/>
       <c r="M26" s="50"/>
@@ -56203,31 +56203,31 @@
         <v>197</v>
       </c>
       <c r="C27" s="50" t="s">
+        <v>304</v>
+      </c>
+      <c r="D27" s="50" t="s">
+        <v>304</v>
+      </c>
+      <c r="E27" s="50" t="s">
         <v>305</v>
       </c>
-      <c r="D27" s="50" t="s">
+      <c r="F27" s="50" t="s">
         <v>305</v>
       </c>
-      <c r="E27" s="50" t="s">
-        <v>306</v>
-      </c>
-      <c r="F27" s="50" t="s">
-        <v>306</v>
-      </c>
       <c r="G27" s="50" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="H27" s="50" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="I27" s="50" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="J27" s="50" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="K27" s="50" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="L27" s="50"/>
       <c r="M27" s="50"/>
@@ -57766,24 +57766,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="46.5" x14ac:dyDescent="0.7">
-      <c r="A1" s="238" t="s">
+      <c r="A1" s="239" t="s">
         <v>141</v>
       </c>
-      <c r="B1" s="238"/>
+      <c r="B1" s="239"/>
       <c r="C1" s="231" t="s">
         <v>64</v>
       </c>
       <c r="D1" s="65" t="s">
+        <v>380</v>
+      </c>
+      <c r="E1" s="65" t="s">
         <v>381</v>
       </c>
-      <c r="E1" s="65" t="s">
+      <c r="F1" s="65" t="s">
+        <v>383</v>
+      </c>
+      <c r="G1" s="65" t="s">
         <v>382</v>
-      </c>
-      <c r="F1" s="65" t="s">
-        <v>384</v>
-      </c>
-      <c r="G1" s="65" t="s">
-        <v>383</v>
       </c>
       <c r="H1" s="65" t="s">
         <v>114</v>
@@ -57792,16 +57792,16 @@
         <v>118</v>
       </c>
       <c r="J1" s="65" t="s">
+        <v>307</v>
+      </c>
+      <c r="K1" s="65" t="s">
         <v>308</v>
-      </c>
-      <c r="K1" s="65" t="s">
-        <v>309</v>
       </c>
       <c r="L1" s="65" t="s">
         <v>122</v>
       </c>
       <c r="M1" s="95" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
     </row>
     <row r="2" spans="1:13" ht="21" x14ac:dyDescent="0.35">
@@ -57840,10 +57840,10 @@
       </c>
     </row>
     <row r="3" spans="1:13" s="1" customFormat="1" ht="25.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="238" t="s">
+      <c r="A3" s="239" t="s">
         <v>140</v>
       </c>
-      <c r="B3" s="238"/>
+      <c r="B3" s="239"/>
       <c r="C3" s="64" t="s">
         <v>65</v>
       </c>
@@ -57875,28 +57875,28 @@
         <v>36</v>
       </c>
       <c r="M3" s="64" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
     </row>
     <row r="4" spans="1:13" s="1" customFormat="1" ht="74.45" customHeight="1" x14ac:dyDescent="0.7">
-      <c r="A4" s="238" t="s">
+      <c r="A4" s="239" t="s">
         <v>137</v>
       </c>
-      <c r="B4" s="238"/>
+      <c r="B4" s="239"/>
       <c r="C4" s="65" t="s">
         <v>64</v>
       </c>
       <c r="D4" s="65" t="s">
+        <v>380</v>
+      </c>
+      <c r="E4" s="65" t="s">
         <v>381</v>
       </c>
-      <c r="E4" s="65" t="s">
+      <c r="F4" s="65" t="s">
+        <v>383</v>
+      </c>
+      <c r="G4" s="65" t="s">
         <v>382</v>
-      </c>
-      <c r="F4" s="65" t="s">
-        <v>384</v>
-      </c>
-      <c r="G4" s="65" t="s">
-        <v>383</v>
       </c>
       <c r="H4" s="65" t="s">
         <v>114</v>
@@ -57905,55 +57905,55 @@
         <v>118</v>
       </c>
       <c r="J4" s="65" t="s">
+        <v>307</v>
+      </c>
+      <c r="K4" s="65" t="s">
         <v>308</v>
-      </c>
-      <c r="K4" s="65" t="s">
-        <v>309</v>
       </c>
       <c r="L4" s="65" t="s">
         <v>122</v>
       </c>
       <c r="M4" s="95" t="s">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" s="1" customFormat="1" ht="409.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="242"/>
+      <c r="B5" s="242"/>
+      <c r="C5" s="208" t="s">
+        <v>393</v>
+      </c>
+      <c r="D5" s="37" t="s">
+        <v>386</v>
+      </c>
+      <c r="E5" s="37" t="s">
+        <v>387</v>
+      </c>
+      <c r="F5" s="37" t="s">
+        <v>388</v>
+      </c>
+      <c r="G5" s="37" t="s">
+        <v>389</v>
+      </c>
+      <c r="H5" s="37" t="s">
+        <v>390</v>
+      </c>
+      <c r="I5" s="37" t="s">
+        <v>391</v>
+      </c>
+      <c r="J5" s="56" t="s">
         <v>310</v>
       </c>
-    </row>
-    <row r="5" spans="1:13" s="1" customFormat="1" ht="409.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="241"/>
-      <c r="B5" s="241"/>
-      <c r="C5" s="208" t="s">
-        <v>394</v>
-      </c>
-      <c r="D5" s="37" t="s">
-        <v>387</v>
-      </c>
-      <c r="E5" s="37" t="s">
-        <v>388</v>
-      </c>
-      <c r="F5" s="37" t="s">
-        <v>389</v>
-      </c>
-      <c r="G5" s="37" t="s">
-        <v>390</v>
-      </c>
-      <c r="H5" s="37" t="s">
-        <v>391</v>
-      </c>
-      <c r="I5" s="37" t="s">
-        <v>392</v>
-      </c>
-      <c r="J5" s="56" t="s">
-        <v>311</v>
-      </c>
       <c r="K5" s="226" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="L5" s="226" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="M5" s="56"/>
     </row>
     <row r="6" spans="1:13" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="240" t="s">
+      <c r="A6" s="241" t="s">
         <v>145</v>
       </c>
       <c r="B6" s="59" t="s">
@@ -57972,7 +57972,7 @@
       <c r="M6" s="67"/>
     </row>
     <row r="7" spans="1:13" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="240"/>
+      <c r="A7" s="241"/>
       <c r="B7" s="60" t="s">
         <v>147</v>
       </c>
@@ -57989,21 +57989,21 @@
       <c r="M7" s="68"/>
     </row>
     <row r="8" spans="1:13" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="240"/>
+      <c r="A8" s="241"/>
       <c r="B8" s="61" t="s">
         <v>149</v>
       </c>
       <c r="C8" s="69" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="D8" s="69" t="s">
+        <v>311</v>
+      </c>
+      <c r="E8" s="69" t="s">
         <v>312</v>
       </c>
-      <c r="E8" s="69" t="s">
-        <v>313</v>
-      </c>
       <c r="F8" s="69" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="G8" s="69" t="s">
         <v>20</v>
@@ -58015,10 +58015,10 @@
         <v>75</v>
       </c>
       <c r="J8" s="69" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="K8" s="11" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="L8" s="11" t="s">
         <v>75</v>
@@ -58026,7 +58026,7 @@
       <c r="M8" s="69"/>
     </row>
     <row r="9" spans="1:13" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="240"/>
+      <c r="A9" s="241"/>
       <c r="B9" s="62" t="s">
         <v>151</v>
       </c>
@@ -58043,7 +58043,7 @@
       <c r="M9" s="71"/>
     </row>
     <row r="10" spans="1:13" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="240"/>
+      <c r="A10" s="241"/>
       <c r="B10" s="60" t="s">
         <v>152</v>
       </c>
@@ -59717,84 +59717,84 @@
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1" s="57" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="B1" s="57" t="s">
         <v>15</v>
       </c>
       <c r="C1" s="57" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="D1" s="57" t="s">
+        <v>315</v>
+      </c>
+      <c r="E1" s="57" t="s">
         <v>316</v>
       </c>
-      <c r="E1" s="57" t="s">
+      <c r="F1" s="57" t="s">
         <v>317</v>
       </c>
-      <c r="F1" s="57" t="s">
+      <c r="G1" s="57" t="s">
         <v>318</v>
       </c>
-      <c r="G1" s="57" t="s">
+      <c r="H1" s="57" t="s">
         <v>319</v>
       </c>
-      <c r="H1" s="57" t="s">
+      <c r="I1" s="57" t="s">
         <v>320</v>
       </c>
-      <c r="I1" s="57" t="s">
+      <c r="J1" s="57" t="s">
         <v>321</v>
       </c>
-      <c r="J1" s="57" t="s">
+      <c r="K1" s="57" t="s">
         <v>322</v>
       </c>
-      <c r="K1" s="57" t="s">
+      <c r="L1" s="57" t="s">
         <v>323</v>
       </c>
-      <c r="L1" s="57" t="s">
+      <c r="M1" s="57" t="s">
         <v>324</v>
-      </c>
-      <c r="M1" s="57" t="s">
-        <v>325</v>
       </c>
     </row>
     <row r="2" spans="1:13" s="91" customFormat="1" ht="408.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="83" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="B2" s="174" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
       <c r="C2" s="174" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="D2" s="83" t="s">
+        <v>325</v>
+      </c>
+      <c r="E2" s="224" t="s">
+        <v>417</v>
+      </c>
+      <c r="F2" s="83" t="s">
         <v>326</v>
       </c>
-      <c r="E2" s="224" t="s">
-        <v>418</v>
-      </c>
-      <c r="F2" s="83" t="s">
+      <c r="G2" s="83" t="s">
         <v>327</v>
       </c>
-      <c r="G2" s="83" t="s">
+      <c r="H2" s="83" t="s">
         <v>328</v>
       </c>
-      <c r="H2" s="83" t="s">
+      <c r="I2" s="83" t="s">
         <v>329</v>
       </c>
-      <c r="I2" s="83" t="s">
+      <c r="J2" s="83" t="s">
         <v>330</v>
       </c>
-      <c r="J2" s="83" t="s">
+      <c r="K2" s="83" t="s">
         <v>331</v>
       </c>
-      <c r="K2" s="83" t="s">
+      <c r="L2" s="83" t="s">
         <v>332</v>
       </c>
-      <c r="L2" s="83" t="s">
+      <c r="M2" s="83" t="s">
         <v>333</v>
-      </c>
-      <c r="M2" s="83" t="s">
-        <v>334</v>
       </c>
     </row>
   </sheetData>
@@ -59804,26 +59804,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="e658002f-fdfe-4e4b-94aa-0526ee42a8ac">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="4ad8f8a2-17e7-49a9-8390-22f3c8f42b39" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x010100C9B53A5B1F235B4EBDF9F22062DFC34D" ma:contentTypeVersion="12" ma:contentTypeDescription="Creare un nuovo documento." ma:contentTypeScope="" ma:versionID="ad5b12d537450e73edf2af95672e184c">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="e658002f-fdfe-4e4b-94aa-0526ee42a8ac" xmlns:ns3="4ad8f8a2-17e7-49a9-8390-22f3c8f42b39" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="ac16958afaf1bb0d1dccad67078e8e2c" ns2:_="" ns3:_="">
     <xsd:import namespace="e658002f-fdfe-4e4b-94aa-0526ee42a8ac"/>
@@ -60040,10 +60020,41 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="e658002f-fdfe-4e4b-94aa-0526ee42a8ac">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="4ad8f8a2-17e7-49a9-8390-22f3c8f42b39" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BA99F9FA-472B-49CB-8CD8-32BE0FD0DC5E}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{31D0029D-E8A7-4DC9-B140-19D450DFB7E0}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="e658002f-fdfe-4e4b-94aa-0526ee42a8ac"/>
+    <ds:schemaRef ds:uri="4ad8f8a2-17e7-49a9-8390-22f3c8f42b39"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -60060,20 +60071,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{31D0029D-E8A7-4DC9-B140-19D450DFB7E0}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BA99F9FA-472B-49CB-8CD8-32BE0FD0DC5E}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="e658002f-fdfe-4e4b-94aa-0526ee42a8ac"/>
-    <ds:schemaRef ds:uri="4ad8f8a2-17e7-49a9-8390-22f3c8f42b39"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
added function in parser for the ramp
</commit_message>
<xml_diff>
--- a/IVM6311_Testing_scripts.xlsx
+++ b/IVM6311_Testing_scripts.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\invlab\Documents\IVM6311ATE\IVM6311ATE\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9AE321D6-0E39-4A77-A663-78EFD2658DA9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{10E293D7-E2B4-4D8A-91F8-21158411646B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="693" firstSheet="1" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -44586,7 +44586,7 @@
         <rFont val="Calibri"/>
       </rPr>
       <t xml:space="preserve">
-Force__VBSO__Ramp__4.5V__0V</t>
+Forceramp__VBSO__4.5V__1V</t>
     </r>
     <r>
       <rPr>
@@ -59804,6 +59804,26 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="e658002f-fdfe-4e4b-94aa-0526ee42a8ac">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="4ad8f8a2-17e7-49a9-8390-22f3c8f42b39" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x010100C9B53A5B1F235B4EBDF9F22062DFC34D" ma:contentTypeVersion="12" ma:contentTypeDescription="Creare un nuovo documento." ma:contentTypeScope="" ma:versionID="ad5b12d537450e73edf2af95672e184c">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="e658002f-fdfe-4e4b-94aa-0526ee42a8ac" xmlns:ns3="4ad8f8a2-17e7-49a9-8390-22f3c8f42b39" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="ac16958afaf1bb0d1dccad67078e8e2c" ns2:_="" ns3:_="">
     <xsd:import namespace="e658002f-fdfe-4e4b-94aa-0526ee42a8ac"/>
@@ -60020,27 +60040,26 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="e658002f-fdfe-4e4b-94aa-0526ee42a8ac">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="4ad8f8a2-17e7-49a9-8390-22f3c8f42b39" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BA99F9FA-472B-49CB-8CD8-32BE0FD0DC5E}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7CBF6B91-9305-4674-87E0-A56D6B941238}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="e658002f-fdfe-4e4b-94aa-0526ee42a8ac"/>
+    <ds:schemaRef ds:uri="4ad8f8a2-17e7-49a9-8390-22f3c8f42b39"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{31D0029D-E8A7-4DC9-B140-19D450DFB7E0}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -60057,23 +60076,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7CBF6B91-9305-4674-87E0-A56D6B941238}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="e658002f-fdfe-4e4b-94aa-0526ee42a8ac"/>
-    <ds:schemaRef ds:uri="4ad8f8a2-17e7-49a9-8390-22f3c8f42b39"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BA99F9FA-472B-49CB-8CD8-32BE0FD0DC5E}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
modified dft_syntaxparser extract_forceramp_instruction and E3648A decresing_Ramp
</commit_message>
<xml_diff>
--- a/IVM6311_Testing_scripts.xlsx
+++ b/IVM6311_Testing_scripts.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\invlab\Documents\IVM6311ATE\IVM6311ATE\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{10E293D7-E2B4-4D8A-91F8-21158411646B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1CD2127-826C-4626-94A1-144CE59D62D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="693" firstSheet="1" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -44586,15 +44586,15 @@
         <rFont val="Calibri"/>
       </rPr>
       <t xml:space="preserve">
-Forceramp__VBSO__4.5V__1V</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-      </rPr>
-      <t xml:space="preserve"> "decrease VBSO from 4.5V with steps of 50mV untill FSYN and SDI toggle from Low to High"
+Ramp__VBSO__4.5V__1V </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve">"decrease VBSO from 4.5V with steps of 50mV untill FSYN and SDI toggle from Low to High"
 </t>
     </r>
     <r>
@@ -59804,26 +59804,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="e658002f-fdfe-4e4b-94aa-0526ee42a8ac">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="4ad8f8a2-17e7-49a9-8390-22f3c8f42b39" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x010100C9B53A5B1F235B4EBDF9F22062DFC34D" ma:contentTypeVersion="12" ma:contentTypeDescription="Creare un nuovo documento." ma:contentTypeScope="" ma:versionID="ad5b12d537450e73edf2af95672e184c">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="e658002f-fdfe-4e4b-94aa-0526ee42a8ac" xmlns:ns3="4ad8f8a2-17e7-49a9-8390-22f3c8f42b39" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="ac16958afaf1bb0d1dccad67078e8e2c" ns2:_="" ns3:_="">
     <xsd:import namespace="e658002f-fdfe-4e4b-94aa-0526ee42a8ac"/>
@@ -60040,10 +60020,41 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="e658002f-fdfe-4e4b-94aa-0526ee42a8ac">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="4ad8f8a2-17e7-49a9-8390-22f3c8f42b39" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BA99F9FA-472B-49CB-8CD8-32BE0FD0DC5E}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{31D0029D-E8A7-4DC9-B140-19D450DFB7E0}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="e658002f-fdfe-4e4b-94aa-0526ee42a8ac"/>
+    <ds:schemaRef ds:uri="4ad8f8a2-17e7-49a9-8390-22f3c8f42b39"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -60060,20 +60071,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{31D0029D-E8A7-4DC9-B140-19D450DFB7E0}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BA99F9FA-472B-49CB-8CD8-32BE0FD0DC5E}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="e658002f-fdfe-4e4b-94aa-0526ee42a8ac"/>
-    <ds:schemaRef ds:uri="4ad8f8a2-17e7-49a9-8390-22f3c8f42b39"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
BST boostrap working added function for ramp in E3648 and added in dft parser the instrction for extract the ramp operations
</commit_message>
<xml_diff>
--- a/IVM6311_Testing_scripts.xlsx
+++ b/IVM6311_Testing_scripts.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\invlab\Documents\IVM6311ATE\IVM6311ATE\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1CD2127-826C-4626-94A1-144CE59D62D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A4E59BA4-31B7-40F2-8277-54EAAE5FF313}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="693" firstSheet="1" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -44586,7 +44586,7 @@
         <rFont val="Calibri"/>
       </rPr>
       <t xml:space="preserve">
-Ramp__VBSO__4.5V__1V </t>
+Ramp__VBSO__4.5v__1v </t>
     </r>
     <r>
       <rPr>
@@ -59804,6 +59804,26 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="e658002f-fdfe-4e4b-94aa-0526ee42a8ac">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="4ad8f8a2-17e7-49a9-8390-22f3c8f42b39" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x010100C9B53A5B1F235B4EBDF9F22062DFC34D" ma:contentTypeVersion="12" ma:contentTypeDescription="Creare un nuovo documento." ma:contentTypeScope="" ma:versionID="ad5b12d537450e73edf2af95672e184c">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="e658002f-fdfe-4e4b-94aa-0526ee42a8ac" xmlns:ns3="4ad8f8a2-17e7-49a9-8390-22f3c8f42b39" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="ac16958afaf1bb0d1dccad67078e8e2c" ns2:_="" ns3:_="">
     <xsd:import namespace="e658002f-fdfe-4e4b-94aa-0526ee42a8ac"/>
@@ -60020,27 +60040,26 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="e658002f-fdfe-4e4b-94aa-0526ee42a8ac">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="4ad8f8a2-17e7-49a9-8390-22f3c8f42b39" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BA99F9FA-472B-49CB-8CD8-32BE0FD0DC5E}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7CBF6B91-9305-4674-87E0-A56D6B941238}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="e658002f-fdfe-4e4b-94aa-0526ee42a8ac"/>
+    <ds:schemaRef ds:uri="4ad8f8a2-17e7-49a9-8390-22f3c8f42b39"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{31D0029D-E8A7-4DC9-B140-19D450DFB7E0}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -60057,23 +60076,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7CBF6B91-9305-4674-87E0-A56D6B941238}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="e658002f-fdfe-4e4b-94aa-0526ee42a8ac"/>
-    <ds:schemaRef ds:uri="4ad8f8a2-17e7-49a9-8390-22f3c8f42b39"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BA99F9FA-472B-49CB-8CD8-32BE0FD0DC5E}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
almost all tests are working
</commit_message>
<xml_diff>
--- a/IVM6311_Testing_scripts.xlsx
+++ b/IVM6311_Testing_scripts.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\invlab\Documents\IVM6311ATE\IVM6311ATE\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A4E59BA4-31B7-40F2-8277-54EAAE5FF313}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87085ABF-6B5C-4043-B0E2-286644F0AD24}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="693" firstSheet="1" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1492" uniqueCount="436">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1494" uniqueCount="436">
   <si>
     <t>Revision</t>
   </si>
@@ -51618,8 +51618,12 @@
       <c r="Z8" s="69" t="s">
         <v>422</v>
       </c>
-      <c r="AA8" s="69"/>
-      <c r="AB8" s="69"/>
+      <c r="AA8" s="233" t="s">
+        <v>422</v>
+      </c>
+      <c r="AB8" s="233" t="s">
+        <v>422</v>
+      </c>
       <c r="AC8" s="11" t="s">
         <v>242</v>
       </c>
@@ -59804,26 +59808,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="e658002f-fdfe-4e4b-94aa-0526ee42a8ac">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="4ad8f8a2-17e7-49a9-8390-22f3c8f42b39" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x010100C9B53A5B1F235B4EBDF9F22062DFC34D" ma:contentTypeVersion="12" ma:contentTypeDescription="Creare un nuovo documento." ma:contentTypeScope="" ma:versionID="ad5b12d537450e73edf2af95672e184c">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="e658002f-fdfe-4e4b-94aa-0526ee42a8ac" xmlns:ns3="4ad8f8a2-17e7-49a9-8390-22f3c8f42b39" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="ac16958afaf1bb0d1dccad67078e8e2c" ns2:_="" ns3:_="">
     <xsd:import namespace="e658002f-fdfe-4e4b-94aa-0526ee42a8ac"/>
@@ -60040,10 +60024,41 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="e658002f-fdfe-4e4b-94aa-0526ee42a8ac">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="4ad8f8a2-17e7-49a9-8390-22f3c8f42b39" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BA99F9FA-472B-49CB-8CD8-32BE0FD0DC5E}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{31D0029D-E8A7-4DC9-B140-19D450DFB7E0}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="e658002f-fdfe-4e4b-94aa-0526ee42a8ac"/>
+    <ds:schemaRef ds:uri="4ad8f8a2-17e7-49a9-8390-22f3c8f42b39"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -60060,20 +60075,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{31D0029D-E8A7-4DC9-B140-19D450DFB7E0}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BA99F9FA-472B-49CB-8CD8-32BE0FD0DC5E}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="e658002f-fdfe-4e4b-94aa-0526ee42a8ac"/>
-    <ds:schemaRef ds:uri="4ad8f8a2-17e7-49a9-8390-22f3c8f42b39"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
boost tests working all together
</commit_message>
<xml_diff>
--- a/IVM6311_Testing_scripts.xlsx
+++ b/IVM6311_Testing_scripts.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\invlab\Documents\IVM6311ATE\IVM6311ATE\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87085ABF-6B5C-4043-B0E2-286644F0AD24}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57DF2B8A-9384-4766-B82F-D38867055CC4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="693" firstSheet="1" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -51378,7 +51378,7 @@
       <c r="K5" s="189" t="s">
         <v>427</v>
       </c>
-      <c r="L5" s="183" t="s">
+      <c r="L5" s="221" t="s">
         <v>412</v>
       </c>
       <c r="M5" s="221" t="s">
@@ -59808,6 +59808,26 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="e658002f-fdfe-4e4b-94aa-0526ee42a8ac">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="4ad8f8a2-17e7-49a9-8390-22f3c8f42b39" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x010100C9B53A5B1F235B4EBDF9F22062DFC34D" ma:contentTypeVersion="12" ma:contentTypeDescription="Creare un nuovo documento." ma:contentTypeScope="" ma:versionID="ad5b12d537450e73edf2af95672e184c">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="e658002f-fdfe-4e4b-94aa-0526ee42a8ac" xmlns:ns3="4ad8f8a2-17e7-49a9-8390-22f3c8f42b39" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="ac16958afaf1bb0d1dccad67078e8e2c" ns2:_="" ns3:_="">
     <xsd:import namespace="e658002f-fdfe-4e4b-94aa-0526ee42a8ac"/>
@@ -60024,27 +60044,26 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="e658002f-fdfe-4e4b-94aa-0526ee42a8ac">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="4ad8f8a2-17e7-49a9-8390-22f3c8f42b39" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BA99F9FA-472B-49CB-8CD8-32BE0FD0DC5E}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7CBF6B91-9305-4674-87E0-A56D6B941238}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="e658002f-fdfe-4e4b-94aa-0526ee42a8ac"/>
+    <ds:schemaRef ds:uri="4ad8f8a2-17e7-49a9-8390-22f3c8f42b39"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{31D0029D-E8A7-4DC9-B140-19D450DFB7E0}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -60061,23 +60080,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7CBF6B91-9305-4674-87E0-A56D6B941238}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="e658002f-fdfe-4e4b-94aa-0526ee42a8ac"/>
-    <ds:schemaRef ds:uri="4ad8f8a2-17e7-49a9-8390-22f3c8f42b39"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BA99F9FA-472B-49CB-8CD8-32BE0FD0DC5E}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
im modifing the boost tests, in particular zc
</commit_message>
<xml_diff>
--- a/IVM6311_Testing_scripts.xlsx
+++ b/IVM6311_Testing_scripts.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\invlab\Documents\IVM6311ATE\IVM6311ATE\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57DF2B8A-9384-4766-B82F-D38867055CC4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6FF782F5-2FCA-4B09-A9CD-C61098F56775}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="693" firstSheet="1" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32997,32 +32997,6 @@
     </r>
   </si>
   <si>
-    <t xml:space="preserve">"Run__startup
-Run__Boost_test_default
-Wait__delay__0.1ms
-0xFE_0x00 ""Select page 0""
-0xB0[1]_0x01 ""ocp en
-0xB2[1]_0x01 ""ls_sel on""
-0xC0[2:0]_0x01 ""OCP threshold set to 200mA""
-0xFE_0x01 ""Select page 1""
-0x1A_0x10 ""TSW to OCP Sense""
-Wait__delay__0.1ms
-0xFE_0x00 ""Select page 0""
-0xB2[0]_0x01 ""Power Force en""
-0xFE_0x01 ""Select page 1""
-Wait__delay__0.1ms
-0x15[2]_0x01 ""Force ocp""
-0x19[1]_0x01 ""bst_test en""
-Wait__delay__0.1ms
-Measure__Voltage__SDWN
-Trim__0xB2[5]_0xB1[3:0] ""trim in 2 different registers, what is the correct command""
-Calculate__MinError
-0x1A_0x00
-0x19_0x00
-"
-</t>
-  </si>
-  <si>
     <r>
       <t xml:space="preserve">Run_startup  
 </t>
@@ -40113,68 +40087,6 @@
   </si>
   <si>
     <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF00B0F0"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>0xFE_0x01</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> "Select page 1"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF00B0F0"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">0x0F_0x08
-0x10_0x08
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FFFF3399"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">FORCE__SDWN__OPEN
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF00B0F0"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>0x19_0x80</t>
-    </r>
-  </si>
-  <si>
-    <r>
       <t xml:space="preserve">Run_startup
 Run_Boost_test_default
 Run_Enable_Ana_Testpoint
@@ -42741,718 +42653,6 @@
         <scheme val="minor"/>
       </rPr>
       <t>0x1A_0x00
-0x19_0x00
-0x03_0x00
-0x04_0x00</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Run__startup
-Run__Boost_test_default
-Force__VBIAS__5V
-Force__VBSO__3.6V
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0070C0"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">0xFE_0x00 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>"Select page 0"</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0070C0"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">
-0x00_0x0F </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>"Power-up"</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0070C0"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">
-0xB0_0x00 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>"en 1 bst low"</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0070C0"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">
-0xB1_0x00</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> "en 2 bst low"</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0070C0"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">
-0xB3[4:3]_0x00</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> "en 3 bst low"</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0070C0"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">
-0x18[6]_0x01 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>"Enable Mirr"</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0070C0"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">
-0xFE_0x00 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>"Select page 0"</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0070C0"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">
-0xB1[6]_0x01</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> "Bootstrap en"</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0070C0"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">
-0xB2[1]_0x00</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> "ls_sel off"</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0070C0"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">
-0xB4[2:0]_0x06</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> "hsa_hsb on byp off"</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0070C0"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">
-0xFE_0x01 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>"Select page 1"</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0070C0"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">
-0x17[6]_0x01 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>"Force Mirr"</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0070C0"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">
-0x16[6]_0x01</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> "Force Bootstrap"</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0070C0"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FFFF3399"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="4" tint="-0.249977111117893"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>Wait__delay__0.1ms</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FFFF3399"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0070C0"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>0xFE_0x00</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> "Select page 0"</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0070C0"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">
-0xB0[6]_0x01</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> "zc en"</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0070C0"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">
-0xB0[0]_0x01 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>"bst en"</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0070C0"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">
-0xCA_0x10 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>"bst bso"</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0070C0"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">
-0xFE_0x01 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>"Select page 1"</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0070C0"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">
-0x0F[4]_0x01 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>"force bst bso"</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0070C0"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">
-0x15[4]_0x01 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>"force bst en"</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0070C0"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">
-0x16[7]_0x01 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>"force bst zc en"</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0070C0"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">
-0x03_0x04 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>"FSYN en"</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0070C0"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">
-0x04_0x16 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>"FSYN=bst_zc1 "</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0070C0"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FFFF3399"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="4" tint="-0.249977111117893"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>Wait__delay__0.1ms</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FFFF3399"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0070C0"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">0xFE_0x00 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>"Select page 0"</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0070C0"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">
-0xB2[0]_0x01</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> "Power Force en"</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0070C0"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">
-0xFE_0x01 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>"Select page 1"</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0070C0"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF002060"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="4" tint="-0.249977111117893"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>Wait__delay__0.1ms</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF002060"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FFFF3399"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">
-Force__SW__-100mA"sink current -100mA"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0070C0"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">0x19[1]_0x01 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>"bst_test en"</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FFFF3399"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="4" tint="-0.249977111117893"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">Wait__delay__0.1ms
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FFFF3399"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">
-Measure__Voltage__FSYN "it should be 1"
-Force__SW__100mA "inject"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="4" tint="-0.249977111117893"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>Wait__delay__0.1ms</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF002060"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FFFF3399"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">
-Measure__Voltage__FSYN "it should be 0"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="4" tint="-0.249977111117893"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>Wait__delay__0.1ms</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FFFF3399"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0070C0"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">
 0x19_0x00
 0x03_0x00
 0x04_0x00</t>
@@ -44678,6 +43878,1232 @@
 0x04_0x00
 0x1A_0x00
 0x19_0x00</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF00B0F0"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>0xFE_0x01</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> "Select page 1"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF00B0F0"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">0x0F_0x88
+0x10_0x08
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF3399"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">FORCE__SDWN__OPEN
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF00B0F0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>0x19_0x80</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Run__startup
+Run__Boost_test_default
+Run__Enable_Ana_Testpoint
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF7030A0"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Wait__delay__0.1ms
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF3399"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF4472C4"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>0xFE_0x00</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> "Select page 0"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF4472C4"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>0xB0[1]_0x01</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> "ocp en
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF4472C4"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>0xB2[1]_0x01</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> "ls_sel on"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF4472C4"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>0xC0[2:0]_0x03</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> "OCP threshold set to 400mA"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF4472C4"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">0xFE_0x01 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">"Select page 1"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF4472C4"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>0x1A_0x10</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> "TSW to OCP Sense"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0070C0"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">0x03_0x07 </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">"FSYN testpoint enable"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0070C0"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">0x04_0x18 </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">"FSYN = ana_bst_ocp_1"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF3399"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF7030A0"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Wait__delay__0.1ms
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF4472C4"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+0xFE_0x00</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> "Select page 0"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF4472C4"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>0xB2[0]_0x01</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> "Power Force en"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF4472C4"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>0xFE_0x01</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> "Select page 1"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0070C0"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">0x0F_0x80
+0xB0_0x0E
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF7030A0"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Wait__delay__0.1ms
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF4472C4"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>0x15[2]_0x01</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> "Force ocp"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF4472C4"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>0x19[1]_0x01</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> "bst_test en"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF7030A0"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Wait__delay__0.1ms
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF70AD47"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Measure__Voltage__SDWN </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">"optional"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF00B050"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Force__SW__400mA
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF9BC2E6"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+TrimSweep - </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFC65911"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>0xB2[5]_0xB1[3:0]</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF9BC2E6"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>"</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFED7D31"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>trim in 2 different registers - Sweep codes starting from b0000,1111 to b0000,0000 than from b0001,1111 to b0001,0000</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF3399"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF00B050"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Measure_Voltage_FSYN</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> "Check the transition Low to High"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF3399"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF4472C4"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">0x1A_0x00
+0x19_0x00
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFC65911"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Run__startup
+Run__Boost_test_default
+Force__VBIAS__5V
+Force__VBSO__3.6V
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0070C0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">0xFE_0x00 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>"Select page 0"</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0070C0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+0x00_0x0F </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>"Power-up"</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0070C0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+0xB0_0x00 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>"en 1 bst low"</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0070C0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+0xB1_0x00</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> "en 2 bst low"</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0070C0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+0xB3[4:3]_0x00</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> "en 3 bst low"</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0070C0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+0x18[6]_0x01 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>"Enable Mirr"</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0070C0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+0xFE_0x00 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>"Select page 0"</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0070C0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+0xB1[6]_0x01</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> "Bootstrap en"</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0070C0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+0xB2[1]_0x00</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> "ls_sel off"</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0070C0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+0xB4[2:0]_0x06</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> "hsa_hsb on byp off"</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0070C0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+0xFE_0x01 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>"Select page 1"</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0070C0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+0x17[6]_0x01 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>"Force Mirr"</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0070C0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+0x16[6]_0x01</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> "Force Bootstrap"</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0070C0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF3399"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="4" tint="-0.249977111117893"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Wait__delay__0.1ms</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF3399"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0070C0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>0xFE_0x00</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> "Select page 0"</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0070C0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+0xB0[6]_0x01</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> "zc en"</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0070C0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+0xB0[0]_0x01 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>"bst en"</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0070C0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+0xCA_0x10 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>"bst bso"</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0070C0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+0xFE_0x01 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>"Select page 1"</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0070C0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+0x0F[4]_0x01 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>"force bst bso"</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0070C0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+0x15[4]_0x01 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>"force bst en"</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0070C0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+0x16[7]_0x01 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>"force bst zc en"</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0070C0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+0x03_0x04 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>"FSYN en"</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0070C0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+0x04_0x16 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>"FSYN=bst_zc1 "</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0070C0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF3399"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="4" tint="-0.249977111117893"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Wait__delay__0.1ms</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF3399"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0070C0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">0xFE_0x00 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>"Select page 0"</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0070C0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+0xB2[0]_0x01</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> "Power Force en"</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0070C0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+0xFE_0x01 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>"Select page 1"</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0070C0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF002060"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="4" tint="-0.249977111117893"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Wait__delay__0.1ms
+0x19[1]_0x01 "bst_test en"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF3399"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Force__SW__220mA</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="4" tint="-0.249977111117893"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> "inject"
+Wait__delay__0.1ms
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF3399"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Measure__Voltage__FSYN</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="4" tint="-0.249977111117893"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> "it should be 0"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF002060"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF3399"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+Force__SW__-100mA"sink current -100mA"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0070C0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Wait__delay__0.1ms</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF3399"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+Measure__Voltage__FSYN "it should be 0"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0070C0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+0x19_0x00
+0x03_0x00
+0x04_0x00</t>
     </r>
   </si>
 </sst>
@@ -46504,12 +46930,12 @@
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <mruColors>
+      <color rgb="FFFF3399"/>
       <color rgb="FFFF33CC"/>
       <color rgb="FFFF66FF"/>
       <color rgb="FF00CC00"/>
       <color rgb="FFFF6699"/>
       <color rgb="FF8D77F9"/>
-      <color rgb="FFFF3399"/>
       <color rgb="FF28CF75"/>
       <color rgb="FF00D0C6"/>
       <color rgb="FF2DFFF5"/>
@@ -47962,7 +48388,7 @@
     <col min="2" max="2" width="36.140625" bestFit="1" customWidth="1"/>
     <col min="3" max="4" width="73.42578125" customWidth="1"/>
     <col min="5" max="5" width="62.7109375" customWidth="1"/>
-    <col min="6" max="6" width="57.5703125" customWidth="1"/>
+    <col min="6" max="6" width="59.28515625" style="101" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="21" x14ac:dyDescent="0.35">
@@ -47979,8 +48405,8 @@
       <c r="E1" s="9" t="s">
         <v>144</v>
       </c>
-      <c r="F1" s="65" t="s">
-        <v>102</v>
+      <c r="F1" s="17" t="s">
+        <v>138</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="21" x14ac:dyDescent="0.35">
@@ -47995,8 +48421,8 @@
       <c r="E2" s="16" t="s">
         <v>139</v>
       </c>
-      <c r="F2" s="16" t="s">
-        <v>139</v>
+      <c r="F2" s="206" t="s">
+        <v>220</v>
       </c>
     </row>
     <row r="3" spans="1:6" ht="21" x14ac:dyDescent="0.35">
@@ -48013,7 +48439,7 @@
       <c r="E3" s="15" t="s">
         <v>99</v>
       </c>
-      <c r="F3" s="64" t="s">
+      <c r="F3" s="205" t="s">
         <v>65</v>
       </c>
     </row>
@@ -48031,7 +48457,7 @@
       <c r="E4" s="9" t="s">
         <v>144</v>
       </c>
-      <c r="F4" s="65" t="s">
+      <c r="F4" s="138" t="s">
         <v>102</v>
       </c>
     </row>
@@ -48039,16 +48465,16 @@
       <c r="A5" s="235"/>
       <c r="B5" s="236"/>
       <c r="C5" s="204" t="s">
+        <v>417</v>
+      </c>
+      <c r="D5" s="204" t="s">
         <v>418</v>
       </c>
-      <c r="D5" s="204" t="s">
-        <v>419</v>
-      </c>
       <c r="E5" s="204" t="s">
-        <v>404</v>
-      </c>
-      <c r="F5" s="189" t="s">
-        <v>392</v>
+        <v>403</v>
+      </c>
+      <c r="F5" s="188" t="s">
+        <v>434</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="22.5" x14ac:dyDescent="0.3">
@@ -48063,9 +48489,9 @@
       </c>
       <c r="D6" s="38"/>
       <c r="E6" s="38" t="s">
-        <v>406</v>
-      </c>
-      <c r="F6" s="67"/>
+        <v>405</v>
+      </c>
+      <c r="F6" s="139"/>
     </row>
     <row r="7" spans="1:6" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A7" s="237"/>
@@ -48077,7 +48503,7 @@
       </c>
       <c r="D7" s="217"/>
       <c r="E7" s="8"/>
-      <c r="F7" s="68"/>
+      <c r="F7" s="140"/>
     </row>
     <row r="8" spans="1:6" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A8" s="237"/>
@@ -48088,12 +48514,12 @@
         <v>208</v>
       </c>
       <c r="D8" s="11" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="E8" s="11" t="s">
-        <v>405</v>
-      </c>
-      <c r="F8" s="69"/>
+        <v>404</v>
+      </c>
+      <c r="F8" s="141"/>
     </row>
     <row r="9" spans="1:6" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A9" s="237"/>
@@ -48105,7 +48531,7 @@
       </c>
       <c r="D9" s="39"/>
       <c r="E9" s="230"/>
-      <c r="F9" s="71"/>
+      <c r="F9" s="142"/>
     </row>
     <row r="10" spans="1:6" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A10" s="237"/>
@@ -48117,9 +48543,9 @@
       </c>
       <c r="D10" s="8"/>
       <c r="E10" s="229" t="s">
-        <v>407</v>
-      </c>
-      <c r="F10" s="68"/>
+        <v>406</v>
+      </c>
+      <c r="F10" s="140"/>
     </row>
     <row r="11" spans="1:6" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A11" s="4"/>
@@ -48135,7 +48561,7 @@
       <c r="E11" s="5" t="s">
         <v>156</v>
       </c>
-      <c r="F11" s="72"/>
+      <c r="F11" s="143"/>
     </row>
     <row r="12" spans="1:6" ht="42" x14ac:dyDescent="0.35">
       <c r="A12" s="6" t="s">
@@ -48153,7 +48579,7 @@
       <c r="E12" s="7" t="s">
         <v>159</v>
       </c>
-      <c r="F12" s="7"/>
+      <c r="F12" s="100"/>
     </row>
     <row r="13" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A13" s="18" t="s">
@@ -48171,7 +48597,7 @@
       <c r="E13" s="49" t="s">
         <v>162</v>
       </c>
-      <c r="F13" s="85" t="s">
+      <c r="F13" s="144" t="s">
         <v>163</v>
       </c>
     </row>
@@ -48191,7 +48617,7 @@
       <c r="E14" s="50" t="s">
         <v>162</v>
       </c>
-      <c r="F14" s="85" t="s">
+      <c r="F14" s="144" t="s">
         <v>163</v>
       </c>
     </row>
@@ -48212,7 +48638,7 @@
         <v>168</v>
       </c>
       <c r="F15" s="85" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
     </row>
     <row r="16" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
@@ -48231,7 +48657,7 @@
       <c r="E16" s="50" t="s">
         <v>168</v>
       </c>
-      <c r="F16" s="85" t="s">
+      <c r="F16" s="144" t="s">
         <v>171</v>
       </c>
     </row>
@@ -48249,7 +48675,7 @@
         <v>174</v>
       </c>
       <c r="E17" s="50"/>
-      <c r="F17" s="85" t="s">
+      <c r="F17" s="144" t="s">
         <v>175</v>
       </c>
     </row>
@@ -48263,7 +48689,7 @@
       <c r="C18" s="50"/>
       <c r="D18" s="50"/>
       <c r="E18" s="50"/>
-      <c r="F18" s="85"/>
+      <c r="F18" s="144"/>
     </row>
     <row r="19" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A19" s="20" t="s">
@@ -48275,7 +48701,7 @@
       <c r="C19" s="50"/>
       <c r="D19" s="50"/>
       <c r="E19" s="50"/>
-      <c r="F19" s="85"/>
+      <c r="F19" s="144"/>
     </row>
     <row r="20" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A20" s="20" t="s">
@@ -48289,7 +48715,7 @@
       <c r="E20" s="50" t="s">
         <v>182</v>
       </c>
-      <c r="F20" s="85"/>
+      <c r="F20" s="144"/>
     </row>
     <row r="21" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A21" s="20" t="s">
@@ -48301,7 +48727,7 @@
       <c r="C21" s="50"/>
       <c r="D21" s="50"/>
       <c r="E21" s="50"/>
-      <c r="F21" s="85"/>
+      <c r="F21" s="144"/>
     </row>
     <row r="22" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A22" s="20" t="s">
@@ -48313,7 +48739,7 @@
       <c r="C22" s="50"/>
       <c r="D22" s="50"/>
       <c r="E22" s="50"/>
-      <c r="F22" s="87"/>
+      <c r="F22" s="145"/>
     </row>
     <row r="23" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A23" s="18" t="s">
@@ -48325,7 +48751,7 @@
       <c r="C23" s="49"/>
       <c r="D23" s="49"/>
       <c r="E23" s="49"/>
-      <c r="F23" s="84" t="s">
+      <c r="F23" s="146" t="s">
         <v>163</v>
       </c>
     </row>
@@ -48339,7 +48765,7 @@
       <c r="C24" s="50"/>
       <c r="D24" s="50"/>
       <c r="E24" s="50"/>
-      <c r="F24" s="85" t="s">
+      <c r="F24" s="144" t="s">
         <v>191</v>
       </c>
     </row>
@@ -48353,7 +48779,7 @@
       <c r="C25" s="50"/>
       <c r="D25" s="50"/>
       <c r="E25" s="50"/>
-      <c r="F25" s="85"/>
+      <c r="F25" s="144"/>
     </row>
     <row r="26" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A26" s="20" t="s">
@@ -48365,7 +48791,7 @@
       <c r="C26" s="50"/>
       <c r="D26" s="50"/>
       <c r="E26" s="50"/>
-      <c r="F26" s="85"/>
+      <c r="F26" s="144"/>
     </row>
     <row r="27" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A27" s="20" t="s">
@@ -48377,7 +48803,7 @@
       <c r="C27" s="50"/>
       <c r="D27" s="50"/>
       <c r="E27" s="50"/>
-      <c r="F27" s="85"/>
+      <c r="F27" s="144"/>
     </row>
     <row r="28" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A28" s="20" t="s">
@@ -48395,7 +48821,7 @@
       <c r="E28" s="50" t="s">
         <v>111</v>
       </c>
-      <c r="F28" s="85" t="s">
+      <c r="F28" s="144" t="s">
         <v>111</v>
       </c>
     </row>
@@ -48405,7 +48831,7 @@
       <c r="C29" s="50"/>
       <c r="D29" s="50"/>
       <c r="E29" s="50"/>
-      <c r="F29" s="76"/>
+      <c r="F29" s="147"/>
     </row>
     <row r="30" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A30" s="52"/>
@@ -48413,7 +48839,7 @@
       <c r="C30" s="50"/>
       <c r="D30" s="50"/>
       <c r="E30" s="50"/>
-      <c r="F30" s="76"/>
+      <c r="F30" s="147"/>
     </row>
     <row r="31" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A31" s="53"/>
@@ -48421,7 +48847,7 @@
       <c r="C31" s="51"/>
       <c r="D31" s="51"/>
       <c r="E31" s="50"/>
-      <c r="F31" s="80"/>
+      <c r="F31" s="147"/>
     </row>
     <row r="32" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A32" s="47"/>
@@ -48429,7 +48855,7 @@
       <c r="C32" s="51"/>
       <c r="D32" s="51"/>
       <c r="E32" s="50"/>
-      <c r="F32" s="80"/>
+      <c r="F32" s="147"/>
     </row>
     <row r="33" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A33" s="47"/>
@@ -48437,7 +48863,7 @@
       <c r="C33" s="51"/>
       <c r="D33" s="51"/>
       <c r="E33" s="50"/>
-      <c r="F33" s="80"/>
+      <c r="F33" s="147"/>
     </row>
     <row r="34" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A34" s="47"/>
@@ -48445,7 +48871,7 @@
       <c r="C34" s="51"/>
       <c r="D34" s="51"/>
       <c r="E34" s="50"/>
-      <c r="F34" s="80"/>
+      <c r="F34" s="147"/>
     </row>
     <row r="35" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A35" s="47"/>
@@ -48453,7 +48879,7 @@
       <c r="C35" s="51"/>
       <c r="D35" s="51"/>
       <c r="E35" s="50"/>
-      <c r="F35" s="80"/>
+      <c r="F35" s="147"/>
     </row>
     <row r="36" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A36" s="47"/>
@@ -48461,7 +48887,7 @@
       <c r="C36" s="51"/>
       <c r="D36" s="51"/>
       <c r="E36" s="50"/>
-      <c r="F36" s="80"/>
+      <c r="F36" s="147"/>
     </row>
     <row r="37" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A37" s="47"/>
@@ -48469,7 +48895,7 @@
       <c r="C37" s="51"/>
       <c r="D37" s="51"/>
       <c r="E37" s="50"/>
-      <c r="F37" s="80"/>
+      <c r="F37" s="147"/>
     </row>
     <row r="38" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A38" s="47"/>
@@ -48477,7 +48903,7 @@
       <c r="C38" s="51"/>
       <c r="D38" s="51"/>
       <c r="E38" s="50"/>
-      <c r="F38" s="80"/>
+      <c r="F38" s="147"/>
     </row>
     <row r="39" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A39" s="47"/>
@@ -48485,7 +48911,7 @@
       <c r="C39" s="51"/>
       <c r="D39" s="51"/>
       <c r="E39" s="50"/>
-      <c r="F39" s="80"/>
+      <c r="F39" s="147"/>
     </row>
     <row r="40" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A40" s="47"/>
@@ -48493,7 +48919,7 @@
       <c r="C40" s="51"/>
       <c r="D40" s="51"/>
       <c r="E40" s="50"/>
-      <c r="F40" s="80"/>
+      <c r="F40" s="147"/>
     </row>
     <row r="41" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A41" s="47"/>
@@ -48501,7 +48927,7 @@
       <c r="C41" s="51"/>
       <c r="D41" s="51"/>
       <c r="E41" s="50"/>
-      <c r="F41" s="80"/>
+      <c r="F41" s="147"/>
     </row>
     <row r="42" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A42" s="47"/>
@@ -48509,7 +48935,7 @@
       <c r="C42" s="51"/>
       <c r="D42" s="51"/>
       <c r="E42" s="50"/>
-      <c r="F42" s="80"/>
+      <c r="F42" s="147"/>
     </row>
     <row r="43" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A43" s="47"/>
@@ -48517,7 +48943,7 @@
       <c r="C43" s="51"/>
       <c r="D43" s="51"/>
       <c r="E43" s="50"/>
-      <c r="F43" s="80"/>
+      <c r="F43" s="147"/>
     </row>
     <row r="44" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A44" s="47"/>
@@ -48525,7 +48951,7 @@
       <c r="C44" s="51"/>
       <c r="D44" s="51"/>
       <c r="E44" s="50"/>
-      <c r="F44" s="80"/>
+      <c r="F44" s="147"/>
     </row>
     <row r="45" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A45" s="47"/>
@@ -48533,7 +48959,7 @@
       <c r="C45" s="51"/>
       <c r="D45" s="51"/>
       <c r="E45" s="50"/>
-      <c r="F45" s="80"/>
+      <c r="F45" s="147"/>
     </row>
     <row r="46" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A46" s="47"/>
@@ -48541,7 +48967,7 @@
       <c r="C46" s="51"/>
       <c r="D46" s="51"/>
       <c r="E46" s="50"/>
-      <c r="F46" s="80"/>
+      <c r="F46" s="147"/>
     </row>
     <row r="47" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A47" s="47"/>
@@ -48549,7 +48975,7 @@
       <c r="C47" s="51"/>
       <c r="D47" s="51"/>
       <c r="E47" s="50"/>
-      <c r="F47" s="80"/>
+      <c r="F47" s="147"/>
     </row>
     <row r="48" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A48" s="47"/>
@@ -48557,7 +48983,7 @@
       <c r="C48" s="51"/>
       <c r="D48" s="51"/>
       <c r="E48" s="50"/>
-      <c r="F48" s="80"/>
+      <c r="F48" s="147"/>
     </row>
     <row r="49" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A49" s="47"/>
@@ -48565,7 +48991,7 @@
       <c r="C49" s="51"/>
       <c r="D49" s="51"/>
       <c r="E49" s="50"/>
-      <c r="F49" s="80"/>
+      <c r="F49" s="147"/>
     </row>
     <row r="50" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A50" s="47"/>
@@ -48573,7 +48999,7 @@
       <c r="C50" s="51"/>
       <c r="D50" s="51"/>
       <c r="E50" s="50"/>
-      <c r="F50" s="80"/>
+      <c r="F50" s="147"/>
     </row>
     <row r="51" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A51" s="48"/>
@@ -48581,7 +49007,7 @@
       <c r="C51" s="50"/>
       <c r="D51" s="50"/>
       <c r="E51" s="50"/>
-      <c r="F51" s="76"/>
+      <c r="F51" s="147"/>
     </row>
     <row r="52" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A52" s="20"/>
@@ -48589,7 +49015,7 @@
       <c r="C52" s="50"/>
       <c r="D52" s="50"/>
       <c r="E52" s="50"/>
-      <c r="F52" s="76"/>
+      <c r="F52" s="147"/>
     </row>
     <row r="53" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A53" s="20"/>
@@ -48597,7 +49023,7 @@
       <c r="C53" s="50"/>
       <c r="D53" s="50"/>
       <c r="E53" s="50"/>
-      <c r="F53" s="76"/>
+      <c r="F53" s="147"/>
     </row>
     <row r="54" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A54" s="20"/>
@@ -48605,7 +49031,7 @@
       <c r="C54" s="50"/>
       <c r="D54" s="50"/>
       <c r="E54" s="50"/>
-      <c r="F54" s="76"/>
+      <c r="F54" s="147"/>
     </row>
     <row r="55" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A55" s="20"/>
@@ -48613,7 +49039,7 @@
       <c r="C55" s="50"/>
       <c r="D55" s="50"/>
       <c r="E55" s="50"/>
-      <c r="F55" s="76"/>
+      <c r="F55" s="147"/>
     </row>
     <row r="56" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A56" s="20"/>
@@ -48621,7 +49047,7 @@
       <c r="C56" s="50"/>
       <c r="D56" s="50"/>
       <c r="E56" s="50"/>
-      <c r="F56" s="76"/>
+      <c r="F56" s="147"/>
     </row>
     <row r="57" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A57" s="20"/>
@@ -48629,7 +49055,7 @@
       <c r="C57" s="50"/>
       <c r="D57" s="50"/>
       <c r="E57" s="50"/>
-      <c r="F57" s="76"/>
+      <c r="F57" s="147"/>
     </row>
     <row r="58" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A58" s="20"/>
@@ -48637,7 +49063,7 @@
       <c r="C58" s="50"/>
       <c r="D58" s="50"/>
       <c r="E58" s="50"/>
-      <c r="F58" s="76"/>
+      <c r="F58" s="147"/>
     </row>
     <row r="59" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A59" s="20"/>
@@ -48645,7 +49071,7 @@
       <c r="C59" s="50"/>
       <c r="D59" s="50"/>
       <c r="E59" s="50"/>
-      <c r="F59" s="76"/>
+      <c r="F59" s="147"/>
     </row>
     <row r="60" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A60" s="20"/>
@@ -48653,7 +49079,7 @@
       <c r="C60" s="50"/>
       <c r="D60" s="50"/>
       <c r="E60" s="50"/>
-      <c r="F60" s="76"/>
+      <c r="F60" s="147"/>
     </row>
     <row r="61" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A61" s="20"/>
@@ -48661,7 +49087,7 @@
       <c r="C61" s="50"/>
       <c r="D61" s="50"/>
       <c r="E61" s="50"/>
-      <c r="F61" s="76"/>
+      <c r="F61" s="147"/>
     </row>
     <row r="62" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A62" s="20"/>
@@ -48669,7 +49095,7 @@
       <c r="C62" s="50"/>
       <c r="D62" s="50"/>
       <c r="E62" s="50"/>
-      <c r="F62" s="76"/>
+      <c r="F62" s="147"/>
     </row>
     <row r="63" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A63" s="20"/>
@@ -48677,7 +49103,7 @@
       <c r="C63" s="22"/>
       <c r="D63" s="22"/>
       <c r="E63" s="22"/>
-      <c r="F63" s="75"/>
+      <c r="F63" s="148"/>
     </row>
     <row r="64" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A64" s="20"/>
@@ -48685,7 +49111,7 @@
       <c r="C64" s="22"/>
       <c r="D64" s="22"/>
       <c r="E64" s="22"/>
-      <c r="F64" s="75"/>
+      <c r="F64" s="148"/>
     </row>
     <row r="65" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A65" s="20"/>
@@ -48693,7 +49119,7 @@
       <c r="C65" s="22"/>
       <c r="D65" s="22"/>
       <c r="E65" s="22"/>
-      <c r="F65" s="75"/>
+      <c r="F65" s="148"/>
     </row>
     <row r="66" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A66" s="20"/>
@@ -48701,7 +49127,7 @@
       <c r="C66" s="22"/>
       <c r="D66" s="22"/>
       <c r="E66" s="22"/>
-      <c r="F66" s="75"/>
+      <c r="F66" s="148"/>
     </row>
     <row r="67" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A67" s="20"/>
@@ -48709,7 +49135,7 @@
       <c r="C67" s="22"/>
       <c r="D67" s="22"/>
       <c r="E67" s="22"/>
-      <c r="F67" s="75"/>
+      <c r="F67" s="148"/>
     </row>
     <row r="68" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A68" s="20"/>
@@ -48717,7 +49143,7 @@
       <c r="C68" s="22"/>
       <c r="D68" s="22"/>
       <c r="E68" s="22"/>
-      <c r="F68" s="75"/>
+      <c r="F68" s="148"/>
     </row>
     <row r="69" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A69" s="20"/>
@@ -48725,7 +49151,7 @@
       <c r="C69" s="22"/>
       <c r="D69" s="22"/>
       <c r="E69" s="22"/>
-      <c r="F69" s="75"/>
+      <c r="F69" s="148"/>
     </row>
     <row r="70" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A70" s="20"/>
@@ -48733,7 +49159,7 @@
       <c r="C70" s="22"/>
       <c r="D70" s="22"/>
       <c r="E70" s="22"/>
-      <c r="F70" s="75"/>
+      <c r="F70" s="148"/>
     </row>
     <row r="71" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A71" s="20"/>
@@ -48741,7 +49167,7 @@
       <c r="C71" s="22"/>
       <c r="D71" s="22"/>
       <c r="E71" s="22"/>
-      <c r="F71" s="75"/>
+      <c r="F71" s="148"/>
     </row>
     <row r="72" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A72" s="20"/>
@@ -48749,7 +49175,7 @@
       <c r="C72" s="22"/>
       <c r="D72" s="22"/>
       <c r="E72" s="22"/>
-      <c r="F72" s="75"/>
+      <c r="F72" s="148"/>
     </row>
     <row r="73" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A73" s="20"/>
@@ -48757,7 +49183,7 @@
       <c r="C73" s="22"/>
       <c r="D73" s="22"/>
       <c r="E73" s="22"/>
-      <c r="F73" s="75"/>
+      <c r="F73" s="148"/>
     </row>
     <row r="74" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A74" s="20"/>
@@ -48765,7 +49191,7 @@
       <c r="C74" s="22"/>
       <c r="D74" s="22"/>
       <c r="E74" s="22"/>
-      <c r="F74" s="75"/>
+      <c r="F74" s="148"/>
     </row>
     <row r="75" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A75" s="20"/>
@@ -48773,7 +49199,7 @@
       <c r="C75" s="22"/>
       <c r="D75" s="22"/>
       <c r="E75" s="22"/>
-      <c r="F75" s="75"/>
+      <c r="F75" s="148"/>
     </row>
     <row r="76" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A76" s="20"/>
@@ -48781,7 +49207,7 @@
       <c r="C76" s="22"/>
       <c r="D76" s="22"/>
       <c r="E76" s="22"/>
-      <c r="F76" s="75"/>
+      <c r="F76" s="148"/>
     </row>
     <row r="77" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A77" s="20"/>
@@ -48789,7 +49215,7 @@
       <c r="C77" s="22"/>
       <c r="D77" s="22"/>
       <c r="E77" s="22"/>
-      <c r="F77" s="75"/>
+      <c r="F77" s="148"/>
     </row>
     <row r="78" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A78" s="20"/>
@@ -48797,7 +49223,7 @@
       <c r="C78" s="22"/>
       <c r="D78" s="22"/>
       <c r="E78" s="22"/>
-      <c r="F78" s="75"/>
+      <c r="F78" s="148"/>
     </row>
     <row r="79" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A79" s="20"/>
@@ -48805,7 +49231,7 @@
       <c r="C79" s="22"/>
       <c r="D79" s="22"/>
       <c r="E79" s="22"/>
-      <c r="F79" s="75"/>
+      <c r="F79" s="148"/>
     </row>
     <row r="80" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A80" s="20"/>
@@ -48813,7 +49239,7 @@
       <c r="C80" s="22"/>
       <c r="D80" s="22"/>
       <c r="E80" s="22"/>
-      <c r="F80" s="75"/>
+      <c r="F80" s="148"/>
     </row>
     <row r="81" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A81" s="20"/>
@@ -48821,7 +49247,7 @@
       <c r="C81" s="22"/>
       <c r="D81" s="22"/>
       <c r="E81" s="22"/>
-      <c r="F81" s="75"/>
+      <c r="F81" s="148"/>
     </row>
     <row r="82" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A82" s="20"/>
@@ -48829,7 +49255,7 @@
       <c r="C82" s="22"/>
       <c r="D82" s="22"/>
       <c r="E82" s="22"/>
-      <c r="F82" s="75"/>
+      <c r="F82" s="148"/>
     </row>
     <row r="83" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A83" s="20"/>
@@ -48837,7 +49263,7 @@
       <c r="C83" s="22"/>
       <c r="D83" s="22"/>
       <c r="E83" s="22"/>
-      <c r="F83" s="75"/>
+      <c r="F83" s="148"/>
     </row>
     <row r="84" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A84" s="20"/>
@@ -48845,7 +49271,7 @@
       <c r="C84" s="22"/>
       <c r="D84" s="22"/>
       <c r="E84" s="22"/>
-      <c r="F84" s="75"/>
+      <c r="F84" s="148"/>
     </row>
     <row r="85" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A85" s="20"/>
@@ -48853,7 +49279,7 @@
       <c r="C85" s="22"/>
       <c r="D85" s="22"/>
       <c r="E85" s="22"/>
-      <c r="F85" s="75"/>
+      <c r="F85" s="148"/>
     </row>
     <row r="86" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A86" s="20"/>
@@ -48861,7 +49287,7 @@
       <c r="C86" s="22"/>
       <c r="D86" s="22"/>
       <c r="E86" s="22"/>
-      <c r="F86" s="75"/>
+      <c r="F86" s="148"/>
     </row>
     <row r="87" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A87" s="20"/>
@@ -48869,7 +49295,7 @@
       <c r="C87" s="22"/>
       <c r="D87" s="22"/>
       <c r="E87" s="22"/>
-      <c r="F87" s="75"/>
+      <c r="F87" s="148"/>
     </row>
     <row r="88" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A88" s="20"/>
@@ -48877,7 +49303,7 @@
       <c r="C88" s="22"/>
       <c r="D88" s="22"/>
       <c r="E88" s="22"/>
-      <c r="F88" s="75"/>
+      <c r="F88" s="148"/>
     </row>
     <row r="89" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A89" s="20"/>
@@ -48885,7 +49311,7 @@
       <c r="C89" s="22"/>
       <c r="D89" s="22"/>
       <c r="E89" s="22"/>
-      <c r="F89" s="75"/>
+      <c r="F89" s="148"/>
     </row>
     <row r="90" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A90" s="20"/>
@@ -48893,7 +49319,7 @@
       <c r="C90" s="22"/>
       <c r="D90" s="22"/>
       <c r="E90" s="22"/>
-      <c r="F90" s="75"/>
+      <c r="F90" s="148"/>
     </row>
     <row r="91" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A91" s="20"/>
@@ -48901,7 +49327,7 @@
       <c r="C91" s="22"/>
       <c r="D91" s="22"/>
       <c r="E91" s="22"/>
-      <c r="F91" s="75"/>
+      <c r="F91" s="148"/>
     </row>
     <row r="92" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A92" s="20"/>
@@ -48909,7 +49335,7 @@
       <c r="C92" s="22"/>
       <c r="D92" s="22"/>
       <c r="E92" s="22"/>
-      <c r="F92" s="75"/>
+      <c r="F92" s="148"/>
     </row>
     <row r="93" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A93" s="20"/>
@@ -48917,7 +49343,7 @@
       <c r="C93" s="22"/>
       <c r="D93" s="22"/>
       <c r="E93" s="22"/>
-      <c r="F93" s="75"/>
+      <c r="F93" s="148"/>
     </row>
     <row r="94" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A94" s="21"/>
@@ -48925,7 +49351,7 @@
       <c r="C94" s="19"/>
       <c r="D94" s="19"/>
       <c r="E94" s="19"/>
-      <c r="F94" s="73"/>
+      <c r="F94" s="149"/>
     </row>
     <row r="95" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A95" s="20"/>
@@ -48933,7 +49359,7 @@
       <c r="C95" s="22"/>
       <c r="D95" s="22"/>
       <c r="E95" s="22"/>
-      <c r="F95" s="75"/>
+      <c r="F95" s="148"/>
     </row>
     <row r="96" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A96" s="20"/>
@@ -48941,7 +49367,7 @@
       <c r="C96" s="22"/>
       <c r="D96" s="22"/>
       <c r="E96" s="22"/>
-      <c r="F96" s="75"/>
+      <c r="F96" s="148"/>
     </row>
     <row r="97" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A97" s="20"/>
@@ -48949,7 +49375,7 @@
       <c r="C97" s="22"/>
       <c r="D97" s="22"/>
       <c r="E97" s="22"/>
-      <c r="F97" s="75"/>
+      <c r="F97" s="148"/>
     </row>
     <row r="98" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A98" s="20"/>
@@ -48957,7 +49383,7 @@
       <c r="C98" s="22"/>
       <c r="D98" s="22"/>
       <c r="E98" s="22"/>
-      <c r="F98" s="75"/>
+      <c r="F98" s="148"/>
     </row>
     <row r="99" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A99" s="20"/>
@@ -48965,7 +49391,7 @@
       <c r="C99" s="22"/>
       <c r="D99" s="22"/>
       <c r="E99" s="22"/>
-      <c r="F99" s="75"/>
+      <c r="F99" s="148"/>
     </row>
     <row r="100" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A100" s="20"/>
@@ -48973,7 +49399,7 @@
       <c r="C100" s="22"/>
       <c r="D100" s="22"/>
       <c r="E100" s="22"/>
-      <c r="F100" s="75"/>
+      <c r="F100" s="148"/>
     </row>
     <row r="101" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A101" s="20"/>
@@ -48981,7 +49407,7 @@
       <c r="C101" s="19"/>
       <c r="D101" s="19"/>
       <c r="E101" s="19"/>
-      <c r="F101" s="73"/>
+      <c r="F101" s="149"/>
     </row>
     <row r="102" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A102" s="20"/>
@@ -48989,7 +49415,7 @@
       <c r="C102" s="22"/>
       <c r="D102" s="22"/>
       <c r="E102" s="22"/>
-      <c r="F102" s="75"/>
+      <c r="F102" s="148"/>
     </row>
     <row r="103" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A103" s="20"/>
@@ -48997,7 +49423,7 @@
       <c r="C103" s="22"/>
       <c r="D103" s="22"/>
       <c r="E103" s="22"/>
-      <c r="F103" s="75"/>
+      <c r="F103" s="148"/>
     </row>
     <row r="104" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A104" s="20"/>
@@ -49005,7 +49431,7 @@
       <c r="C104" s="22"/>
       <c r="D104" s="22"/>
       <c r="E104" s="22"/>
-      <c r="F104" s="75"/>
+      <c r="F104" s="148"/>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -51352,40 +51778,40 @@
       <c r="A5" s="240"/>
       <c r="B5" s="240"/>
       <c r="C5" s="183" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="D5" s="183" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="E5" s="183" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="F5" s="221" t="s">
-        <v>434</v>
+        <v>431</v>
       </c>
       <c r="G5" s="183" t="s">
+        <v>409</v>
+      </c>
+      <c r="H5" s="189" t="s">
+        <v>422</v>
+      </c>
+      <c r="I5" s="189" t="s">
         <v>410</v>
       </c>
-      <c r="H5" s="189" t="s">
-        <v>423</v>
-      </c>
-      <c r="I5" s="189" t="s">
+      <c r="J5" s="189" t="s">
+        <v>428</v>
+      </c>
+      <c r="K5" s="189" t="s">
+        <v>425</v>
+      </c>
+      <c r="L5" s="221" t="s">
         <v>411</v>
       </c>
-      <c r="J5" s="189" t="s">
-        <v>430</v>
-      </c>
-      <c r="K5" s="189" t="s">
-        <v>427</v>
-      </c>
-      <c r="L5" s="221" t="s">
+      <c r="M5" s="221" t="s">
         <v>412</v>
       </c>
-      <c r="M5" s="221" t="s">
-        <v>413</v>
-      </c>
       <c r="N5" s="183" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="O5" s="221" t="s">
         <v>231</v>
@@ -51397,22 +51823,22 @@
         <v>233</v>
       </c>
       <c r="R5" s="221" t="s">
-        <v>429</v>
+        <v>427</v>
       </c>
       <c r="S5" s="188" t="s">
         <v>234</v>
       </c>
       <c r="T5" s="189" t="s">
-        <v>431</v>
+        <v>429</v>
       </c>
       <c r="U5" s="189" t="s">
-        <v>432</v>
+        <v>430</v>
       </c>
       <c r="V5" s="189" t="s">
         <v>235</v>
       </c>
       <c r="W5" s="190" t="s">
-        <v>433</v>
+        <v>435</v>
       </c>
       <c r="X5" s="190" t="s">
         <v>236</v>
@@ -51421,13 +51847,13 @@
         <v>237</v>
       </c>
       <c r="Z5" s="190" t="s">
-        <v>435</v>
+        <v>432</v>
       </c>
       <c r="AA5" s="189" t="s">
+        <v>413</v>
+      </c>
+      <c r="AB5" s="189" t="s">
         <v>414</v>
-      </c>
-      <c r="AB5" s="189" t="s">
-        <v>415</v>
       </c>
       <c r="AC5" s="221" t="s">
         <v>238</v>
@@ -51553,7 +51979,7 @@
         <v>149</v>
       </c>
       <c r="C8" s="69" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="D8" s="69" t="s">
         <v>239</v>
@@ -51565,16 +51991,16 @@
         <v>44</v>
       </c>
       <c r="G8" s="69" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
       <c r="H8" s="69" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
       <c r="I8" s="69" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
       <c r="J8" s="69" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
       <c r="K8" s="69" t="s">
         <v>241</v>
@@ -51595,34 +52021,34 @@
         <v>240</v>
       </c>
       <c r="Q8" s="69" t="s">
-        <v>428</v>
+        <v>426</v>
       </c>
       <c r="R8" s="153" t="s">
         <v>239</v>
       </c>
       <c r="S8" s="141"/>
       <c r="T8" s="119" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
       <c r="U8" s="69" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
       <c r="V8" s="69" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
       <c r="W8" s="233" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
       <c r="X8" s="69"/>
       <c r="Y8" s="69"/>
       <c r="Z8" s="69" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
       <c r="AA8" s="233" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
       <c r="AB8" s="233" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
       <c r="AC8" s="11" t="s">
         <v>242</v>
@@ -55450,28 +55876,28 @@
         <v>272</v>
       </c>
       <c r="E5" s="203" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="F5" s="203" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="G5" s="203" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="H5" s="203" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="I5" s="203" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="J5" s="203" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="K5" s="203" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="L5" s="203" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="M5" s="202" t="s">
         <v>273</v>
@@ -57925,7 +58351,7 @@
       <c r="A5" s="242"/>
       <c r="B5" s="242"/>
       <c r="C5" s="208" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="D5" s="37" t="s">
         <v>386</v>
@@ -57949,10 +58375,10 @@
         <v>310</v>
       </c>
       <c r="K5" s="226" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="L5" s="226" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="M5" s="56"/>
     </row>
@@ -59762,10 +60188,10 @@
     </row>
     <row r="2" spans="1:13" s="91" customFormat="1" ht="408.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="83" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="B2" s="174" t="s">
-        <v>426</v>
+        <v>433</v>
       </c>
       <c r="C2" s="174" t="s">
         <v>385</v>
@@ -59774,7 +60200,7 @@
         <v>325</v>
       </c>
       <c r="E2" s="224" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="F2" s="83" t="s">
         <v>326</v>
@@ -59808,26 +60234,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="e658002f-fdfe-4e4b-94aa-0526ee42a8ac">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="4ad8f8a2-17e7-49a9-8390-22f3c8f42b39" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x010100C9B53A5B1F235B4EBDF9F22062DFC34D" ma:contentTypeVersion="12" ma:contentTypeDescription="Creare un nuovo documento." ma:contentTypeScope="" ma:versionID="ad5b12d537450e73edf2af95672e184c">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="e658002f-fdfe-4e4b-94aa-0526ee42a8ac" xmlns:ns3="4ad8f8a2-17e7-49a9-8390-22f3c8f42b39" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="ac16958afaf1bb0d1dccad67078e8e2c" ns2:_="" ns3:_="">
     <xsd:import namespace="e658002f-fdfe-4e4b-94aa-0526ee42a8ac"/>
@@ -60044,10 +60450,41 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="e658002f-fdfe-4e4b-94aa-0526ee42a8ac">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="4ad8f8a2-17e7-49a9-8390-22f3c8f42b39" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BA99F9FA-472B-49CB-8CD8-32BE0FD0DC5E}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{31D0029D-E8A7-4DC9-B140-19D450DFB7E0}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="e658002f-fdfe-4e4b-94aa-0526ee42a8ac"/>
+    <ds:schemaRef ds:uri="4ad8f8a2-17e7-49a9-8390-22f3c8f42b39"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -60064,20 +60501,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{31D0029D-E8A7-4DC9-B140-19D450DFB7E0}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BA99F9FA-472B-49CB-8CD8-32BE0FD0DC5E}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="e658002f-fdfe-4e4b-94aa-0526ee42a8ac"/>
-    <ds:schemaRef ds:uri="4ad8f8a2-17e7-49a9-8390-22f3c8f42b39"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
ZC not working. all the others tests are working
</commit_message>
<xml_diff>
--- a/IVM6311_Testing_scripts.xlsx
+++ b/IVM6311_Testing_scripts.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\invlab\Documents\IVM6311ATE\IVM6311ATE\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6FF782F5-2FCA-4B09-A9CD-C61098F56775}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D8CC5AC7-B8FF-412B-A85A-343013851D73}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="693" firstSheet="1" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36194,471 +36194,6 @@
   <si>
     <r>
       <t xml:space="preserve">Run__startup
-Run__Boost_test_default
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FFFF3399"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Force__VBSO_3.6V</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FFFF3399"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-Force__OUTP__ 0V </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">"PA positive output"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FFFF33CC"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Force__OUTN__0V</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> "PA negative output"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FFFF3399"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF7030A0"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">Wait__delay__0.1ms
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF4472C4"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-0xFE_0x00</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> "Select page 0"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF4472C4"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>0xB1[7]_0x01</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> "env_err en"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF4472C4"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>0xB0[0]_0x01</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> "bst general en"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF4472C4"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>0xFE_0x01</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> "Select page 1"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF4472C4"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>0x03_0x04</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> "FSYN en"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF4472C4"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>0x04_0x09</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> "FSYN=bst_env_err"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF7030A0"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">Wait__delay__0.1ms
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF4472C4"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-0xFE_0x00 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">"Select page 0"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF4472C4"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>0xB2[0]_0x01</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> "Power Force en"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF4472C4"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>0xFE_0x01</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> "Select page 1"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF4472C4"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>0x15[4]_0x01</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> "Force bst general en"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF7030A0"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">Wait__delay__0.1ms
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF4472C4"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>0x15[1]_0x01</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> "force env_err"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF4472C4"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>0x19[1]_0x01</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> "bst_test en"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF7030A0"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">Wait__delay__0.1ms
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF70AD47"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Measure__Voltage__FSYN</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> "it should be 0 since the ref is higher than the PA OUTPUT"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FFFF33CC"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Force__OUTP__3.6V</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> "PA positive output"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF7030A0"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">Wait__delay__0.1ms
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF70AD47"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Measure__Voltage__FSYN</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> "now it should be 1 since the PA output should be higher than the ref"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF4472C4"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>0xFE_0x01</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> "Select page 1"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF4472C4"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>0x19_0x00
-0x03_0x00
-0x04_0x00</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Run__startup
 </t>
     </r>
     <r>
@@ -44437,6 +43972,7 @@
 Run__Boost_test_default
 Force__VBIAS__5V
 Force__VBSO__3.6V
+Force__SW__3.6V
 </t>
     </r>
     <r>
@@ -45102,6 +44638,471 @@
       </rPr>
       <t xml:space="preserve">
 0x19_0x00
+0x03_0x00
+0x04_0x00</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Run__startup
+Run__Boost_test_default
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FFFF3399"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Force__VBSO__3.6V</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF3399"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Force__OUTP__ 0V </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">"PA positive output"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF33CC"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Force__OUTN__0V</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> "PA negative output"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF3399"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF7030A0"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Wait__delay__0.1ms
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF4472C4"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+0xFE_0x00</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> "Select page 0"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF4472C4"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>0xB1[7]_0x01</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> "env_err en"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF4472C4"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>0xB0[0]_0x01</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> "bst general en"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF4472C4"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>0xFE_0x01</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> "Select page 1"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF4472C4"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>0x03_0x04</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> "FSYN en"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF4472C4"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>0x04_0x09</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> "FSYN=bst_env_err"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF7030A0"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Wait__delay__0.1ms
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF4472C4"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+0xFE_0x00 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">"Select page 0"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF4472C4"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>0xB2[0]_0x01</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> "Power Force en"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF4472C4"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>0xFE_0x01</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> "Select page 1"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF4472C4"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>0x15[4]_0x01</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> "Force bst general en"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF7030A0"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Wait__delay__0.1ms
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF4472C4"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>0x15[1]_0x01</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> "force env_err"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF4472C4"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>0x19[1]_0x01</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> "bst_test en"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF7030A0"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Wait__delay__0.1ms
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF70AD47"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Measure__Voltage__FSYN</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> "it should be 0 since the ref is higher than the PA OUTPUT"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF33CC"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Force__OUTP__3.6V</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> "PA positive output"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF7030A0"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Wait__delay__0.1ms
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF70AD47"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Measure__Voltage__FSYN</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> "now it should be 1 since the PA output should be higher than the ref"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF4472C4"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>0xFE_0x01</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> "Select page 1"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF4472C4"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>0x19_0x00
 0x03_0x00
 0x04_0x00</t>
     </r>
@@ -48465,16 +48466,16 @@
       <c r="A5" s="235"/>
       <c r="B5" s="236"/>
       <c r="C5" s="204" t="s">
+        <v>416</v>
+      </c>
+      <c r="D5" s="204" t="s">
         <v>417</v>
-      </c>
-      <c r="D5" s="204" t="s">
-        <v>418</v>
       </c>
       <c r="E5" s="204" t="s">
         <v>403</v>
       </c>
       <c r="F5" s="188" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="22.5" x14ac:dyDescent="0.3">
@@ -51778,31 +51779,31 @@
       <c r="A5" s="240"/>
       <c r="B5" s="240"/>
       <c r="C5" s="183" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="D5" s="183" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="E5" s="183" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
       <c r="F5" s="221" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
       <c r="G5" s="183" t="s">
         <v>409</v>
       </c>
       <c r="H5" s="189" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
       <c r="I5" s="189" t="s">
         <v>410</v>
       </c>
       <c r="J5" s="189" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="K5" s="189" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="L5" s="221" t="s">
         <v>411</v>
@@ -51811,7 +51812,7 @@
         <v>412</v>
       </c>
       <c r="N5" s="183" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="O5" s="221" t="s">
         <v>231</v>
@@ -51823,22 +51824,22 @@
         <v>233</v>
       </c>
       <c r="R5" s="221" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
       <c r="S5" s="188" t="s">
         <v>234</v>
       </c>
       <c r="T5" s="189" t="s">
+        <v>428</v>
+      </c>
+      <c r="U5" s="189" t="s">
         <v>429</v>
-      </c>
-      <c r="U5" s="189" t="s">
-        <v>430</v>
       </c>
       <c r="V5" s="189" t="s">
         <v>235</v>
       </c>
       <c r="W5" s="190" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
       <c r="X5" s="190" t="s">
         <v>236</v>
@@ -51847,13 +51848,13 @@
         <v>237</v>
       </c>
       <c r="Z5" s="190" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
       <c r="AA5" s="189" t="s">
+        <v>435</v>
+      </c>
+      <c r="AB5" s="189" t="s">
         <v>413</v>
-      </c>
-      <c r="AB5" s="189" t="s">
-        <v>414</v>
       </c>
       <c r="AC5" s="221" t="s">
         <v>238</v>
@@ -51991,16 +51992,16 @@
         <v>44</v>
       </c>
       <c r="G8" s="69" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="H8" s="69" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="I8" s="69" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="J8" s="69" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="K8" s="69" t="s">
         <v>241</v>
@@ -52021,34 +52022,34 @@
         <v>240</v>
       </c>
       <c r="Q8" s="69" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="R8" s="153" t="s">
         <v>239</v>
       </c>
       <c r="S8" s="141"/>
       <c r="T8" s="119" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="U8" s="69" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="V8" s="69" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="W8" s="233" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="X8" s="69"/>
       <c r="Y8" s="69"/>
       <c r="Z8" s="69" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="AA8" s="233" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="AB8" s="233" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="AC8" s="11" t="s">
         <v>242</v>
@@ -60188,10 +60189,10 @@
     </row>
     <row r="2" spans="1:13" s="91" customFormat="1" ht="408.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="83" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="B2" s="174" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
       <c r="C2" s="174" t="s">
         <v>385</v>
@@ -60200,7 +60201,7 @@
         <v>325</v>
       </c>
       <c r="E2" s="224" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="F2" s="83" t="s">
         <v>326</v>
@@ -60234,6 +60235,26 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="e658002f-fdfe-4e4b-94aa-0526ee42a8ac">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="4ad8f8a2-17e7-49a9-8390-22f3c8f42b39" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x010100C9B53A5B1F235B4EBDF9F22062DFC34D" ma:contentTypeVersion="12" ma:contentTypeDescription="Creare un nuovo documento." ma:contentTypeScope="" ma:versionID="ad5b12d537450e73edf2af95672e184c">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="e658002f-fdfe-4e4b-94aa-0526ee42a8ac" xmlns:ns3="4ad8f8a2-17e7-49a9-8390-22f3c8f42b39" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="ac16958afaf1bb0d1dccad67078e8e2c" ns2:_="" ns3:_="">
     <xsd:import namespace="e658002f-fdfe-4e4b-94aa-0526ee42a8ac"/>
@@ -60450,27 +60471,26 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="e658002f-fdfe-4e4b-94aa-0526ee42a8ac">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="4ad8f8a2-17e7-49a9-8390-22f3c8f42b39" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BA99F9FA-472B-49CB-8CD8-32BE0FD0DC5E}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7CBF6B91-9305-4674-87E0-A56D6B941238}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="e658002f-fdfe-4e4b-94aa-0526ee42a8ac"/>
+    <ds:schemaRef ds:uri="4ad8f8a2-17e7-49a9-8390-22f3c8f42b39"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{31D0029D-E8A7-4DC9-B140-19D450DFB7E0}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -60487,23 +60507,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7CBF6B91-9305-4674-87E0-A56D6B941238}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="e658002f-fdfe-4e4b-94aa-0526ee42a8ac"/>
-    <ds:schemaRef ds:uri="4ad8f8a2-17e7-49a9-8390-22f3c8f42b39"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BA99F9FA-472B-49CB-8CD8-32BE0FD0DC5E}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
BST_ZC now is working
</commit_message>
<xml_diff>
--- a/IVM6311_Testing_scripts.xlsx
+++ b/IVM6311_Testing_scripts.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\invlab\Documents\IVM6311ATE\IVM6311ATE\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D8CC5AC7-B8FF-412B-A85A-343013851D73}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2803ECF-15AF-4D0C-BDC9-D3A873E638C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="693" firstSheet="1" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -43970,9 +43970,473 @@
     <r>
       <t xml:space="preserve">Run__startup
 Run__Boost_test_default
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FFFF3399"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Force__VBSO__3.6V</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF3399"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Force__OUTP__ 0V </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">"PA positive output"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF33CC"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Force__OUTN__0V</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> "PA negative output"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF3399"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF7030A0"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Wait__delay__0.1ms
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF4472C4"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+0xFE_0x00</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> "Select page 0"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF4472C4"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>0xB1[7]_0x01</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> "env_err en"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF4472C4"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>0xB0[0]_0x01</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> "bst general en"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF4472C4"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>0xFE_0x01</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> "Select page 1"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF4472C4"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>0x03_0x04</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> "FSYN en"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF4472C4"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>0x04_0x09</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> "FSYN=bst_env_err"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF7030A0"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Wait__delay__0.1ms
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF4472C4"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+0xFE_0x00 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">"Select page 0"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF4472C4"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>0xB2[0]_0x01</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> "Power Force en"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF4472C4"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>0xFE_0x01</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> "Select page 1"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF4472C4"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>0x15[4]_0x01</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> "Force bst general en"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF7030A0"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Wait__delay__0.1ms
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF4472C4"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>0x15[1]_0x01</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> "force env_err"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF4472C4"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>0x19[1]_0x01</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> "bst_test en"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF7030A0"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Wait__delay__0.1ms
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF70AD47"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Measure__Voltage__FSYN</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> "it should be 0 since the ref is higher than the PA OUTPUT"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF33CC"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Force__OUTP__3.6V</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> "PA positive output"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF7030A0"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Wait__delay__0.1ms
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF70AD47"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Measure__Voltage__FSYN</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> "now it should be 1 since the PA output should be higher than the ref"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF4472C4"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>0xFE_0x01</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> "Select page 1"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF4472C4"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>0x19_0x00
+0x03_0x00
+0x04_0x00</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Run__startup
+Run__Boost_test_default
 Force__VBIAS__5V
 Force__VBSO__3.6V
-Force__SW__3.6V
 </t>
     </r>
     <r>
@@ -44556,7 +45020,7 @@
         <rFont val="Calibri"/>
         <family val="2"/>
       </rPr>
-      <t>Force__SW__220mA</t>
+      <t>Force__SW__100mA</t>
     </r>
     <r>
       <rPr>
@@ -44638,471 +45102,6 @@
       </rPr>
       <t xml:space="preserve">
 0x19_0x00
-0x03_0x00
-0x04_0x00</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Run__startup
-Run__Boost_test_default
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FFFF3399"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Force__VBSO__3.6V</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FFFF3399"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-Force__OUTP__ 0V </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">"PA positive output"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FFFF33CC"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Force__OUTN__0V</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> "PA negative output"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FFFF3399"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF7030A0"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">Wait__delay__0.1ms
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF4472C4"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-0xFE_0x00</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> "Select page 0"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF4472C4"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>0xB1[7]_0x01</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> "env_err en"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF4472C4"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>0xB0[0]_0x01</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> "bst general en"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF4472C4"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>0xFE_0x01</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> "Select page 1"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF4472C4"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>0x03_0x04</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> "FSYN en"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF4472C4"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>0x04_0x09</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> "FSYN=bst_env_err"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF7030A0"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">Wait__delay__0.1ms
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF4472C4"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-0xFE_0x00 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">"Select page 0"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF4472C4"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>0xB2[0]_0x01</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> "Power Force en"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF4472C4"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>0xFE_0x01</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> "Select page 1"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF4472C4"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>0x15[4]_0x01</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> "Force bst general en"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF7030A0"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">Wait__delay__0.1ms
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF4472C4"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>0x15[1]_0x01</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> "force env_err"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF4472C4"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>0x19[1]_0x01</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> "bst_test en"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF7030A0"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">Wait__delay__0.1ms
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF70AD47"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Measure__Voltage__FSYN</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> "it should be 0 since the ref is higher than the PA OUTPUT"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FFFF33CC"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Force__OUTP__3.6V</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> "PA positive output"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF7030A0"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">Wait__delay__0.1ms
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF70AD47"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Measure__Voltage__FSYN</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> "now it should be 1 since the PA output should be higher than the ref"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF4472C4"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>0xFE_0x01</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> "Select page 1"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF4472C4"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>0x19_0x00
 0x03_0x00
 0x04_0x00</t>
     </r>
@@ -51839,7 +51838,7 @@
         <v>235</v>
       </c>
       <c r="W5" s="190" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="X5" s="190" t="s">
         <v>236</v>
@@ -51851,7 +51850,7 @@
         <v>431</v>
       </c>
       <c r="AA5" s="189" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
       <c r="AB5" s="189" t="s">
         <v>413</v>
@@ -60235,26 +60234,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="e658002f-fdfe-4e4b-94aa-0526ee42a8ac">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="4ad8f8a2-17e7-49a9-8390-22f3c8f42b39" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x010100C9B53A5B1F235B4EBDF9F22062DFC34D" ma:contentTypeVersion="12" ma:contentTypeDescription="Creare un nuovo documento." ma:contentTypeScope="" ma:versionID="ad5b12d537450e73edf2af95672e184c">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="e658002f-fdfe-4e4b-94aa-0526ee42a8ac" xmlns:ns3="4ad8f8a2-17e7-49a9-8390-22f3c8f42b39" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="ac16958afaf1bb0d1dccad67078e8e2c" ns2:_="" ns3:_="">
     <xsd:import namespace="e658002f-fdfe-4e4b-94aa-0526ee42a8ac"/>
@@ -60471,10 +60450,41 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="e658002f-fdfe-4e4b-94aa-0526ee42a8ac">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="4ad8f8a2-17e7-49a9-8390-22f3c8f42b39" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BA99F9FA-472B-49CB-8CD8-32BE0FD0DC5E}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{31D0029D-E8A7-4DC9-B140-19D450DFB7E0}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="e658002f-fdfe-4e4b-94aa-0526ee42a8ac"/>
+    <ds:schemaRef ds:uri="4ad8f8a2-17e7-49a9-8390-22f3c8f42b39"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -60491,20 +60501,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{31D0029D-E8A7-4DC9-B140-19D450DFB7E0}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BA99F9FA-472B-49CB-8CD8-32BE0FD0DC5E}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="e658002f-fdfe-4e4b-94aa-0526ee42a8ac"/>
-    <ds:schemaRef ds:uri="4ad8f8a2-17e7-49a9-8390-22f3c8f42b39"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
added function in dft_syntaxparser for single and double register trimming, started to write in the reference the bst_ocp_trim
</commit_message>
<xml_diff>
--- a/IVM6311_Testing_scripts.xlsx
+++ b/IVM6311_Testing_scripts.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\invlab\Documents\IVM6311ATE\IVM6311ATE\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2803ECF-15AF-4D0C-BDC9-D3A873E638C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{315617C6-53BF-4635-8BC4-70ABB34E066B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="693" firstSheet="1" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="693" firstSheet="1" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Revision" sheetId="3" r:id="rId1"/>
@@ -43481,495 +43481,6 @@
     <r>
       <t xml:space="preserve">Run__startup
 Run__Boost_test_default
-Run__Enable_Ana_Testpoint
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF7030A0"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">Wait__delay__0.1ms
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FFFF3399"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF4472C4"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>0xFE_0x00</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> "Select page 0"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF4472C4"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>0xB0[1]_0x01</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> "ocp en
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF4472C4"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>0xB2[1]_0x01</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> "ls_sel on"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF4472C4"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>0xC0[2:0]_0x03</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> "OCP threshold set to 400mA"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF4472C4"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">0xFE_0x01 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">"Select page 1"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF4472C4"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>0x1A_0x10</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> "TSW to OCP Sense"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0070C0"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">0x03_0x07 </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">"FSYN testpoint enable"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0070C0"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">0x04_0x18 </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">"FSYN = ana_bst_ocp_1"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FFFF3399"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF7030A0"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">Wait__delay__0.1ms
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF4472C4"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-0xFE_0x00</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> "Select page 0"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF4472C4"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>0xB2[0]_0x01</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> "Power Force en"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF4472C4"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>0xFE_0x01</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> "Select page 1"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0070C0"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">0x0F_0x80
-0xB0_0x0E
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF7030A0"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">Wait__delay__0.1ms
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF4472C4"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>0x15[2]_0x01</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> "Force ocp"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF4472C4"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>0x19[1]_0x01</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> "bst_test en"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF7030A0"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-Wait__delay__0.1ms
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF70AD47"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">Measure__Voltage__SDWN </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">"optional"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF00B050"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-Force__SW__400mA
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF9BC2E6"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-TrimSweep - </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FFC65911"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>0xB2[5]_0xB1[3:0]</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF9BC2E6"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>"</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FFED7D31"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>trim in 2 different registers - Sweep codes starting from b0000,1111 to b0000,0000 than from b0001,1111 to b0001,0000</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FFFF3399"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF00B050"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Measure_Voltage_FSYN</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> "Check the transition Low to High"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FFFF3399"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF4472C4"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">0x1A_0x00
-0x19_0x00
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FFC65911"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Run__startup
-Run__Boost_test_default
 </t>
     </r>
     <r>
@@ -45104,6 +44615,495 @@
 0x19_0x00
 0x03_0x00
 0x04_0x00</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Run__startup
+Run__Boost_test_default
+Run__Enable_Ana_Testpoint
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF7030A0"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Wait__delay__0.1ms
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF3399"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF4472C4"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>0xFE_0x00</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> "Select page 0"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF4472C4"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>0xB0[1]_0x01</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> "ocp en
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF4472C4"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>0xB2[1]_0x01</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> "ls_sel on"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF4472C4"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>0xC0[2:0]_0x03</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> "OCP threshold set to 400mA"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF4472C4"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">0xFE_0x01 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">"Select page 1"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF4472C4"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>0x1A_0x10</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> "TSW to OCP Sense"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0070C0"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">0x03_0x07 </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">"FSYN testpoint enable"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0070C0"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">0x04_0x18 </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">"FSYN = ana_bst_ocp_1"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF3399"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF7030A0"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Wait__delay__0.1ms
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF4472C4"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+0xFE_0x00</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> "Select page 0"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF4472C4"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>0xB2[0]_0x01</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> "Power Force en"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF4472C4"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>0xFE_0x01</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> "Select page 1"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0070C0"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">0x0F_0x80
+0xB0_0x0E
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF7030A0"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Wait__delay__0.1ms
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF4472C4"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>0x15[2]_0x01</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> "Force ocp"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF4472C4"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>0x19[1]_0x01</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> "bst_test en"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF7030A0"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Wait__delay__0.1ms
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF70AD47"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Measure__Voltage__SDWN </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">"optional"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF00B050"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Force__SW__400mA
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF9BC2E6"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+TrimSweep__</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFC65911"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>0xB2[5]__0xB1[3:0]</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF9BC2E6"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>"</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFED7D31"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>trim in 2 different registers - Sweep codes starting from b0000,1111 to b0000,0000 than from b0001,1111 to b0001,0000</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF3399"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF00B050"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Measure_Voltage_FSYN</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> "Check the transition Low to High"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF3399"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF4472C4"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">0x1A_0x00
+0x19_0x00
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFC65911"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
     </r>
   </si>
 </sst>
@@ -45115,7 +45115,7 @@
     <numFmt numFmtId="164" formatCode="#,##0.0"/>
     <numFmt numFmtId="165" formatCode="#,##0.000"/>
   </numFmts>
-  <fonts count="123" x14ac:knownFonts="1">
+  <fonts count="124" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -45903,6 +45903,14 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="15">
     <fill>
@@ -46301,7 +46309,7 @@
     <xf numFmtId="9" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="118" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="244">
+  <cellXfs count="245">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -46920,6 +46928,7 @@
     <xf numFmtId="3" fontId="26" fillId="7" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="123" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Normale" xfId="0" builtinId="0"/>
@@ -48382,7 +48391,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{67A58BE6-10B8-478E-A3FE-3CA6A691AC11}">
-  <dimension ref="A1:F104"/>
+  <dimension ref="A1:I104"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="36.140625" bestFit="1" customWidth="1"/>
@@ -48391,7 +48400,7 @@
     <col min="6" max="6" width="59.28515625" style="101" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="21" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:9" ht="21" x14ac:dyDescent="0.35">
       <c r="A1" s="234" t="s">
         <v>375</v>
       </c>
@@ -48405,11 +48414,11 @@
       <c r="E1" s="9" t="s">
         <v>144</v>
       </c>
-      <c r="F1" s="17" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" ht="21" x14ac:dyDescent="0.35">
+      <c r="F1" s="138" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" ht="21" x14ac:dyDescent="0.35">
       <c r="A2" s="2"/>
       <c r="B2" s="2"/>
       <c r="C2" s="16" t="s">
@@ -48425,7 +48434,7 @@
         <v>220</v>
       </c>
     </row>
-    <row r="3" spans="1:6" ht="21" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:9" ht="21" x14ac:dyDescent="0.35">
       <c r="A3" s="234" t="s">
         <v>140</v>
       </c>
@@ -48443,7 +48452,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="4" spans="1:6" ht="21" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:9" ht="21" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="234" t="s">
         <v>137</v>
       </c>
@@ -48461,7 +48470,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="5" spans="1:6" ht="409.5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A5" s="235"/>
       <c r="B5" s="236"/>
       <c r="C5" s="204" t="s">
@@ -48474,10 +48483,11 @@
         <v>403</v>
       </c>
       <c r="F5" s="188" t="s">
-        <v>433</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" ht="22.5" x14ac:dyDescent="0.3">
+        <v>435</v>
+      </c>
+      <c r="I5" s="244"/>
+    </row>
+    <row r="6" spans="1:9" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A6" s="237" t="s">
         <v>145</v>
       </c>
@@ -48493,7 +48503,7 @@
       </c>
       <c r="F6" s="139"/>
     </row>
-    <row r="7" spans="1:6" ht="22.5" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:9" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A7" s="237"/>
       <c r="B7" s="14" t="s">
         <v>147</v>
@@ -48505,7 +48515,7 @@
       <c r="E7" s="8"/>
       <c r="F7" s="140"/>
     </row>
-    <row r="8" spans="1:6" ht="22.5" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:9" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A8" s="237"/>
       <c r="B8" s="10" t="s">
         <v>149</v>
@@ -48521,7 +48531,7 @@
       </c>
       <c r="F8" s="141"/>
     </row>
-    <row r="9" spans="1:6" ht="22.5" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:9" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A9" s="237"/>
       <c r="B9" s="12" t="s">
         <v>151</v>
@@ -48533,7 +48543,7 @@
       <c r="E9" s="230"/>
       <c r="F9" s="142"/>
     </row>
-    <row r="10" spans="1:6" ht="22.5" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:9" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A10" s="237"/>
       <c r="B10" s="14" t="s">
         <v>152</v>
@@ -48547,7 +48557,7 @@
       </c>
       <c r="F10" s="140"/>
     </row>
-    <row r="11" spans="1:6" ht="22.5" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:9" ht="22.5" x14ac:dyDescent="0.3">
       <c r="A11" s="4"/>
       <c r="B11" s="4" t="s">
         <v>154</v>
@@ -48563,7 +48573,7 @@
       </c>
       <c r="F11" s="143"/>
     </row>
-    <row r="12" spans="1:6" ht="42" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:9" ht="42" x14ac:dyDescent="0.35">
       <c r="A12" s="6" t="s">
         <v>157</v>
       </c>
@@ -48581,7 +48591,7 @@
       </c>
       <c r="F12" s="100"/>
     </row>
-    <row r="13" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:9" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A13" s="18" t="s">
         <v>160</v>
       </c>
@@ -48601,7 +48611,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="14" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:9" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A14" s="20" t="s">
         <v>164</v>
       </c>
@@ -48621,7 +48631,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="15" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:9" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A15" s="20" t="s">
         <v>166</v>
       </c>
@@ -48641,7 +48651,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="16" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:9" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A16" s="20" t="s">
         <v>169</v>
       </c>
@@ -51838,7 +51848,7 @@
         <v>235</v>
       </c>
       <c r="W5" s="190" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
       <c r="X5" s="190" t="s">
         <v>236</v>
@@ -51850,7 +51860,7 @@
         <v>431</v>
       </c>
       <c r="AA5" s="189" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
       <c r="AB5" s="189" t="s">
         <v>413</v>
@@ -60234,6 +60244,26 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="e658002f-fdfe-4e4b-94aa-0526ee42a8ac">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="4ad8f8a2-17e7-49a9-8390-22f3c8f42b39" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x010100C9B53A5B1F235B4EBDF9F22062DFC34D" ma:contentTypeVersion="12" ma:contentTypeDescription="Creare un nuovo documento." ma:contentTypeScope="" ma:versionID="ad5b12d537450e73edf2af95672e184c">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="e658002f-fdfe-4e4b-94aa-0526ee42a8ac" xmlns:ns3="4ad8f8a2-17e7-49a9-8390-22f3c8f42b39" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="ac16958afaf1bb0d1dccad67078e8e2c" ns2:_="" ns3:_="">
     <xsd:import namespace="e658002f-fdfe-4e4b-94aa-0526ee42a8ac"/>
@@ -60450,27 +60480,26 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="e658002f-fdfe-4e4b-94aa-0526ee42a8ac">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="4ad8f8a2-17e7-49a9-8390-22f3c8f42b39" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BA99F9FA-472B-49CB-8CD8-32BE0FD0DC5E}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7CBF6B91-9305-4674-87E0-A56D6B941238}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="e658002f-fdfe-4e4b-94aa-0526ee42a8ac"/>
+    <ds:schemaRef ds:uri="4ad8f8a2-17e7-49a9-8390-22f3c8f42b39"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{31D0029D-E8A7-4DC9-B140-19D450DFB7E0}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -60487,23 +60516,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7CBF6B91-9305-4674-87E0-A56D6B941238}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="e658002f-fdfe-4e4b-94aa-0526ee42a8ac"/>
-    <ds:schemaRef ds:uri="4ad8f8a2-17e7-49a9-8390-22f3c8f42b39"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BA99F9FA-472B-49CB-8CD8-32BE0FD0DC5E}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
adding trimming for bst_ocp_trim and modified class reference (added execute boost test default, signal for the ocp_tri_test
</commit_message>
<xml_diff>
--- a/IVM6311_Testing_scripts.xlsx
+++ b/IVM6311_Testing_scripts.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\invlab\Documents\IVM6311ATE\IVM6311ATE\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{323EBC44-2FB1-421A-A55A-1D4805D961BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F21B56F-B518-4CF6-85C1-4E9EF1F2E89A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="693" firstSheet="1" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -46898,6 +46898,13 @@
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="123" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="124" fillId="3" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="4" fillId="6" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="2" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
@@ -46927,13 +46934,6 @@
     </xf>
     <xf numFmtId="3" fontId="26" fillId="7" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="124" fillId="3" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="4" fillId="6" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="2" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -48407,10 +48407,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="21" x14ac:dyDescent="0.35">
-      <c r="A1" s="235" t="s">
+      <c r="A1" s="238" t="s">
         <v>374</v>
       </c>
-      <c r="B1" s="235"/>
+      <c r="B1" s="238"/>
       <c r="C1" s="9" t="s">
         <v>142</v>
       </c>
@@ -48441,10 +48441,10 @@
       </c>
     </row>
     <row r="3" spans="1:9" ht="21" x14ac:dyDescent="0.35">
-      <c r="A3" s="235" t="s">
+      <c r="A3" s="238" t="s">
         <v>140</v>
       </c>
-      <c r="B3" s="235"/>
+      <c r="B3" s="238"/>
       <c r="C3" s="15" t="s">
         <v>60</v>
       </c>
@@ -48459,10 +48459,10 @@
       </c>
     </row>
     <row r="4" spans="1:9" ht="21" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="235" t="s">
+      <c r="A4" s="238" t="s">
         <v>137</v>
       </c>
-      <c r="B4" s="235"/>
+      <c r="B4" s="238"/>
       <c r="C4" s="9" t="s">
         <v>142</v>
       </c>
@@ -48477,8 +48477,8 @@
       </c>
     </row>
     <row r="5" spans="1:9" ht="409.5" x14ac:dyDescent="0.25">
-      <c r="A5" s="236"/>
-      <c r="B5" s="237"/>
+      <c r="A5" s="239"/>
+      <c r="B5" s="240"/>
       <c r="C5" s="204" t="s">
         <v>415</v>
       </c>
@@ -48494,7 +48494,7 @@
       <c r="I5" s="234"/>
     </row>
     <row r="6" spans="1:9" ht="22.5" x14ac:dyDescent="0.3">
-      <c r="A6" s="238" t="s">
+      <c r="A6" s="241" t="s">
         <v>145</v>
       </c>
       <c r="B6" s="13" t="s">
@@ -48510,7 +48510,7 @@
       <c r="F6" s="139"/>
     </row>
     <row r="7" spans="1:9" ht="22.5" x14ac:dyDescent="0.3">
-      <c r="A7" s="238"/>
+      <c r="A7" s="241"/>
       <c r="B7" s="14" t="s">
         <v>147</v>
       </c>
@@ -48522,7 +48522,7 @@
       <c r="F7" s="140"/>
     </row>
     <row r="8" spans="1:9" ht="22.5" x14ac:dyDescent="0.3">
-      <c r="A8" s="238"/>
+      <c r="A8" s="241"/>
       <c r="B8" s="10" t="s">
         <v>149</v>
       </c>
@@ -48535,12 +48535,12 @@
       <c r="E8" s="11" t="s">
         <v>403</v>
       </c>
-      <c r="F8" s="246" t="s">
+      <c r="F8" s="236" t="s">
         <v>419</v>
       </c>
     </row>
     <row r="9" spans="1:9" ht="22.5" x14ac:dyDescent="0.3">
-      <c r="A9" s="238"/>
+      <c r="A9" s="241"/>
       <c r="B9" s="12" t="s">
         <v>151</v>
       </c>
@@ -48552,7 +48552,7 @@
       <c r="F9" s="142"/>
     </row>
     <row r="10" spans="1:9" ht="22.5" x14ac:dyDescent="0.3">
-      <c r="A10" s="238"/>
+      <c r="A10" s="241"/>
       <c r="B10" s="14" t="s">
         <v>152</v>
       </c>
@@ -48579,7 +48579,7 @@
       <c r="E11" s="5" t="s">
         <v>434</v>
       </c>
-      <c r="F11" s="247" t="s">
+      <c r="F11" s="237" t="s">
         <v>155</v>
       </c>
     </row>
@@ -49477,10 +49477,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="21" x14ac:dyDescent="0.35">
-      <c r="A1" s="235" t="s">
+      <c r="A1" s="238" t="s">
         <v>137</v>
       </c>
-      <c r="B1" s="235"/>
+      <c r="B1" s="238"/>
       <c r="C1" s="17" t="s">
         <v>138</v>
       </c>
@@ -49511,10 +49511,10 @@
       </c>
     </row>
     <row r="3" spans="1:6" ht="21" x14ac:dyDescent="0.35">
-      <c r="A3" s="235" t="s">
+      <c r="A3" s="238" t="s">
         <v>140</v>
       </c>
-      <c r="B3" s="235"/>
+      <c r="B3" s="238"/>
       <c r="C3" s="15" t="s">
         <v>79</v>
       </c>
@@ -49529,10 +49529,10 @@
       </c>
     </row>
     <row r="4" spans="1:6" ht="21" x14ac:dyDescent="0.35">
-      <c r="A4" s="235" t="s">
+      <c r="A4" s="238" t="s">
         <v>141</v>
       </c>
-      <c r="B4" s="235"/>
+      <c r="B4" s="238"/>
       <c r="C4" s="9" t="s">
         <v>199</v>
       </c>
@@ -49547,8 +49547,8 @@
       </c>
     </row>
     <row r="5" spans="1:6" ht="273" x14ac:dyDescent="0.25">
-      <c r="A5" s="236"/>
-      <c r="B5" s="237"/>
+      <c r="A5" s="239"/>
+      <c r="B5" s="240"/>
       <c r="C5" s="37" t="s">
         <v>203</v>
       </c>
@@ -49563,7 +49563,7 @@
       </c>
     </row>
     <row r="6" spans="1:6" ht="22.5" x14ac:dyDescent="0.3">
-      <c r="A6" s="239" t="s">
+      <c r="A6" s="242" t="s">
         <v>145</v>
       </c>
       <c r="B6" s="13" t="s">
@@ -49581,7 +49581,7 @@
       </c>
     </row>
     <row r="7" spans="1:6" ht="22.5" x14ac:dyDescent="0.3">
-      <c r="A7" s="239"/>
+      <c r="A7" s="242"/>
       <c r="B7" s="14" t="s">
         <v>147</v>
       </c>
@@ -49597,7 +49597,7 @@
       </c>
     </row>
     <row r="8" spans="1:6" ht="22.5" x14ac:dyDescent="0.3">
-      <c r="A8" s="239"/>
+      <c r="A8" s="242"/>
       <c r="B8" s="10" t="s">
         <v>149</v>
       </c>
@@ -49615,7 +49615,7 @@
       </c>
     </row>
     <row r="9" spans="1:6" ht="22.5" x14ac:dyDescent="0.3">
-      <c r="A9" s="239"/>
+      <c r="A9" s="242"/>
       <c r="B9" s="12" t="s">
         <v>151</v>
       </c>
@@ -49631,7 +49631,7 @@
       </c>
     </row>
     <row r="10" spans="1:6" ht="22.5" x14ac:dyDescent="0.3">
-      <c r="A10" s="239"/>
+      <c r="A10" s="242"/>
       <c r="B10" s="14" t="s">
         <v>152</v>
       </c>
@@ -50399,10 +50399,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="21" x14ac:dyDescent="0.35">
-      <c r="A1" s="235" t="s">
+      <c r="A1" s="238" t="s">
         <v>141</v>
       </c>
-      <c r="B1" s="235"/>
+      <c r="B1" s="238"/>
       <c r="C1" s="103" t="s">
         <v>210</v>
       </c>
@@ -50431,10 +50431,10 @@
       </c>
     </row>
     <row r="3" spans="1:6" s="1" customFormat="1" ht="25.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="235" t="s">
+      <c r="A3" s="238" t="s">
         <v>140</v>
       </c>
-      <c r="B3" s="235"/>
+      <c r="B3" s="238"/>
       <c r="C3" s="102" t="s">
         <v>20</v>
       </c>
@@ -50449,10 +50449,10 @@
       </c>
     </row>
     <row r="4" spans="1:6" s="1" customFormat="1" ht="74.45" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="235" t="s">
+      <c r="A4" s="238" t="s">
         <v>137</v>
       </c>
-      <c r="B4" s="235"/>
+      <c r="B4" s="238"/>
       <c r="C4" s="103" t="s">
         <v>210</v>
       </c>
@@ -50467,8 +50467,8 @@
       </c>
     </row>
     <row r="5" spans="1:6" s="1" customFormat="1" ht="409.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="236"/>
-      <c r="B5" s="237"/>
+      <c r="A5" s="239"/>
+      <c r="B5" s="240"/>
       <c r="C5" s="207" t="s">
         <v>213</v>
       </c>
@@ -50483,7 +50483,7 @@
       </c>
     </row>
     <row r="6" spans="1:6" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="239" t="s">
+      <c r="A6" s="242" t="s">
         <v>145</v>
       </c>
       <c r="B6" s="13" t="s">
@@ -50497,7 +50497,7 @@
       </c>
     </row>
     <row r="7" spans="1:6" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="239"/>
+      <c r="A7" s="242"/>
       <c r="B7" s="14" t="s">
         <v>147</v>
       </c>
@@ -50507,7 +50507,7 @@
       <c r="F7" s="130"/>
     </row>
     <row r="8" spans="1:6" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="239"/>
+      <c r="A8" s="242"/>
       <c r="B8" s="10" t="s">
         <v>149</v>
       </c>
@@ -50525,7 +50525,7 @@
       </c>
     </row>
     <row r="9" spans="1:6" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="239"/>
+      <c r="A9" s="242"/>
       <c r="B9" s="12" t="s">
         <v>151</v>
       </c>
@@ -50537,7 +50537,7 @@
       </c>
     </row>
     <row r="10" spans="1:6" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="239"/>
+      <c r="A10" s="242"/>
       <c r="B10" s="14" t="s">
         <v>152</v>
       </c>
@@ -51451,10 +51451,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:29" ht="21" x14ac:dyDescent="0.35">
-      <c r="A1" s="240" t="s">
+      <c r="A1" s="243" t="s">
         <v>137</v>
       </c>
-      <c r="B1" s="240"/>
+      <c r="B1" s="243"/>
       <c r="C1" s="65" t="s">
         <v>19</v>
       </c>
@@ -51621,10 +51621,10 @@
       </c>
     </row>
     <row r="3" spans="1:29" s="1" customFormat="1" ht="25.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="240" t="s">
+      <c r="A3" s="243" t="s">
         <v>140</v>
       </c>
-      <c r="B3" s="240"/>
+      <c r="B3" s="243"/>
       <c r="C3" s="182" t="s">
         <v>20</v>
       </c>
@@ -51708,10 +51708,10 @@
       </c>
     </row>
     <row r="4" spans="1:29" s="1" customFormat="1" ht="74.45" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="240" t="s">
+      <c r="A4" s="243" t="s">
         <v>141</v>
       </c>
-      <c r="B4" s="240"/>
+      <c r="B4" s="243"/>
       <c r="C4" s="65" t="s">
         <v>19</v>
       </c>
@@ -51795,8 +51795,8 @@
       </c>
     </row>
     <row r="5" spans="1:29" s="1" customFormat="1" ht="409.5" x14ac:dyDescent="0.25">
-      <c r="A5" s="241"/>
-      <c r="B5" s="241"/>
+      <c r="A5" s="244"/>
+      <c r="B5" s="244"/>
       <c r="C5" s="183" t="s">
         <v>413</v>
       </c>
@@ -51880,7 +51880,7 @@
       </c>
     </row>
     <row r="6" spans="1:29" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="242" t="s">
+      <c r="A6" s="245" t="s">
         <v>145</v>
       </c>
       <c r="B6" s="59" t="s">
@@ -51959,7 +51959,7 @@
       <c r="AC6" s="67"/>
     </row>
     <row r="7" spans="1:29" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="242"/>
+      <c r="A7" s="245"/>
       <c r="B7" s="60" t="s">
         <v>147</v>
       </c>
@@ -51994,7 +51994,7 @@
       <c r="AC7" s="68"/>
     </row>
     <row r="8" spans="1:29" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="242"/>
+      <c r="A8" s="245"/>
       <c r="B8" s="61" t="s">
         <v>149</v>
       </c>
@@ -52077,7 +52077,7 @@
       </c>
     </row>
     <row r="9" spans="1:29" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="242"/>
+      <c r="A9" s="245"/>
       <c r="B9" s="62" t="s">
         <v>151</v>
       </c>
@@ -52152,7 +52152,7 @@
       <c r="AC9" s="71"/>
     </row>
     <row r="10" spans="1:29" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="242"/>
+      <c r="A10" s="245"/>
       <c r="B10" s="60" t="s">
         <v>152</v>
       </c>
@@ -52294,7 +52294,7 @@
       <c r="P12" s="7"/>
       <c r="Q12" s="7"/>
       <c r="R12" s="109"/>
-      <c r="S12" s="245"/>
+      <c r="S12" s="235"/>
       <c r="T12" s="122"/>
       <c r="U12" s="7"/>
       <c r="V12" s="7"/>
@@ -55691,10 +55691,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="21" x14ac:dyDescent="0.35">
-      <c r="A1" s="240" t="s">
+      <c r="A1" s="243" t="s">
         <v>137</v>
       </c>
-      <c r="B1" s="240"/>
+      <c r="B1" s="243"/>
       <c r="C1" s="17" t="s">
         <v>138</v>
       </c>
@@ -55789,10 +55789,10 @@
       </c>
     </row>
     <row r="3" spans="1:17" s="1" customFormat="1" ht="25.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="240" t="s">
+      <c r="A3" s="243" t="s">
         <v>140</v>
       </c>
-      <c r="B3" s="240"/>
+      <c r="B3" s="243"/>
       <c r="C3" s="15" t="s">
         <v>99</v>
       </c>
@@ -55840,10 +55840,10 @@
       </c>
     </row>
     <row r="4" spans="1:17" s="1" customFormat="1" ht="97.15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="240" t="s">
+      <c r="A4" s="243" t="s">
         <v>141</v>
       </c>
-      <c r="B4" s="240"/>
+      <c r="B4" s="243"/>
       <c r="C4" s="65" t="s">
         <v>255</v>
       </c>
@@ -55891,8 +55891,8 @@
       </c>
     </row>
     <row r="5" spans="1:17" s="1" customFormat="1" ht="409.6" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="243"/>
-      <c r="B5" s="244"/>
+      <c r="A5" s="246"/>
+      <c r="B5" s="247"/>
       <c r="C5" s="219" t="s">
         <v>270</v>
       </c>
@@ -55940,7 +55940,7 @@
       </c>
     </row>
     <row r="6" spans="1:17" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="242" t="s">
+      <c r="A6" s="245" t="s">
         <v>145</v>
       </c>
       <c r="B6" s="59" t="s">
@@ -55963,7 +55963,7 @@
       <c r="Q6" s="38"/>
     </row>
     <row r="7" spans="1:17" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="242"/>
+      <c r="A7" s="245"/>
       <c r="B7" s="60" t="s">
         <v>147</v>
       </c>
@@ -55984,7 +55984,7 @@
       <c r="Q7" s="8"/>
     </row>
     <row r="8" spans="1:17" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="242"/>
+      <c r="A8" s="245"/>
       <c r="B8" s="61" t="s">
         <v>149</v>
       </c>
@@ -56029,7 +56029,7 @@
       </c>
     </row>
     <row r="9" spans="1:17" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="242"/>
+      <c r="A9" s="245"/>
       <c r="B9" s="62" t="s">
         <v>151</v>
       </c>
@@ -56054,7 +56054,7 @@
       <c r="Q9" s="39"/>
     </row>
     <row r="10" spans="1:17" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="242"/>
+      <c r="A10" s="245"/>
       <c r="B10" s="60" t="s">
         <v>152</v>
       </c>
@@ -58220,10 +58220,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="46.5" x14ac:dyDescent="0.7">
-      <c r="A1" s="240" t="s">
+      <c r="A1" s="243" t="s">
         <v>141</v>
       </c>
-      <c r="B1" s="240"/>
+      <c r="B1" s="243"/>
       <c r="C1" s="231" t="s">
         <v>64</v>
       </c>
@@ -58294,10 +58294,10 @@
       </c>
     </row>
     <row r="3" spans="1:13" s="1" customFormat="1" ht="25.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="240" t="s">
+      <c r="A3" s="243" t="s">
         <v>140</v>
       </c>
-      <c r="B3" s="240"/>
+      <c r="B3" s="243"/>
       <c r="C3" s="64" t="s">
         <v>65</v>
       </c>
@@ -58333,10 +58333,10 @@
       </c>
     </row>
     <row r="4" spans="1:13" s="1" customFormat="1" ht="74.45" customHeight="1" x14ac:dyDescent="0.7">
-      <c r="A4" s="240" t="s">
+      <c r="A4" s="243" t="s">
         <v>137</v>
       </c>
-      <c r="B4" s="240"/>
+      <c r="B4" s="243"/>
       <c r="C4" s="65" t="s">
         <v>64</v>
       </c>
@@ -58372,8 +58372,8 @@
       </c>
     </row>
     <row r="5" spans="1:13" s="1" customFormat="1" ht="409.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="243"/>
-      <c r="B5" s="243"/>
+      <c r="A5" s="246"/>
+      <c r="B5" s="246"/>
       <c r="C5" s="208" t="s">
         <v>391</v>
       </c>
@@ -58407,7 +58407,7 @@
       <c r="M5" s="56"/>
     </row>
     <row r="6" spans="1:13" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="242" t="s">
+      <c r="A6" s="245" t="s">
         <v>145</v>
       </c>
       <c r="B6" s="59" t="s">
@@ -58426,7 +58426,7 @@
       <c r="M6" s="67"/>
     </row>
     <row r="7" spans="1:13" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="242"/>
+      <c r="A7" s="245"/>
       <c r="B7" s="60" t="s">
         <v>147</v>
       </c>
@@ -58443,7 +58443,7 @@
       <c r="M7" s="68"/>
     </row>
     <row r="8" spans="1:13" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="242"/>
+      <c r="A8" s="245"/>
       <c r="B8" s="61" t="s">
         <v>149</v>
       </c>
@@ -58480,7 +58480,7 @@
       <c r="M8" s="69"/>
     </row>
     <row r="9" spans="1:13" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="242"/>
+      <c r="A9" s="245"/>
       <c r="B9" s="62" t="s">
         <v>151</v>
       </c>
@@ -58497,7 +58497,7 @@
       <c r="M9" s="71"/>
     </row>
     <row r="10" spans="1:13" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="242"/>
+      <c r="A10" s="245"/>
       <c r="B10" s="60" t="s">
         <v>152</v>
       </c>
@@ -60258,6 +60258,26 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="e658002f-fdfe-4e4b-94aa-0526ee42a8ac">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="4ad8f8a2-17e7-49a9-8390-22f3c8f42b39" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x010100C9B53A5B1F235B4EBDF9F22062DFC34D" ma:contentTypeVersion="12" ma:contentTypeDescription="Creare un nuovo documento." ma:contentTypeScope="" ma:versionID="ad5b12d537450e73edf2af95672e184c">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="e658002f-fdfe-4e4b-94aa-0526ee42a8ac" xmlns:ns3="4ad8f8a2-17e7-49a9-8390-22f3c8f42b39" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="ac16958afaf1bb0d1dccad67078e8e2c" ns2:_="" ns3:_="">
     <xsd:import namespace="e658002f-fdfe-4e4b-94aa-0526ee42a8ac"/>
@@ -60474,27 +60494,26 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="e658002f-fdfe-4e4b-94aa-0526ee42a8ac">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="4ad8f8a2-17e7-49a9-8390-22f3c8f42b39" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BA99F9FA-472B-49CB-8CD8-32BE0FD0DC5E}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7CBF6B91-9305-4674-87E0-A56D6B941238}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="e658002f-fdfe-4e4b-94aa-0526ee42a8ac"/>
+    <ds:schemaRef ds:uri="4ad8f8a2-17e7-49a9-8390-22f3c8f42b39"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{31D0029D-E8A7-4DC9-B140-19D450DFB7E0}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -60511,23 +60530,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7CBF6B91-9305-4674-87E0-A56D6B941238}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="e658002f-fdfe-4e4b-94aa-0526ee42a8ac"/>
-    <ds:schemaRef ds:uri="4ad8f8a2-17e7-49a9-8390-22f3c8f42b39"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BA99F9FA-472B-49CB-8CD8-32BE0FD0DC5E}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
bst_ocp in trimming copy works
</commit_message>
<xml_diff>
--- a/IVM6311_Testing_scripts.xlsx
+++ b/IVM6311_Testing_scripts.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\invlab\Documents\IVM6311ATE\IVM6311ATE\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA6ED2E1-C175-4E99-906C-C73E9AD1BFF3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D27A519A-7C69-4D8A-B7DB-2F86D93A0CCB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="693" firstSheet="1" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -60267,17 +60267,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="e658002f-fdfe-4e4b-94aa-0526ee42a8ac">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="4ad8f8a2-17e7-49a9-8390-22f3c8f42b39" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x010100C9B53A5B1F235B4EBDF9F22062DFC34D" ma:contentTypeVersion="12" ma:contentTypeDescription="Creare un nuovo documento." ma:contentTypeScope="" ma:versionID="ad5b12d537450e73edf2af95672e184c">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="e658002f-fdfe-4e4b-94aa-0526ee42a8ac" xmlns:ns3="4ad8f8a2-17e7-49a9-8390-22f3c8f42b39" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="ac16958afaf1bb0d1dccad67078e8e2c" ns2:_="" ns3:_="">
     <xsd:import namespace="e658002f-fdfe-4e4b-94aa-0526ee42a8ac"/>
@@ -60494,6 +60483,17 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="e658002f-fdfe-4e4b-94aa-0526ee42a8ac">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="4ad8f8a2-17e7-49a9-8390-22f3c8f42b39" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BA99F9FA-472B-49CB-8CD8-32BE0FD0DC5E}">
   <ds:schemaRefs>
@@ -60503,17 +60503,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7CBF6B91-9305-4674-87E0-A56D6B941238}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="e658002f-fdfe-4e4b-94aa-0526ee42a8ac"/>
-    <ds:schemaRef ds:uri="4ad8f8a2-17e7-49a9-8390-22f3c8f42b39"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{31D0029D-E8A7-4DC9-B140-19D450DFB7E0}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -60530,4 +60519,15 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7CBF6B91-9305-4674-87E0-A56D6B941238}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="e658002f-fdfe-4e4b-94aa-0526ee42a8ac"/>
+    <ds:schemaRef ds:uri="4ad8f8a2-17e7-49a9-8390-22f3c8f42b39"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
ocp trim working in the debug script
</commit_message>
<xml_diff>
--- a/IVM6311_Testing_scripts.xlsx
+++ b/IVM6311_Testing_scripts.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28025"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28129"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\invlab\Documents\IVM6311ATE\IVM6311ATE\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A20F906F-E020-4931-9634-B254499D276C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{076C87D1-2ACF-4D82-A513-63A4D60C46A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="693" firstSheet="1" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="693" firstSheet="1" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Revision" sheetId="3" r:id="rId1"/>
@@ -46383,7 +46383,7 @@
     <xf numFmtId="9" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="118" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="250">
+  <cellXfs count="249">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -46980,6 +46980,9 @@
     <xf numFmtId="49" fontId="4" fillId="2" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="83" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
@@ -47009,12 +47012,6 @@
     </xf>
     <xf numFmtId="3" fontId="26" fillId="7" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="83" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -48488,10 +48485,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="21" x14ac:dyDescent="0.35">
-      <c r="A1" s="238" t="s">
+      <c r="A1" s="239" t="s">
         <v>373</v>
       </c>
-      <c r="B1" s="238"/>
+      <c r="B1" s="239"/>
       <c r="C1" s="9" t="s">
         <v>142</v>
       </c>
@@ -48522,10 +48519,10 @@
       </c>
     </row>
     <row r="3" spans="1:9" ht="21" x14ac:dyDescent="0.35">
-      <c r="A3" s="238" t="s">
+      <c r="A3" s="239" t="s">
         <v>140</v>
       </c>
-      <c r="B3" s="238"/>
+      <c r="B3" s="239"/>
       <c r="C3" s="15" t="s">
         <v>60</v>
       </c>
@@ -48540,10 +48537,10 @@
       </c>
     </row>
     <row r="4" spans="1:9" ht="21" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="238" t="s">
+      <c r="A4" s="239" t="s">
         <v>137</v>
       </c>
-      <c r="B4" s="238"/>
+      <c r="B4" s="239"/>
       <c r="C4" s="9" t="s">
         <v>142</v>
       </c>
@@ -48558,8 +48555,8 @@
       </c>
     </row>
     <row r="5" spans="1:9" ht="409.5" x14ac:dyDescent="0.25">
-      <c r="A5" s="239"/>
-      <c r="B5" s="240"/>
+      <c r="A5" s="240"/>
+      <c r="B5" s="241"/>
       <c r="C5" s="204" t="s">
         <v>412</v>
       </c>
@@ -48575,7 +48572,7 @@
       <c r="I5" s="234"/>
     </row>
     <row r="6" spans="1:9" ht="22.5" x14ac:dyDescent="0.3">
-      <c r="A6" s="241" t="s">
+      <c r="A6" s="242" t="s">
         <v>145</v>
       </c>
       <c r="B6" s="13" t="s">
@@ -48591,7 +48588,7 @@
       <c r="F6" s="139"/>
     </row>
     <row r="7" spans="1:9" ht="22.5" x14ac:dyDescent="0.3">
-      <c r="A7" s="241"/>
+      <c r="A7" s="242"/>
       <c r="B7" s="14" t="s">
         <v>147</v>
       </c>
@@ -48603,7 +48600,7 @@
       <c r="F7" s="140"/>
     </row>
     <row r="8" spans="1:9" ht="22.5" x14ac:dyDescent="0.3">
-      <c r="A8" s="241"/>
+      <c r="A8" s="242"/>
       <c r="B8" s="10" t="s">
         <v>149</v>
       </c>
@@ -48621,7 +48618,7 @@
       </c>
     </row>
     <row r="9" spans="1:9" ht="22.5" x14ac:dyDescent="0.3">
-      <c r="A9" s="241"/>
+      <c r="A9" s="242"/>
       <c r="B9" s="12" t="s">
         <v>151</v>
       </c>
@@ -48633,7 +48630,7 @@
       <c r="F9" s="142"/>
     </row>
     <row r="10" spans="1:9" ht="22.5" x14ac:dyDescent="0.3">
-      <c r="A10" s="241"/>
+      <c r="A10" s="242"/>
       <c r="B10" s="14" t="s">
         <v>152</v>
       </c>
@@ -49558,10 +49555,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="21" x14ac:dyDescent="0.35">
-      <c r="A1" s="238" t="s">
+      <c r="A1" s="239" t="s">
         <v>137</v>
       </c>
-      <c r="B1" s="238"/>
+      <c r="B1" s="239"/>
       <c r="C1" s="17" t="s">
         <v>138</v>
       </c>
@@ -49592,10 +49589,10 @@
       </c>
     </row>
     <row r="3" spans="1:6" ht="21" x14ac:dyDescent="0.35">
-      <c r="A3" s="238" t="s">
+      <c r="A3" s="239" t="s">
         <v>140</v>
       </c>
-      <c r="B3" s="238"/>
+      <c r="B3" s="239"/>
       <c r="C3" s="15" t="s">
         <v>79</v>
       </c>
@@ -49610,10 +49607,10 @@
       </c>
     </row>
     <row r="4" spans="1:6" ht="21" x14ac:dyDescent="0.35">
-      <c r="A4" s="238" t="s">
+      <c r="A4" s="239" t="s">
         <v>141</v>
       </c>
-      <c r="B4" s="238"/>
+      <c r="B4" s="239"/>
       <c r="C4" s="9" t="s">
         <v>199</v>
       </c>
@@ -49628,8 +49625,8 @@
       </c>
     </row>
     <row r="5" spans="1:6" ht="273" x14ac:dyDescent="0.25">
-      <c r="A5" s="239"/>
-      <c r="B5" s="240"/>
+      <c r="A5" s="240"/>
+      <c r="B5" s="241"/>
       <c r="C5" s="37" t="s">
         <v>203</v>
       </c>
@@ -49644,7 +49641,7 @@
       </c>
     </row>
     <row r="6" spans="1:6" ht="22.5" x14ac:dyDescent="0.3">
-      <c r="A6" s="242" t="s">
+      <c r="A6" s="243" t="s">
         <v>145</v>
       </c>
       <c r="B6" s="13" t="s">
@@ -49662,7 +49659,7 @@
       </c>
     </row>
     <row r="7" spans="1:6" ht="22.5" x14ac:dyDescent="0.3">
-      <c r="A7" s="242"/>
+      <c r="A7" s="243"/>
       <c r="B7" s="14" t="s">
         <v>147</v>
       </c>
@@ -49678,7 +49675,7 @@
       </c>
     </row>
     <row r="8" spans="1:6" ht="22.5" x14ac:dyDescent="0.3">
-      <c r="A8" s="242"/>
+      <c r="A8" s="243"/>
       <c r="B8" s="10" t="s">
         <v>149</v>
       </c>
@@ -49696,7 +49693,7 @@
       </c>
     </row>
     <row r="9" spans="1:6" ht="22.5" x14ac:dyDescent="0.3">
-      <c r="A9" s="242"/>
+      <c r="A9" s="243"/>
       <c r="B9" s="12" t="s">
         <v>151</v>
       </c>
@@ -49712,7 +49709,7 @@
       </c>
     </row>
     <row r="10" spans="1:6" ht="22.5" x14ac:dyDescent="0.3">
-      <c r="A10" s="242"/>
+      <c r="A10" s="243"/>
       <c r="B10" s="14" t="s">
         <v>152</v>
       </c>
@@ -50480,10 +50477,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="21" x14ac:dyDescent="0.35">
-      <c r="A1" s="238" t="s">
+      <c r="A1" s="239" t="s">
         <v>141</v>
       </c>
-      <c r="B1" s="238"/>
+      <c r="B1" s="239"/>
       <c r="C1" s="103" t="s">
         <v>210</v>
       </c>
@@ -50512,10 +50509,10 @@
       </c>
     </row>
     <row r="3" spans="1:6" s="1" customFormat="1" ht="25.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="238" t="s">
+      <c r="A3" s="239" t="s">
         <v>140</v>
       </c>
-      <c r="B3" s="238"/>
+      <c r="B3" s="239"/>
       <c r="C3" s="102" t="s">
         <v>20</v>
       </c>
@@ -50530,10 +50527,10 @@
       </c>
     </row>
     <row r="4" spans="1:6" s="1" customFormat="1" ht="74.45" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="238" t="s">
+      <c r="A4" s="239" t="s">
         <v>137</v>
       </c>
-      <c r="B4" s="238"/>
+      <c r="B4" s="239"/>
       <c r="C4" s="103" t="s">
         <v>210</v>
       </c>
@@ -50548,8 +50545,8 @@
       </c>
     </row>
     <row r="5" spans="1:6" s="1" customFormat="1" ht="409.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="239"/>
-      <c r="B5" s="240"/>
+      <c r="A5" s="240"/>
+      <c r="B5" s="241"/>
       <c r="C5" s="207" t="s">
         <v>213</v>
       </c>
@@ -50564,7 +50561,7 @@
       </c>
     </row>
     <row r="6" spans="1:6" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="242" t="s">
+      <c r="A6" s="243" t="s">
         <v>145</v>
       </c>
       <c r="B6" s="13" t="s">
@@ -50578,7 +50575,7 @@
       </c>
     </row>
     <row r="7" spans="1:6" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="242"/>
+      <c r="A7" s="243"/>
       <c r="B7" s="14" t="s">
         <v>147</v>
       </c>
@@ -50588,7 +50585,7 @@
       <c r="F7" s="130"/>
     </row>
     <row r="8" spans="1:6" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="242"/>
+      <c r="A8" s="243"/>
       <c r="B8" s="10" t="s">
         <v>149</v>
       </c>
@@ -50606,7 +50603,7 @@
       </c>
     </row>
     <row r="9" spans="1:6" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="242"/>
+      <c r="A9" s="243"/>
       <c r="B9" s="12" t="s">
         <v>151</v>
       </c>
@@ -50618,7 +50615,7 @@
       </c>
     </row>
     <row r="10" spans="1:6" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="242"/>
+      <c r="A10" s="243"/>
       <c r="B10" s="14" t="s">
         <v>152</v>
       </c>
@@ -51532,10 +51529,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:29" ht="21" x14ac:dyDescent="0.35">
-      <c r="A1" s="243" t="s">
+      <c r="A1" s="244" t="s">
         <v>137</v>
       </c>
-      <c r="B1" s="243"/>
+      <c r="B1" s="244"/>
       <c r="C1" s="65" t="s">
         <v>19</v>
       </c>
@@ -51702,10 +51699,10 @@
       </c>
     </row>
     <row r="3" spans="1:29" s="1" customFormat="1" ht="25.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="243" t="s">
+      <c r="A3" s="244" t="s">
         <v>140</v>
       </c>
-      <c r="B3" s="243"/>
+      <c r="B3" s="244"/>
       <c r="C3" s="182" t="s">
         <v>20</v>
       </c>
@@ -51789,10 +51786,10 @@
       </c>
     </row>
     <row r="4" spans="1:29" s="1" customFormat="1" ht="74.45" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="243" t="s">
+      <c r="A4" s="244" t="s">
         <v>141</v>
       </c>
-      <c r="B4" s="243"/>
+      <c r="B4" s="244"/>
       <c r="C4" s="65" t="s">
         <v>19</v>
       </c>
@@ -51876,8 +51873,8 @@
       </c>
     </row>
     <row r="5" spans="1:29" s="1" customFormat="1" ht="409.5" x14ac:dyDescent="0.25">
-      <c r="A5" s="244"/>
-      <c r="B5" s="244"/>
+      <c r="A5" s="245"/>
+      <c r="B5" s="245"/>
       <c r="C5" s="183" t="s">
         <v>435</v>
       </c>
@@ -51887,7 +51884,7 @@
       <c r="E5" s="183" t="s">
         <v>437</v>
       </c>
-      <c r="F5" s="249" t="s">
+      <c r="F5" s="183" t="s">
         <v>423</v>
       </c>
       <c r="G5" s="183" t="s">
@@ -51923,7 +51920,7 @@
       <c r="Q5" s="221" t="s">
         <v>232</v>
       </c>
-      <c r="R5" s="249" t="s">
+      <c r="R5" s="183" t="s">
         <v>433</v>
       </c>
       <c r="S5" s="189" t="s">
@@ -51961,7 +51958,7 @@
       </c>
     </row>
     <row r="6" spans="1:29" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="245" t="s">
+      <c r="A6" s="246" t="s">
         <v>145</v>
       </c>
       <c r="B6" s="59" t="s">
@@ -52040,7 +52037,7 @@
       <c r="AC6" s="67"/>
     </row>
     <row r="7" spans="1:29" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="245"/>
+      <c r="A7" s="246"/>
       <c r="B7" s="60" t="s">
         <v>147</v>
       </c>
@@ -52075,7 +52072,7 @@
       <c r="AC7" s="68"/>
     </row>
     <row r="8" spans="1:29" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="245"/>
+      <c r="A8" s="246"/>
       <c r="B8" s="61" t="s">
         <v>149</v>
       </c>
@@ -52158,7 +52155,7 @@
       </c>
     </row>
     <row r="9" spans="1:29" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="245"/>
+      <c r="A9" s="246"/>
       <c r="B9" s="62" t="s">
         <v>151</v>
       </c>
@@ -52233,7 +52230,7 @@
       <c r="AC9" s="71"/>
     </row>
     <row r="10" spans="1:29" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="245"/>
+      <c r="A10" s="246"/>
       <c r="B10" s="60" t="s">
         <v>152</v>
       </c>
@@ -55772,10 +55769,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="21" x14ac:dyDescent="0.35">
-      <c r="A1" s="243" t="s">
+      <c r="A1" s="244" t="s">
         <v>137</v>
       </c>
-      <c r="B1" s="243"/>
+      <c r="B1" s="244"/>
       <c r="C1" s="17" t="s">
         <v>138</v>
       </c>
@@ -55870,10 +55867,10 @@
       </c>
     </row>
     <row r="3" spans="1:17" s="1" customFormat="1" ht="25.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="243" t="s">
+      <c r="A3" s="244" t="s">
         <v>140</v>
       </c>
-      <c r="B3" s="243"/>
+      <c r="B3" s="244"/>
       <c r="C3" s="15" t="s">
         <v>99</v>
       </c>
@@ -55921,10 +55918,10 @@
       </c>
     </row>
     <row r="4" spans="1:17" s="1" customFormat="1" ht="97.15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="243" t="s">
+      <c r="A4" s="244" t="s">
         <v>141</v>
       </c>
-      <c r="B4" s="243"/>
+      <c r="B4" s="244"/>
       <c r="C4" s="65" t="s">
         <v>254</v>
       </c>
@@ -55972,8 +55969,8 @@
       </c>
     </row>
     <row r="5" spans="1:17" s="1" customFormat="1" ht="409.6" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="246"/>
-      <c r="B5" s="247"/>
+      <c r="A5" s="247"/>
+      <c r="B5" s="248"/>
       <c r="C5" s="219" t="s">
         <v>269</v>
       </c>
@@ -56021,7 +56018,7 @@
       </c>
     </row>
     <row r="6" spans="1:17" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="245" t="s">
+      <c r="A6" s="246" t="s">
         <v>145</v>
       </c>
       <c r="B6" s="59" t="s">
@@ -56044,7 +56041,7 @@
       <c r="Q6" s="38"/>
     </row>
     <row r="7" spans="1:17" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="245"/>
+      <c r="A7" s="246"/>
       <c r="B7" s="60" t="s">
         <v>147</v>
       </c>
@@ -56065,7 +56062,7 @@
       <c r="Q7" s="8"/>
     </row>
     <row r="8" spans="1:17" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="245"/>
+      <c r="A8" s="246"/>
       <c r="B8" s="61" t="s">
         <v>149</v>
       </c>
@@ -56110,7 +56107,7 @@
       </c>
     </row>
     <row r="9" spans="1:17" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="245"/>
+      <c r="A9" s="246"/>
       <c r="B9" s="62" t="s">
         <v>151</v>
       </c>
@@ -56135,7 +56132,7 @@
       <c r="Q9" s="39"/>
     </row>
     <row r="10" spans="1:17" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="245"/>
+      <c r="A10" s="246"/>
       <c r="B10" s="60" t="s">
         <v>152</v>
       </c>
@@ -58301,10 +58298,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="46.5" x14ac:dyDescent="0.7">
-      <c r="A1" s="243" t="s">
+      <c r="A1" s="244" t="s">
         <v>141</v>
       </c>
-      <c r="B1" s="243"/>
+      <c r="B1" s="244"/>
       <c r="C1" s="231" t="s">
         <v>64</v>
       </c>
@@ -58375,10 +58372,10 @@
       </c>
     </row>
     <row r="3" spans="1:13" s="1" customFormat="1" ht="25.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="243" t="s">
+      <c r="A3" s="244" t="s">
         <v>140</v>
       </c>
-      <c r="B3" s="243"/>
+      <c r="B3" s="244"/>
       <c r="C3" s="64" t="s">
         <v>65</v>
       </c>
@@ -58414,10 +58411,10 @@
       </c>
     </row>
     <row r="4" spans="1:13" s="1" customFormat="1" ht="74.45" customHeight="1" x14ac:dyDescent="0.7">
-      <c r="A4" s="243" t="s">
+      <c r="A4" s="244" t="s">
         <v>137</v>
       </c>
-      <c r="B4" s="243"/>
+      <c r="B4" s="244"/>
       <c r="C4" s="65" t="s">
         <v>64</v>
       </c>
@@ -58453,8 +58450,8 @@
       </c>
     </row>
     <row r="5" spans="1:13" s="1" customFormat="1" ht="409.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="246"/>
-      <c r="B5" s="246"/>
+      <c r="A5" s="247"/>
+      <c r="B5" s="247"/>
       <c r="C5" s="208" t="s">
         <v>389</v>
       </c>
@@ -58488,7 +58485,7 @@
       <c r="M5" s="56"/>
     </row>
     <row r="6" spans="1:13" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="245" t="s">
+      <c r="A6" s="246" t="s">
         <v>145</v>
       </c>
       <c r="B6" s="59" t="s">
@@ -58507,7 +58504,7 @@
       <c r="M6" s="67"/>
     </row>
     <row r="7" spans="1:13" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="245"/>
+      <c r="A7" s="246"/>
       <c r="B7" s="60" t="s">
         <v>147</v>
       </c>
@@ -58524,7 +58521,7 @@
       <c r="M7" s="68"/>
     </row>
     <row r="8" spans="1:13" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="245"/>
+      <c r="A8" s="246"/>
       <c r="B8" s="61" t="s">
         <v>149</v>
       </c>
@@ -58561,7 +58558,7 @@
       <c r="M8" s="69"/>
     </row>
     <row r="9" spans="1:13" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="245"/>
+      <c r="A9" s="246"/>
       <c r="B9" s="62" t="s">
         <v>151</v>
       </c>
@@ -58578,7 +58575,7 @@
       <c r="M9" s="71"/>
     </row>
     <row r="10" spans="1:13" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="245"/>
+      <c r="A10" s="246"/>
       <c r="B10" s="60" t="s">
         <v>152</v>
       </c>
@@ -60303,10 +60300,10 @@
       <c r="B2" s="174" t="s">
         <v>425</v>
       </c>
-      <c r="C2" s="248" t="s">
+      <c r="C2" s="238" t="s">
         <v>431</v>
       </c>
-      <c r="D2" s="248" t="s">
+      <c r="D2" s="238" t="s">
         <v>432</v>
       </c>
       <c r="E2" s="83" t="s">
@@ -60347,14 +60344,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="e658002f-fdfe-4e4b-94aa-0526ee42a8ac">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="4ad8f8a2-17e7-49a9-8390-22f3c8f42b39" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -60575,21 +60570,20 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="e658002f-fdfe-4e4b-94aa-0526ee42a8ac">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="4ad8f8a2-17e7-49a9-8390-22f3c8f42b39" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7CBF6B91-9305-4674-87E0-A56D6B941238}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BA99F9FA-472B-49CB-8CD8-32BE0FD0DC5E}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="e658002f-fdfe-4e4b-94aa-0526ee42a8ac"/>
-    <ds:schemaRef ds:uri="4ad8f8a2-17e7-49a9-8390-22f3c8f42b39"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -60614,9 +60608,12 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BA99F9FA-472B-49CB-8CD8-32BE0FD0DC5E}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7CBF6B91-9305-4674-87E0-A56D6B941238}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="e658002f-fdfe-4e4b-94aa-0526ee42a8ac"/>
+    <ds:schemaRef ds:uri="4ad8f8a2-17e7-49a9-8390-22f3c8f42b39"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
removed the forcing SW 3.6 from test boost default
</commit_message>
<xml_diff>
--- a/IVM6311_Testing_scripts.xlsx
+++ b/IVM6311_Testing_scripts.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\invlab\Documents\IVM6311ATE\IVM6311ATE\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{076C87D1-2ACF-4D82-A513-63A4D60C46A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{337E9289-B19C-4A55-BAEA-A38612B3300C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="693" firstSheet="1" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36393,240 +36393,6 @@
     </r>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FFFF33CC"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">Force__VBIAS__5V
-Force__VBSO__3.6V
-Force__SW__3.6V
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0070C0"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>0xFE_0x00</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> "Select page 0"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0070C0"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>0xB0_0x00</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> "en 1 bst low"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0070C0"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>0xB1_0x00</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> "en 2 bst low"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0070C0"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>0xB3[4:3]_0x00</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> "en 3 bst low"
-0xFE_0x01 "Select page 1"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0070C0"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>0x18[6]_0x01</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> "Enable Mirr"
-0xFE_0x00 "Select page 0"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0070C0"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>0xB1[6]_0x01</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> "Bootstrap en"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0070C0"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>0xB2[1]_0x00</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> "ls_sel off"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0070C0"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>0xB4[2:0]_0x00</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> "hsa_hsb_byp off"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0070C0"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>0xFE_0x01</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> "Select page 1"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0070C0"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>0x17[6]_0x01</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> "Force Mirr"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0070C0"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>0x16[6]_0x01</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> "Force Bootstrap"</t>
-    </r>
-  </si>
-  <si>
     <t xml:space="preserve">Run__Startup
 Run__Enable_Ana_Testpoint
 0xFE_0x01 "Select page 1"
@@ -42096,485 +41862,6 @@
     <t>kHz</t>
   </si>
   <si>
-    <r>
-      <t xml:space="preserve">Run__startup
-Run__Boost_test_default
-Run__Enable_Ana_Testpoint
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF7030A0"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">Wait__delay__0.1ms
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FFFF3399"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF4472C4"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>0xFE_0x00</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> "Select page 0"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF4472C4"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>0xB0[1]_0x01</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> "ocp en
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF4472C4"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>0xB2[1]_0x01</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> "ls_sel on"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF4472C4"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>0xC0[2:0]_0x03</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> "OCP threshold set to 400mA"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF4472C4"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">0xFE_0x01 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">"Select page 1"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF4472C4"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>0x1A_0x10</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> "TSW to OCP Sense"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0070C0"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">0x03_0x07 </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">"FSYN testpoint enable"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0070C0"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">0x04_0x18 </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">"FSYN = ana_bst_ocp_1"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FFFF3399"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF7030A0"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">Wait__delay__0.1ms
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF4472C4"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-0xFE_0x00</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> "Select page 0"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF4472C4"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>0xB2[0]_0x01</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> "Power Force en"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF4472C4"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>0xFE_0x01</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> "Select page 1"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0070C0"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">0x0F_0x80
-0xB0_0x0E
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF7030A0"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">Wait__delay__0.1ms
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF4472C4"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>0x15[2]_0x01</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> "Force ocp"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF4472C4"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>0x19[1]_0x01</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> "bst_test en"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF7030A0"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-Wait__delay__0.1ms</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF00B050"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-Force__SW__400mA
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF9BC2E6"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-TrimSweep__</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FFC65911"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>0xB2[5]__0xB1[3:0]</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF9BC2E6"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>"</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FFED7D31"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>trim in 2 different registers - Sweep codes starting from b0000,1111 to b0000,0000 than from b0001,1111 to b0001,0000</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FFFF3399"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF00B050"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Measure_Voltage_FSYN</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> "Check the transition Low to High"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FFFF3399"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF4472C4"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">0x1A_0x00
-0x19_0x00
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FFC65911"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-  </si>
-  <si>
     <t>Enable_Ana_Testpoint_boost</t>
   </si>
   <si>
@@ -45169,6 +44456,700 @@
       <t xml:space="preserve">
 0x1A_0x00
 0x19_0x00</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF33CC"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Force__VBIAS__5V
+Force__VBSO__3.6V
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0070C0"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>0xFE_0x00</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> "Select page 0"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0070C0"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>0xB0_0x00</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> "en 1 bst low"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0070C0"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>0xB1_0x00</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> "en 2 bst low"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0070C0"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>0xB3[4:3]_0x00</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> "en 3 bst low"
+0xFE_0x01 "Select page 1"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0070C0"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>0x18[6]_0x01</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> "Enable Mirr"
+0xFE_0x00 "Select page 0"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0070C0"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>0xB1[6]_0x01</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> "Bootstrap en"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0070C0"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>0xB2[1]_0x00</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> "ls_sel off"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0070C0"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>0xB4[2:0]_0x00</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> "hsa_hsb_byp off"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0070C0"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>0xFE_0x01</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> "Select page 1"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0070C0"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>0x17[6]_0x01</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> "Force Mirr"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0070C0"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>0x16[6]_0x01</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> "Force Bootstrap"</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Run__startup
+Run__Boost_test_default
+Run__Enable_Ana_Testpoint
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF7030A0"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Wait__delay__0.1ms</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF3399"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF4472C4"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>0xFE_0x00</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> "Select page 0"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF4472C4"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>0xB0[1]_0x01</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> "ocp en
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF4472C4"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>0xB2[1]_0x01</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> "ls_sel on"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF4472C4"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>0xC0[2:0]_0x03</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> "OCP threshold set to 400mA"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF4472C4"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">0xFE_0x01 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">"Select page 1"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF4472C4"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>0x1A_0x10</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> "TSW to OCP Sense"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0070C0"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">0x03_0x07 </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">"FSYN testpoint enable"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0070C0"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">0x04_0x18 </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>"FSYN = ana_bst_ocp_1"</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF3399"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF7030A0"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Wait__delay__0.1ms</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF4472C4"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+0xFE_0x00</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> "Select page 0"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF4472C4"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>0xB2[0]_0x01</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> "Power Force en"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF4472C4"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>0xFE_0x01</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> "Select page 1"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0070C0"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>0x0F_0x80
+0xB0_0x0E</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF7030A0"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Wait__delay__0.1ms
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF4472C4"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>0x15[2]_0x01</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> "Force ocp"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF4472C4"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>0x19[1]_0x01</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> "bst_test en"</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF7030A0"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Wait__delay__0.1ms</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF00B050"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Force__SW__400mA</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF9BC2E6"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+TrimSweep__</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFC65911"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>0xB2[5]__0xB1[3:0]</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF9BC2E6"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>"</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFED7D31"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>trim in 2 different registers - Sweep codes starting from b0000,1111 to b0000,0000 than from b0001,1111 to b0001,0000</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>"</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF3399"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF00B050"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Measure_Voltage_FSYN</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> "Check the transition Low to High"</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF3399"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF4472C4"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">0x1A_0x00
+0x19_0x00
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFC65911"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
     </r>
   </si>
 </sst>
@@ -48558,16 +48539,16 @@
       <c r="A5" s="240"/>
       <c r="B5" s="241"/>
       <c r="C5" s="204" t="s">
+        <v>411</v>
+      </c>
+      <c r="D5" s="204" t="s">
         <v>412</v>
-      </c>
-      <c r="D5" s="204" t="s">
-        <v>413</v>
       </c>
       <c r="E5" s="204" t="s">
         <v>400</v>
       </c>
       <c r="F5" s="188" t="s">
-        <v>429</v>
+        <v>437</v>
       </c>
       <c r="I5" s="234"/>
     </row>
@@ -48614,7 +48595,7 @@
         <v>401</v>
       </c>
       <c r="F8" s="236" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
     </row>
     <row r="9" spans="1:9" ht="22.5" x14ac:dyDescent="0.3">
@@ -48655,7 +48636,7 @@
         <v>155</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="F11" s="237" t="s">
         <v>155</v>
@@ -51876,31 +51857,31 @@
       <c r="A5" s="245"/>
       <c r="B5" s="245"/>
       <c r="C5" s="183" t="s">
+        <v>433</v>
+      </c>
+      <c r="D5" s="183" t="s">
+        <v>434</v>
+      </c>
+      <c r="E5" s="183" t="s">
         <v>435</v>
       </c>
-      <c r="D5" s="183" t="s">
-        <v>436</v>
-      </c>
-      <c r="E5" s="183" t="s">
-        <v>437</v>
-      </c>
       <c r="F5" s="183" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="G5" s="183" t="s">
         <v>406</v>
       </c>
       <c r="H5" s="189" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="I5" s="189" t="s">
         <v>407</v>
       </c>
       <c r="J5" s="189" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="K5" s="189" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="L5" s="221" t="s">
         <v>408</v>
@@ -51909,7 +51890,7 @@
         <v>409</v>
       </c>
       <c r="N5" s="183" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="O5" s="221" t="s">
         <v>230</v>
@@ -51921,22 +51902,22 @@
         <v>232</v>
       </c>
       <c r="R5" s="183" t="s">
-        <v>433</v>
+        <v>431</v>
       </c>
       <c r="S5" s="189" t="s">
-        <v>434</v>
+        <v>432</v>
       </c>
       <c r="T5" s="189" t="s">
+        <v>420</v>
+      </c>
+      <c r="U5" s="189" t="s">
         <v>421</v>
-      </c>
-      <c r="U5" s="189" t="s">
-        <v>422</v>
       </c>
       <c r="V5" s="189" t="s">
         <v>233</v>
       </c>
       <c r="W5" s="190" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
       <c r="X5" s="190" t="s">
         <v>234</v>
@@ -51945,10 +51926,10 @@
         <v>235</v>
       </c>
       <c r="Z5" s="190" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="AA5" s="189" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="AB5" s="189" t="s">
         <v>410</v>
@@ -52089,16 +52070,16 @@
         <v>44</v>
       </c>
       <c r="G8" s="69" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="H8" s="69" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="I8" s="69" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="J8" s="69" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="K8" s="69" t="s">
         <v>239</v>
@@ -52119,36 +52100,36 @@
         <v>238</v>
       </c>
       <c r="Q8" s="69" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
       <c r="R8" s="153" t="s">
         <v>237</v>
       </c>
       <c r="S8" s="141" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="T8" s="119" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="U8" s="69" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="V8" s="69" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="W8" s="233" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="X8" s="69"/>
       <c r="Y8" s="69"/>
       <c r="Z8" s="69" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="AA8" s="233" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="AB8" s="233" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="AC8" s="11" t="s">
         <v>240</v>
@@ -60257,7 +60238,7 @@
         <v>15</v>
       </c>
       <c r="C1" s="57" t="s">
-        <v>430</v>
+        <v>428</v>
       </c>
       <c r="D1" s="57" t="s">
         <v>382</v>
@@ -60295,22 +60276,22 @@
     </row>
     <row r="2" spans="1:14" s="91" customFormat="1" ht="408.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="83" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="B2" s="174" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="C2" s="238" t="s">
-        <v>431</v>
+        <v>429</v>
       </c>
       <c r="D2" s="238" t="s">
-        <v>432</v>
+        <v>430</v>
       </c>
       <c r="E2" s="83" t="s">
         <v>323</v>
       </c>
       <c r="F2" s="224" t="s">
-        <v>411</v>
+        <v>436</v>
       </c>
       <c r="G2" s="83" t="s">
         <v>324</v>
@@ -60344,12 +60325,14 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="e658002f-fdfe-4e4b-94aa-0526ee42a8ac">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="4ad8f8a2-17e7-49a9-8390-22f3c8f42b39" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -60570,20 +60553,21 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="e658002f-fdfe-4e4b-94aa-0526ee42a8ac">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="4ad8f8a2-17e7-49a9-8390-22f3c8f42b39" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BA99F9FA-472B-49CB-8CD8-32BE0FD0DC5E}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7CBF6B91-9305-4674-87E0-A56D6B941238}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="e658002f-fdfe-4e4b-94aa-0526ee42a8ac"/>
+    <ds:schemaRef ds:uri="4ad8f8a2-17e7-49a9-8390-22f3c8f42b39"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -60608,12 +60592,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7CBF6B91-9305-4674-87E0-A56D6B941238}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BA99F9FA-472B-49CB-8CD8-32BE0FD0DC5E}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="e658002f-fdfe-4e4b-94aa-0526ee42a8ac"/>
-    <ds:schemaRef ds:uri="4ad8f8a2-17e7-49a9-8390-22f3c8f42b39"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
working on the ocp, in order to merge trimming debug and reference class script
</commit_message>
<xml_diff>
--- a/IVM6311_Testing_scripts.xlsx
+++ b/IVM6311_Testing_scripts.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\invlab\Documents\IVM6311ATE\IVM6311ATE\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{337E9289-B19C-4A55-BAEA-A38612B3300C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA16C42E-BE95-4F01-9910-83BE7826F2DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="693" firstSheet="1" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="14400" yWindow="0" windowWidth="14400" windowHeight="15600" tabRatio="693" firstSheet="1" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Revision" sheetId="3" r:id="rId1"/>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1500" uniqueCount="438">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1498" uniqueCount="436">
   <si>
     <t>Revision</t>
   </si>
@@ -41862,76 +41862,6 @@
     <t>kHz</t>
   </si>
   <si>
-    <t>Enable_Ana_Testpoint_boost</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF00B0F0"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>0xFE_0x01</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> "Select page 1"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF00B0F0"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">0x0F_0x08
-0x10_0x08
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FFFF3399"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">FORCE__SDWN__OPEN
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF00B0F0"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>0x19_0x80</t>
-    </r>
-  </si>
-  <si>
     <r>
       <rPr>
         <sz val="11"/>
@@ -44781,7 +44711,7 @@
         <rFont val="Calibri"/>
         <scheme val="minor"/>
       </rPr>
-      <t>0xC0[2:0]_0x03</t>
+      <t>0xC0[2:0]_0x01</t>
     </r>
     <r>
       <rPr>
@@ -45035,7 +44965,7 @@
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve">
-Force__SW__400mA</t>
+Force__SW__200mA</t>
     </r>
     <r>
       <rPr>
@@ -48548,7 +48478,7 @@
         <v>400</v>
       </c>
       <c r="F5" s="188" t="s">
-        <v>437</v>
+        <v>435</v>
       </c>
       <c r="I5" s="234"/>
     </row>
@@ -51857,13 +51787,13 @@
       <c r="A5" s="245"/>
       <c r="B5" s="245"/>
       <c r="C5" s="183" t="s">
+        <v>431</v>
+      </c>
+      <c r="D5" s="183" t="s">
+        <v>432</v>
+      </c>
+      <c r="E5" s="183" t="s">
         <v>433</v>
-      </c>
-      <c r="D5" s="183" t="s">
-        <v>434</v>
-      </c>
-      <c r="E5" s="183" t="s">
-        <v>435</v>
       </c>
       <c r="F5" s="183" t="s">
         <v>422</v>
@@ -51902,10 +51832,10 @@
         <v>232</v>
       </c>
       <c r="R5" s="183" t="s">
-        <v>431</v>
+        <v>429</v>
       </c>
       <c r="S5" s="189" t="s">
-        <v>432</v>
+        <v>430</v>
       </c>
       <c r="T5" s="189" t="s">
         <v>420</v>
@@ -60215,22 +60145,22 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{853352DE-922C-4F00-B110-569410679C0C}">
-  <dimension ref="A1:N2"/>
+  <dimension ref="A1:M2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="37.28515625" customWidth="1"/>
-    <col min="2" max="3" width="37.5703125" customWidth="1"/>
-    <col min="4" max="4" width="37.28515625" customWidth="1"/>
-    <col min="5" max="5" width="25.42578125" customWidth="1"/>
-    <col min="6" max="6" width="31.85546875" customWidth="1"/>
-    <col min="7" max="7" width="39.85546875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="50.28515625" customWidth="1"/>
-    <col min="9" max="12" width="42.7109375" customWidth="1"/>
-    <col min="13" max="13" width="42.85546875" customWidth="1"/>
-    <col min="14" max="14" width="29.7109375" customWidth="1"/>
+    <col min="2" max="2" width="37.5703125" customWidth="1"/>
+    <col min="3" max="3" width="37.28515625" customWidth="1"/>
+    <col min="4" max="4" width="25.42578125" customWidth="1"/>
+    <col min="5" max="5" width="31.85546875" customWidth="1"/>
+    <col min="6" max="6" width="39.85546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="50.28515625" customWidth="1"/>
+    <col min="8" max="11" width="42.7109375" customWidth="1"/>
+    <col min="12" max="12" width="42.85546875" customWidth="1"/>
+    <col min="13" max="13" width="29.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1" s="57" t="s">
         <v>312</v>
       </c>
@@ -60238,43 +60168,40 @@
         <v>15</v>
       </c>
       <c r="C1" s="57" t="s">
-        <v>428</v>
+        <v>382</v>
       </c>
       <c r="D1" s="57" t="s">
-        <v>382</v>
+        <v>313</v>
       </c>
       <c r="E1" s="57" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="F1" s="57" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="G1" s="57" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="H1" s="57" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="I1" s="57" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="J1" s="57" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="K1" s="57" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="L1" s="57" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="M1" s="57" t="s">
-        <v>321</v>
-      </c>
-      <c r="N1" s="57" t="s">
         <v>322</v>
       </c>
     </row>
-    <row r="2" spans="1:14" s="91" customFormat="1" ht="408.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:13" s="91" customFormat="1" ht="408.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="83" t="s">
         <v>415</v>
       </c>
@@ -60282,39 +60209,36 @@
         <v>424</v>
       </c>
       <c r="C2" s="238" t="s">
-        <v>429</v>
-      </c>
-      <c r="D2" s="238" t="s">
-        <v>430</v>
-      </c>
-      <c r="E2" s="83" t="s">
+        <v>428</v>
+      </c>
+      <c r="D2" s="83" t="s">
         <v>323</v>
       </c>
-      <c r="F2" s="224" t="s">
-        <v>436</v>
+      <c r="E2" s="224" t="s">
+        <v>434</v>
+      </c>
+      <c r="F2" s="83" t="s">
+        <v>324</v>
       </c>
       <c r="G2" s="83" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="H2" s="83" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="I2" s="83" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="J2" s="83" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="K2" s="83" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="L2" s="83" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="M2" s="83" t="s">
-        <v>330</v>
-      </c>
-      <c r="N2" s="83" t="s">
         <v>331</v>
       </c>
     </row>
@@ -60325,14 +60249,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="e658002f-fdfe-4e4b-94aa-0526ee42a8ac">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="4ad8f8a2-17e7-49a9-8390-22f3c8f42b39" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -60553,21 +60475,20 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="e658002f-fdfe-4e4b-94aa-0526ee42a8ac">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="4ad8f8a2-17e7-49a9-8390-22f3c8f42b39" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7CBF6B91-9305-4674-87E0-A56D6B941238}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BA99F9FA-472B-49CB-8CD8-32BE0FD0DC5E}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="e658002f-fdfe-4e4b-94aa-0526ee42a8ac"/>
-    <ds:schemaRef ds:uri="4ad8f8a2-17e7-49a9-8390-22f3c8f42b39"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -60592,9 +60513,12 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BA99F9FA-472B-49CB-8CD8-32BE0FD0DC5E}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7CBF6B91-9305-4674-87E0-A56D6B941238}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="e658002f-fdfe-4e4b-94aa-0526ee42a8ac"/>
+    <ds:schemaRef ds:uri="4ad8f8a2-17e7-49a9-8390-22f3c8f42b39"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
added function trim_sweep in dft parser, to extract single and double trim sweep register
</commit_message>
<xml_diff>
--- a/IVM6311_Testing_scripts.xlsx
+++ b/IVM6311_Testing_scripts.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\invlab\Documents\IVM6311ATE\IVM6311ATE\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA16C42E-BE95-4F01-9910-83BE7826F2DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82B2A78B-3CC3-4AEF-A525-340983F0FB01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14400" yWindow="0" windowWidth="14400" windowHeight="15600" tabRatio="693" firstSheet="1" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="693" firstSheet="1" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Revision" sheetId="3" r:id="rId1"/>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1498" uniqueCount="436">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1499" uniqueCount="437">
   <si>
     <t>Revision</t>
   </si>
@@ -45081,6 +45081,9 @@
       <t xml:space="preserve">
 </t>
     </r>
+  </si>
+  <si>
+    <t>ADDED POST TRIMMING FOR BST_OCP_TRIM</t>
   </si>
 </sst>
 </file>
@@ -46294,7 +46297,7 @@
     <xf numFmtId="9" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="118" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="249">
+  <cellXfs count="250">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -46924,6 +46927,9 @@
     <xf numFmtId="3" fontId="26" fillId="7" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="49" fontId="26" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Normale" xfId="0" builtinId="0"/>
@@ -48393,6 +48399,7 @@
     <col min="3" max="4" width="73.42578125" customWidth="1"/>
     <col min="5" max="5" width="62.7109375" customWidth="1"/>
     <col min="6" max="6" width="59.28515625" style="101" customWidth="1"/>
+    <col min="7" max="7" width="64.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="21" x14ac:dyDescent="0.35">
@@ -48412,6 +48419,7 @@
       <c r="F1" s="138" t="s">
         <v>102</v>
       </c>
+      <c r="G1" s="249"/>
     </row>
     <row r="2" spans="1:9" ht="21" x14ac:dyDescent="0.35">
       <c r="A2" s="2"/>
@@ -48477,8 +48485,11 @@
       <c r="E5" s="204" t="s">
         <v>400</v>
       </c>
-      <c r="F5" s="188" t="s">
+      <c r="F5" s="189" t="s">
         <v>435</v>
+      </c>
+      <c r="G5" t="s">
+        <v>436</v>
       </c>
       <c r="I5" s="234"/>
     </row>
@@ -60249,12 +60260,14 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="e658002f-fdfe-4e4b-94aa-0526ee42a8ac">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="4ad8f8a2-17e7-49a9-8390-22f3c8f42b39" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -60475,20 +60488,21 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="e658002f-fdfe-4e4b-94aa-0526ee42a8ac">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="4ad8f8a2-17e7-49a9-8390-22f3c8f42b39" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BA99F9FA-472B-49CB-8CD8-32BE0FD0DC5E}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7CBF6B91-9305-4674-87E0-A56D6B941238}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="e658002f-fdfe-4e4b-94aa-0526ee42a8ac"/>
+    <ds:schemaRef ds:uri="4ad8f8a2-17e7-49a9-8390-22f3c8f42b39"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -60513,12 +60527,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7CBF6B91-9305-4674-87E0-A56D6B941238}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BA99F9FA-472B-49CB-8CD8-32BE0FD0DC5E}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="e658002f-fdfe-4e4b-94aa-0526ee42a8ac"/>
-    <ds:schemaRef ds:uri="4ad8f8a2-17e7-49a9-8390-22f3c8f42b39"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
ocp in reference class working
</commit_message>
<xml_diff>
--- a/IVM6311_Testing_scripts.xlsx
+++ b/IVM6311_Testing_scripts.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\invlab\Documents\IVM6311ATE\IVM6311ATE\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A26F310-6443-4D4E-9E96-ED092065E451}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E4704FF-0CA1-4808-AD66-ECCA7DF3C725}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="693" firstSheet="1" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -44622,6 +44622,9 @@
     </r>
   </si>
   <si>
+    <t>ADDED POST TRIMMING FOR BST_OCP_TRIM</t>
+  </si>
+  <si>
     <r>
       <t xml:space="preserve">Run__startup
 Run__Boost_test_default
@@ -44975,7 +44978,7 @@
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve">
-TrimSweep__</t>
+TrimSweep__0xB1[3:0]</t>
     </r>
     <r>
       <rPr>
@@ -44984,7 +44987,7 @@
         <rFont val="Calibri"/>
         <scheme val="minor"/>
       </rPr>
-      <t>0xB2[5]__0xB1[3:0]</t>
+      <t>__0xB2[5]</t>
     </r>
     <r>
       <rPr>
@@ -45081,9 +45084,6 @@
       <t xml:space="preserve">
 </t>
     </r>
-  </si>
-  <si>
-    <t>ADDED POST TRIMMING FOR BST_OCP_TRIM</t>
   </si>
 </sst>
 </file>
@@ -48486,10 +48486,10 @@
         <v>400</v>
       </c>
       <c r="F5" s="189" t="s">
+        <v>436</v>
+      </c>
+      <c r="G5" t="s">
         <v>435</v>
-      </c>
-      <c r="G5" t="s">
-        <v>436</v>
       </c>
       <c r="I5" s="234"/>
     </row>
@@ -60260,12 +60260,14 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="e658002f-fdfe-4e4b-94aa-0526ee42a8ac">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="4ad8f8a2-17e7-49a9-8390-22f3c8f42b39" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -60486,20 +60488,21 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="e658002f-fdfe-4e4b-94aa-0526ee42a8ac">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="4ad8f8a2-17e7-49a9-8390-22f3c8f42b39" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BA99F9FA-472B-49CB-8CD8-32BE0FD0DC5E}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7CBF6B91-9305-4674-87E0-A56D6B941238}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="e658002f-fdfe-4e4b-94aa-0526ee42a8ac"/>
+    <ds:schemaRef ds:uri="4ad8f8a2-17e7-49a9-8390-22f3c8f42b39"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -60524,12 +60527,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7CBF6B91-9305-4674-87E0-A56D6B941238}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BA99F9FA-472B-49CB-8CD8-32BE0FD0DC5E}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="e658002f-fdfe-4e4b-94aa-0526ee42a8ac"/>
-    <ds:schemaRef ds:uri="4ad8f8a2-17e7-49a9-8390-22f3c8f42b39"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Reference_class is working!, trimming i sodne, missed only the burnt of the register
</commit_message>
<xml_diff>
--- a/IVM6311_Testing_scripts.xlsx
+++ b/IVM6311_Testing_scripts.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\invlab\Documents\IVM6311ATE\IVM6311ATE\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E4704FF-0CA1-4808-AD66-ECCA7DF3C725}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D6372C26-B086-47B0-899B-4F97DAC573BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="693" firstSheet="1" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -60260,14 +60260,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="e658002f-fdfe-4e4b-94aa-0526ee42a8ac">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="4ad8f8a2-17e7-49a9-8390-22f3c8f42b39" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -60488,21 +60486,20 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="e658002f-fdfe-4e4b-94aa-0526ee42a8ac">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="4ad8f8a2-17e7-49a9-8390-22f3c8f42b39" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7CBF6B91-9305-4674-87E0-A56D6B941238}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BA99F9FA-472B-49CB-8CD8-32BE0FD0DC5E}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="e658002f-fdfe-4e4b-94aa-0526ee42a8ac"/>
-    <ds:schemaRef ds:uri="4ad8f8a2-17e7-49a9-8390-22f3c8f42b39"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -60527,9 +60524,12 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BA99F9FA-472B-49CB-8CD8-32BE0FD0DC5E}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7CBF6B91-9305-4674-87E0-A56D6B941238}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="e658002f-fdfe-4e4b-94aa-0526ee42a8ac"/>
+    <ds:schemaRef ds:uri="4ad8f8a2-17e7-49a9-8390-22f3c8f42b39"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
working on burning trimming procedure
</commit_message>
<xml_diff>
--- a/IVM6311_Testing_scripts.xlsx
+++ b/IVM6311_Testing_scripts.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\invlab\Documents\IVM6311ATE\IVM6311ATE\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C3C9FDD0-F65B-45CE-B3A7-D65815FC6E97}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB855E87-CA17-4C25-9DC6-E67C8CF427C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="693" firstSheet="1" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -60194,12 +60194,14 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="e658002f-fdfe-4e4b-94aa-0526ee42a8ac">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="4ad8f8a2-17e7-49a9-8390-22f3c8f42b39" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -60420,20 +60422,21 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="e658002f-fdfe-4e4b-94aa-0526ee42a8ac">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="4ad8f8a2-17e7-49a9-8390-22f3c8f42b39" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BA99F9FA-472B-49CB-8CD8-32BE0FD0DC5E}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7CBF6B91-9305-4674-87E0-A56D6B941238}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="e658002f-fdfe-4e4b-94aa-0526ee42a8ac"/>
+    <ds:schemaRef ds:uri="4ad8f8a2-17e7-49a9-8390-22f3c8f42b39"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -60458,12 +60461,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7CBF6B91-9305-4674-87E0-A56D6B941238}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BA99F9FA-472B-49CB-8CD8-32BE0FD0DC5E}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="e658002f-fdfe-4e4b-94aa-0526ee42a8ac"/>
-    <ds:schemaRef ds:uri="4ad8f8a2-17e7-49a9-8390-22f3c8f42b39"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
modified bst_ocp_procedure, remove 0x1A 0x00 and 0x19 cause i lost the communication
</commit_message>
<xml_diff>
--- a/IVM6311_Testing_scripts.xlsx
+++ b/IVM6311_Testing_scripts.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\invlab\Documents\IVM6311ATE\IVM6311ATE\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{23DBA5C6-FFE7-411E-9F94-D6B7E69A0DDA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9599AE53-6FED-495A-BA28-D010A9D65906}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="693" firstSheet="1" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -43011,467 +43011,6 @@
     <t>ADDED POST TRIMMING FOR BST_OCP_TRIM</t>
   </si>
   <si>
-    <r>
-      <t xml:space="preserve">Run__startup
-Run__Boost_test_default
-Run__Enable_Ana_Testpoint
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF7030A0"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Wait__delay__0.1ms</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FFFF3399"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF4472C4"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>0xFE_0x00</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> "Select page 0"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF4472C4"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>0xB0[1]_0x01</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> "ocp en
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF4472C4"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>0xB2[1]_0x01</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> "ls_sel on"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF4472C4"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>0xC0[2:0]_0x01</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> "OCP threshold set to 400mA"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF4472C4"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">0xFE_0x01 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">"Select page 1"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF4472C4"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>0x1A_0x10</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> "TSW to OCP Sense"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0070C0"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">0x03_0x07 </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">"FSYN testpoint enable"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0070C0"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">0x04_0x18 </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>"FSYN = ana_bst_ocp_1"</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FFFF3399"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF7030A0"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Wait__delay__0.1ms</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF4472C4"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-0xFE_0x00</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> "Select page 0"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF4472C4"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>0xB2[0]_0x01</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> "Power Force en"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF4472C4"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>0xFE_0x01</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> "Select page 1"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0070C0"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>0x0F_0x80
-0xB0_0x0E</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF7030A0"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">Wait__delay__0.1ms
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF4472C4"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>0x15[2]_0x01</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> "Force ocp"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF4472C4"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>0x19[1]_0x01</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> "bst_test en"</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF7030A0"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-Wait__delay__0.1ms</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF00B050"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-Force__SW__200mA</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF9BC2E6"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-TrimSweep__0xB1[3:0]</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FFC65911"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>__0xB2[5]</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF9BC2E6"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>"</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FFED7D31"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>trim in 2 different registers - Sweep codes starting from b0000,1111 to b0000,0000 than from b0001,1111 to b0001,0000</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>"</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FFFF3399"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF00B050"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Measure_Voltage_FSYN</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> "Check the transition Low to High"</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FFFF3399"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF4472C4"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">0x1A_0x00
-0x19_0x00
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FFC65911"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-  </si>
-  <si>
     <t xml:space="preserve">Run__Startup
 Run__Enable_Ana_Testpoint
 0xFE_0x01 "Select page 1"
@@ -45046,6 +44585,456 @@
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve">Measure__Voltage_SDWN  </t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Run__startup
+Run__Boost_test_default
+Run__Enable_Ana_Testpoint
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF7030A0"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Wait__delay__0.1ms</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF3399"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF4472C4"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>0xFE_0x00</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> "Select page 0"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF4472C4"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>0xB0[1]_0x01</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> "ocp en
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF4472C4"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>0xB2[1]_0x01</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> "ls_sel on"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF4472C4"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>0xC0[2:0]_0x01</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> "OCP threshold set to 400mA"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF4472C4"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">0xFE_0x01 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">"Select page 1"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF4472C4"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>0x1A_0x10</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> "TSW to OCP Sense"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0070C0"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">0x03_0x07 </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">"FSYN testpoint enable"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0070C0"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">0x04_0x18 </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>"FSYN = ana_bst_ocp_1"</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF3399"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF7030A0"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Wait__delay__0.1ms</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF4472C4"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+0xFE_0x00</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> "Select page 0"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF4472C4"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>0xB2[0]_0x01</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> "Power Force en"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF4472C4"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>0xFE_0x01</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> "Select page 1"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0070C0"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>0x0F_0x80
+0xB0_0x0E</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF7030A0"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Wait__delay__0.1ms
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF4472C4"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>0x15[2]_0x01</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> "Force ocp"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF4472C4"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>0x19[1]_0x01</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> "bst_test en"</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF7030A0"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Wait__delay__0.1ms</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF00B050"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Force__SW__200mA</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF9BC2E6"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+TrimSweep__0xB1[3:0]</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFC65911"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>__0xB2[5]</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF9BC2E6"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>"</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFED7D31"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>trim in 2 different registers - Sweep codes starting from b0000,1111 to b0000,0000 than from b0001,1111 to b0001,0000</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>"</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF3399"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF00B050"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Measure_Voltage_FSYN</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> "Check the transition Low to High"</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF3399"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFC65911"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">0xFE_0x00 "Select page 0"
+</t>
     </r>
   </si>
 </sst>
@@ -48411,16 +48400,16 @@
       <c r="A5" s="240"/>
       <c r="B5" s="241"/>
       <c r="C5" s="204" t="s">
+        <v>425</v>
+      </c>
+      <c r="D5" s="204" t="s">
         <v>426</v>
       </c>
-      <c r="D5" s="204" t="s">
+      <c r="E5" s="204" t="s">
         <v>427</v>
       </c>
-      <c r="E5" s="204" t="s">
-        <v>428</v>
-      </c>
       <c r="F5" s="189" t="s">
-        <v>425</v>
+        <v>436</v>
       </c>
       <c r="G5" t="s">
         <v>424</v>
@@ -58312,31 +58301,31 @@
         <v>383</v>
       </c>
       <c r="D5" s="56" t="s">
+        <v>431</v>
+      </c>
+      <c r="E5" s="56" t="s">
+        <v>430</v>
+      </c>
+      <c r="F5" s="56" t="s">
+        <v>428</v>
+      </c>
+      <c r="G5" s="56" t="s">
+        <v>429</v>
+      </c>
+      <c r="H5" s="56" t="s">
         <v>432</v>
-      </c>
-      <c r="E5" s="56" t="s">
-        <v>431</v>
-      </c>
-      <c r="F5" s="56" t="s">
-        <v>429</v>
-      </c>
-      <c r="G5" s="56" t="s">
-        <v>430</v>
-      </c>
-      <c r="H5" s="56" t="s">
-        <v>433</v>
       </c>
       <c r="I5" s="37" t="s">
         <v>382</v>
       </c>
       <c r="J5" s="56" t="s">
+        <v>433</v>
+      </c>
+      <c r="K5" s="56" t="s">
         <v>434</v>
       </c>
-      <c r="K5" s="56" t="s">
+      <c r="L5" s="56" t="s">
         <v>435</v>
-      </c>
-      <c r="L5" s="56" t="s">
-        <v>436</v>
       </c>
       <c r="M5" s="56"/>
     </row>
@@ -60194,6 +60183,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="e658002f-fdfe-4e4b-94aa-0526ee42a8ac">
@@ -60202,15 +60200,6 @@
     <TaxCatchAll xmlns="4ad8f8a2-17e7-49a9-8390-22f3c8f42b39" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -60431,20 +60420,20 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BA99F9FA-472B-49CB-8CD8-32BE0FD0DC5E}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7CBF6B91-9305-4674-87E0-A56D6B941238}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
     <ds:schemaRef ds:uri="e658002f-fdfe-4e4b-94aa-0526ee42a8ac"/>
     <ds:schemaRef ds:uri="4ad8f8a2-17e7-49a9-8390-22f3c8f42b39"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BA99F9FA-472B-49CB-8CD8-32BE0FD0DC5E}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
trimming and az_comp working, added also script for saving
</commit_message>
<xml_diff>
--- a/IVM6311_Testing_scripts.xlsx
+++ b/IVM6311_Testing_scripts.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\invlab\Documents\IVM6311ATE\IVM6311ATE\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7F8A9ED-E72F-4F8F-93F9-8D1250414E55}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7FAD2F45-D596-40C0-B041-D90B1BDA6164}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="693" firstSheet="1" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="693" firstSheet="1" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Revision" sheetId="3" r:id="rId1"/>
@@ -60183,6 +60183,26 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="e658002f-fdfe-4e4b-94aa-0526ee42a8ac">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="4ad8f8a2-17e7-49a9-8390-22f3c8f42b39" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x010100C9B53A5B1F235B4EBDF9F22062DFC34D" ma:contentTypeVersion="12" ma:contentTypeDescription="Creare un nuovo documento." ma:contentTypeScope="" ma:versionID="ad5b12d537450e73edf2af95672e184c">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="e658002f-fdfe-4e4b-94aa-0526ee42a8ac" xmlns:ns3="4ad8f8a2-17e7-49a9-8390-22f3c8f42b39" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="ac16958afaf1bb0d1dccad67078e8e2c" ns2:_="" ns3:_="">
     <xsd:import namespace="e658002f-fdfe-4e4b-94aa-0526ee42a8ac"/>
@@ -60399,27 +60419,26 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="e658002f-fdfe-4e4b-94aa-0526ee42a8ac">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="4ad8f8a2-17e7-49a9-8390-22f3c8f42b39" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BA99F9FA-472B-49CB-8CD8-32BE0FD0DC5E}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7CBF6B91-9305-4674-87E0-A56D6B941238}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="e658002f-fdfe-4e4b-94aa-0526ee42a8ac"/>
+    <ds:schemaRef ds:uri="4ad8f8a2-17e7-49a9-8390-22f3c8f42b39"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{31D0029D-E8A7-4DC9-B140-19D450DFB7E0}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -60436,23 +60455,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7CBF6B91-9305-4674-87E0-A56D6B941238}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="e658002f-fdfe-4e4b-94aa-0526ee42a8ac"/>
-    <ds:schemaRef ds:uri="4ad8f8a2-17e7-49a9-8390-22f3c8f42b39"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BA99F9FA-472B-49CB-8CD8-32BE0FD0DC5E}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
first test boost working again
</commit_message>
<xml_diff>
--- a/IVM6311_Testing_scripts.xlsx
+++ b/IVM6311_Testing_scripts.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\invlab\Documents\IVM6311ATE\IVM6311ATE\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2BD06F0F-ADD1-48F4-A85E-4991CB11D815}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC2F92F1-58A8-49C9-8934-58C5D366122B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="693" firstSheet="1" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="693" firstSheet="1" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Revision" sheetId="3" r:id="rId1"/>
@@ -31921,1424 +31921,6 @@
         <sz val="11"/>
         <color rgb="FFFF3399"/>
         <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Run_startup
-Run_Boost_test_default
-Enable_Ana_Testpoint</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF4472C4"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>0xFE_0x00</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> "Select page 0"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF4472C4"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>0xB0_0x00</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> "en 1 bst low"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF4472C4"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>0xB1_0x00</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> "en 2 bst low"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF4472C4"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>0xB3[4:3]_0x00</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> "en 3 bst low"</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF4472C4"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-0xFE_0x01</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> "Select page 1"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF4472C4"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>0x1A_0x00</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> "TSW_Mirr test"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF4472C4"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>0x18[6]_0x01</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> "Enable Mirr"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF4472C4"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>0x17[6]_0x01</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> "Force Mirr"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FFFF3399"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Force__SDWN__0.6V</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF7030A0"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Wait__delay__0.1ms</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF4472C4"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>0x19[1]_0x01</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> "bst_test_en 1"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF7030A0"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Wait__delay__0.1ms</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF70AD47"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Measure__Current__SDWN</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> "tswitch mirr measure"
-</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FFFF3399"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Run_startup
-Run_Boost_test_default
-Enable_Ana_Testpoint</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF4472C4"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-0xFE_0x00</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> "Select page 0"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF4472C4"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>0xB0_0x00</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> "en 1 bst low"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF4472C4"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>0xB1_0x00</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> "en 2 bst low"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF4472C4"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>0xB3[4:3]_0x00</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> "en 3 bst low"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF4472C4"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>0x18[6]_0x01</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> "Enable Mirr"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF4472C4"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>0xB1[6]_0x01</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> "Bootstrap en"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF4472C4"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>0xB2[1]_0x00</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> "ls_sel off"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF4472C4"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>0xB4[2:0]_0x00</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> "hsa_hsb_byp off"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF4472C4"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>0xFE_0x01</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> "Select page 1"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF4472C4"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">0x17[6]_0x01 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">"Force Mirr"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF4472C4"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>0x16[6]_0x01</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> "Force Bootstrap"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF7030A0"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Wait__delay__0.1ms</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF4472C4"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>0x1A_0x01</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> "TSwitch SW"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF4472C4"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>0xFE_0x00</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> "Select page 0"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF4472C4"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>0xB2[1]_0x01</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> "ls_sel on"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF4472C4"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>0xB2[0]_0x01</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> "Power Force en"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF4472C4"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>0xFE_0x01</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> "Select page 1"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF7030A0"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Wait__delay__0.1ms</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF4472C4"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>0x19[1]_0x01</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> "bst_test en"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FFFF3399"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Force__SW__400mA</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> "</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FFFFC000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>chiedere comando corrente</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF7030A0"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Wait__delay__0.1ms</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF70AD47"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">Measure__Voltage__SDWN
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF4472C4"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>0x1A_0x02</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> "TSwitch PGND"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF70AD47"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Measure__Voltage__SDWN
-Calculate__diff__RONLS</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF4472C4"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">0x1A_0x00
-0x19_0x00
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FFFF3399"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Run_startup
-Run_Boost_test_default
-Enable_Ana_Testpoint
-Force__VBAT__5V
-Force__VDDIO__1.8V
-Force__VDD__1.8V
-Force__VBIAS__6V
-Force__VBSO__4.3V</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF4472C4"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">0xFE_0x00 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">"Select page 0"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF4472C4"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>0x00_0x0F</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> "Power-up"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF4472C4"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>0xB0_0x00</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> "en 1 bst low"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF4472C4"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>0xB1_0x00</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> "en 2 bst low"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF4472C4"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>0xB3[4:3]_0x00</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> "en 3 bst low"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF4472C4"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>0x18[6]_0x01</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> "Enable Mirr"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF4472C4"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>0xFE_0x00</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> "Select page 0"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF4472C4"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>0xB1[6]_0x01</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> "Bootstrap en"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF4472C4"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>0xB2[1]_0x00</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> "ls_sel off"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF4472C4"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>0xB4[2:0]_0x06</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> "hsa_hsb on byp off"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF4472C4"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>0xFE_0x01</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> "Select page 1"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF4472C4"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>0x1A_0x01</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> "TSwitch SW"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF4472C4"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>0x17[6]_0x01</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> "Force Mirr" 
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF4472C4"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>0x16[6]_0x01</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> "Force Bootstrap"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF7030A0"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Wait__delay__0.1ms</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF4472C4"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>0xFE_0x00</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> "Select page 0"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF4472C4"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>0xB2[0]_0x01</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> "Power Force en"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF4472C4"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>0xFE_0x01</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> "Select page 1"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF7030A0"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Wait__delay__0.1ms</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF4472C4"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>0x19[1]_0x01</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> "bst_test en"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF7030A0"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Wait__delay__0.1ms</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FFFF3399"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Force__SW__-100mA</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> "</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FFFFC000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>sink current -100mA</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">"
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF7030A0"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">Wait__delay__0.1ms
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF92D050"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Measure__Voltage__SDWN
-Measure__Voltage__VBSO</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF4472C4"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF92D050"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Calculate__diff__RONHS</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF4472C4"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-0x1A_0x00
-0x19_0x00</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FFFF3399"/>
-        <rFont val="Calibri"/>
         <scheme val="minor"/>
       </rPr>
       <t>Run_startup
@@ -44772,6 +43354,1424 @@
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> "Force Bootstrap"</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF3399"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Run_startup
+Run_Boost_test_default
+Run_Enable_Ana_Testpoint</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF4472C4"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+0xFE_0x00</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> "Select page 0"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF4472C4"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>0xB0_0x00</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> "en 1 bst low"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF4472C4"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>0xB1_0x00</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> "en 2 bst low"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF4472C4"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>0xB3[4:3]_0x00</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> "en 3 bst low"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF4472C4"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>0x18[6]_0x01</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> "Enable Mirr"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF4472C4"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>0xB1[6]_0x01</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> "Bootstrap en"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF4472C4"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>0xB2[1]_0x00</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> "ls_sel off"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF4472C4"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>0xB4[2:0]_0x00</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> "hsa_hsb_byp off"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF4472C4"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>0xFE_0x01</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> "Select page 1"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF4472C4"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">0x17[6]_0x01 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">"Force Mirr"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF4472C4"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>0x16[6]_0x01</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> "Force Bootstrap"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF7030A0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Wait__delay__0.1ms</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF4472C4"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>0x1A_0x01</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> "TSwitch SW"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF4472C4"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>0xFE_0x00</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> "Select page 0"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF4472C4"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>0xB2[1]_0x01</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> "ls_sel on"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF4472C4"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>0xB2[0]_0x01</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> "Power Force en"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF4472C4"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>0xFE_0x01</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> "Select page 1"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF7030A0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Wait__delay__0.1ms</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF4472C4"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>0x19[1]_0x01</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> "bst_test en"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF3399"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Force__SW__400mA</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> "</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFFC000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>chiedere comando corrente</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF7030A0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Wait__delay__0.1ms</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF70AD47"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Measure__Voltage__SDWN
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF4472C4"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>0x1A_0x02</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> "TSwitch PGND"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF70AD47"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Measure__Voltage__SDWN
+Calculate__diff__RONLS</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF4472C4"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">0x1A_0x00
+0x19_0x00
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF3399"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Run_startup
+Run_Boost_test_default
+Run_Enable_Ana_Testpoint</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF4472C4"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>0xFE_0x00</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> "Select page 0"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF4472C4"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>0xB0_0x00</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> "en 1 bst low"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF4472C4"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>0xB1_0x00</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> "en 2 bst low"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF4472C4"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>0xB3[4:3]_0x00</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> "en 3 bst low"</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF4472C4"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+0xFE_0x01</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> "Select page 1"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF4472C4"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>0x1A_0x00</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> "TSW_Mirr test"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF4472C4"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>0x18[6]_0x01</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> "Enable Mirr"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF4472C4"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>0x17[6]_0x01</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> "Force Mirr"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF3399"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Force__SDWN__0.6V</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF7030A0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Wait__delay__0.1ms</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF4472C4"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>0x19[1]_0x01</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> "bst_test_en 1"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF7030A0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Wait__delay__0.1ms</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF70AD47"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Measure__Current__SDWN</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> "tswitch mirr measure"
+</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF3399"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Run_startup
+Run_Boost_test_default
+Run_Enable_Ana_Testpoint
+Force__VBAT__5V
+Force__VDDIO__1.8V
+Force__VDD__1.8V
+Force__VBIAS__6V
+Force__VBSO__4.3V</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF4472C4"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">0xFE_0x00 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">"Select page 0"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF4472C4"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>0x00_0x0F</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> "Power-up"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF4472C4"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>0xB0_0x00</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> "en 1 bst low"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF4472C4"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>0xB1_0x00</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> "en 2 bst low"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF4472C4"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>0xB3[4:3]_0x00</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> "en 3 bst low"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF4472C4"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>0x18[6]_0x01</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> "Enable Mirr"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF4472C4"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>0xFE_0x00</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> "Select page 0"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF4472C4"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>0xB1[6]_0x01</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> "Bootstrap en"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF4472C4"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>0xB2[1]_0x00</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> "ls_sel off"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF4472C4"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>0xB4[2:0]_0x06</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> "hsa_hsb on byp off"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF4472C4"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>0xFE_0x01</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> "Select page 1"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF4472C4"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>0x1A_0x01</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> "TSwitch SW"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF4472C4"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>0x17[6]_0x01</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> "Force Mirr" 
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF4472C4"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>0x16[6]_0x01</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> "Force Bootstrap"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF7030A0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Wait__delay__0.1ms</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF4472C4"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>0xFE_0x00</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> "Select page 0"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF4472C4"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>0xB2[0]_0x01</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> "Power Force en"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF4472C4"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>0xFE_0x01</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> "Select page 1"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF7030A0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Wait__delay__0.1ms</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF4472C4"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>0x19[1]_0x01</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> "bst_test en"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF7030A0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Wait__delay__0.1ms</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF3399"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Force__SW__-100mA</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> "</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFFC000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>sink current -100mA</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF7030A0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Wait__delay__0.1ms
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF92D050"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Measure__Voltage__SDWN
+Measure__Voltage__VBSO</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF4472C4"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF92D050"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Calculate__diff__RONHS</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF4472C4"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+0x1A_0x00
+0x19_0x00</t>
     </r>
   </si>
 </sst>
@@ -51458,85 +51458,85 @@
       <c r="A5" s="245"/>
       <c r="B5" s="245"/>
       <c r="C5" s="183" t="s">
+        <v>435</v>
+      </c>
+      <c r="D5" s="183" t="s">
+        <v>434</v>
+      </c>
+      <c r="E5" s="183" t="s">
+        <v>436</v>
+      </c>
+      <c r="F5" s="221" t="s">
         <v>410</v>
       </c>
-      <c r="D5" s="183" t="s">
+      <c r="G5" s="183" t="s">
         <v>411</v>
       </c>
-      <c r="E5" s="183" t="s">
+      <c r="H5" s="189" t="s">
         <v>412</v>
       </c>
-      <c r="F5" s="221" t="s">
+      <c r="I5" s="189" t="s">
         <v>413</v>
       </c>
-      <c r="G5" s="183" t="s">
+      <c r="J5" s="189" t="s">
         <v>414</v>
       </c>
-      <c r="H5" s="189" t="s">
+      <c r="K5" s="189" t="s">
         <v>415</v>
       </c>
-      <c r="I5" s="189" t="s">
+      <c r="L5" s="221" t="s">
         <v>416</v>
       </c>
-      <c r="J5" s="189" t="s">
+      <c r="M5" s="221" t="s">
         <v>417</v>
       </c>
-      <c r="K5" s="189" t="s">
+      <c r="N5" s="183" t="s">
         <v>418</v>
       </c>
-      <c r="L5" s="221" t="s">
+      <c r="O5" s="221" t="s">
         <v>419</v>
       </c>
-      <c r="M5" s="221" t="s">
+      <c r="P5" s="221" t="s">
         <v>420</v>
       </c>
-      <c r="N5" s="183" t="s">
+      <c r="Q5" s="221" t="s">
         <v>421</v>
       </c>
-      <c r="O5" s="221" t="s">
+      <c r="R5" s="221" t="s">
         <v>422</v>
       </c>
-      <c r="P5" s="221" t="s">
+      <c r="S5" s="189" t="s">
         <v>423</v>
       </c>
-      <c r="Q5" s="221" t="s">
+      <c r="T5" s="189" t="s">
         <v>424</v>
       </c>
-      <c r="R5" s="221" t="s">
+      <c r="U5" s="189" t="s">
         <v>425</v>
       </c>
-      <c r="S5" s="189" t="s">
+      <c r="V5" s="189" t="s">
         <v>426</v>
       </c>
-      <c r="T5" s="189" t="s">
+      <c r="W5" s="190" t="s">
         <v>427</v>
       </c>
-      <c r="U5" s="189" t="s">
+      <c r="X5" s="190" t="s">
         <v>428</v>
-      </c>
-      <c r="V5" s="189" t="s">
-        <v>429</v>
-      </c>
-      <c r="W5" s="190" t="s">
-        <v>430</v>
-      </c>
-      <c r="X5" s="190" t="s">
-        <v>431</v>
       </c>
       <c r="Y5" s="190" t="s">
         <v>230</v>
       </c>
       <c r="Z5" s="190" t="s">
+        <v>429</v>
+      </c>
+      <c r="AA5" s="189" t="s">
+        <v>430</v>
+      </c>
+      <c r="AB5" s="189" t="s">
+        <v>431</v>
+      </c>
+      <c r="AC5" s="221" t="s">
         <v>432</v>
-      </c>
-      <c r="AA5" s="189" t="s">
-        <v>433</v>
-      </c>
-      <c r="AB5" s="189" t="s">
-        <v>434</v>
-      </c>
-      <c r="AC5" s="221" t="s">
-        <v>435</v>
       </c>
     </row>
     <row r="6" spans="1:29" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -59886,7 +59886,7 @@
         <v>316</v>
       </c>
       <c r="E2" s="224" t="s">
-        <v>436</v>
+        <v>433</v>
       </c>
       <c r="F2" s="83" t="s">
         <v>317</v>
@@ -59920,6 +59920,26 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="e658002f-fdfe-4e4b-94aa-0526ee42a8ac">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="4ad8f8a2-17e7-49a9-8390-22f3c8f42b39" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x010100C9B53A5B1F235B4EBDF9F22062DFC34D" ma:contentTypeVersion="12" ma:contentTypeDescription="Creare un nuovo documento." ma:contentTypeScope="" ma:versionID="ad5b12d537450e73edf2af95672e184c">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="e658002f-fdfe-4e4b-94aa-0526ee42a8ac" xmlns:ns3="4ad8f8a2-17e7-49a9-8390-22f3c8f42b39" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="ac16958afaf1bb0d1dccad67078e8e2c" ns2:_="" ns3:_="">
     <xsd:import namespace="e658002f-fdfe-4e4b-94aa-0526ee42a8ac"/>
@@ -60136,27 +60156,26 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="e658002f-fdfe-4e4b-94aa-0526ee42a8ac">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="4ad8f8a2-17e7-49a9-8390-22f3c8f42b39" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BA99F9FA-472B-49CB-8CD8-32BE0FD0DC5E}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7CBF6B91-9305-4674-87E0-A56D6B941238}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="e658002f-fdfe-4e4b-94aa-0526ee42a8ac"/>
+    <ds:schemaRef ds:uri="4ad8f8a2-17e7-49a9-8390-22f3c8f42b39"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{31D0029D-E8A7-4DC9-B140-19D450DFB7E0}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -60173,23 +60192,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7CBF6B91-9305-4674-87E0-A56D6B941238}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="e658002f-fdfe-4e4b-94aa-0526ee42a8ac"/>
-    <ds:schemaRef ds:uri="4ad8f8a2-17e7-49a9-8390-22f3c8f42b39"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BA99F9FA-472B-49CB-8CD8-32BE0FD0DC5E}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
working on boost on the boost_class
</commit_message>
<xml_diff>
--- a/IVM6311_Testing_scripts.xlsx
+++ b/IVM6311_Testing_scripts.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\invlab\Documents\IVM6311ATE\IVM6311ATE\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E56DFE1D-E013-4441-9FDC-538130888A70}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F26A290A-BAEC-4279-B8BE-3C1AE32B7F8A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="693" firstSheet="1" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -60158,26 +60158,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="e658002f-fdfe-4e4b-94aa-0526ee42a8ac">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="4ad8f8a2-17e7-49a9-8390-22f3c8f42b39" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x010100C9B53A5B1F235B4EBDF9F22062DFC34D" ma:contentTypeVersion="12" ma:contentTypeDescription="Creare un nuovo documento." ma:contentTypeScope="" ma:versionID="ad5b12d537450e73edf2af95672e184c">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="e658002f-fdfe-4e4b-94aa-0526ee42a8ac" xmlns:ns3="4ad8f8a2-17e7-49a9-8390-22f3c8f42b39" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="ac16958afaf1bb0d1dccad67078e8e2c" ns2:_="" ns3:_="">
     <xsd:import namespace="e658002f-fdfe-4e4b-94aa-0526ee42a8ac"/>
@@ -60394,10 +60374,41 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="e658002f-fdfe-4e4b-94aa-0526ee42a8ac">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="4ad8f8a2-17e7-49a9-8390-22f3c8f42b39" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BA99F9FA-472B-49CB-8CD8-32BE0FD0DC5E}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{31D0029D-E8A7-4DC9-B140-19D450DFB7E0}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="e658002f-fdfe-4e4b-94aa-0526ee42a8ac"/>
+    <ds:schemaRef ds:uri="4ad8f8a2-17e7-49a9-8390-22f3c8f42b39"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -60414,20 +60425,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{31D0029D-E8A7-4DC9-B140-19D450DFB7E0}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BA99F9FA-472B-49CB-8CD8-32BE0FD0DC5E}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="e658002f-fdfe-4e4b-94aa-0526ee42a8ac"/>
-    <ds:schemaRef ds:uri="4ad8f8a2-17e7-49a9-8390-22f3c8f42b39"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
all the tests of the boost singularly are working
</commit_message>
<xml_diff>
--- a/IVM6311_Testing_scripts.xlsx
+++ b/IVM6311_Testing_scripts.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\invlab\Documents\IVM6311ATE\IVM6311ATE\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9833F347-F349-41A5-9FC1-D96A9A3DA879}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{121782B0-F185-43B3-BF77-2793D7ED7A30}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="693" firstSheet="1" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -60166,6 +60166,26 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="e658002f-fdfe-4e4b-94aa-0526ee42a8ac">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="4ad8f8a2-17e7-49a9-8390-22f3c8f42b39" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x010100C9B53A5B1F235B4EBDF9F22062DFC34D" ma:contentTypeVersion="12" ma:contentTypeDescription="Creare un nuovo documento." ma:contentTypeScope="" ma:versionID="ad5b12d537450e73edf2af95672e184c">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="e658002f-fdfe-4e4b-94aa-0526ee42a8ac" xmlns:ns3="4ad8f8a2-17e7-49a9-8390-22f3c8f42b39" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="ac16958afaf1bb0d1dccad67078e8e2c" ns2:_="" ns3:_="">
     <xsd:import namespace="e658002f-fdfe-4e4b-94aa-0526ee42a8ac"/>
@@ -60382,27 +60402,26 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="e658002f-fdfe-4e4b-94aa-0526ee42a8ac">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="4ad8f8a2-17e7-49a9-8390-22f3c8f42b39" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BA99F9FA-472B-49CB-8CD8-32BE0FD0DC5E}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7CBF6B91-9305-4674-87E0-A56D6B941238}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="e658002f-fdfe-4e4b-94aa-0526ee42a8ac"/>
+    <ds:schemaRef ds:uri="4ad8f8a2-17e7-49a9-8390-22f3c8f42b39"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{31D0029D-E8A7-4DC9-B140-19D450DFB7E0}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -60419,23 +60438,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7CBF6B91-9305-4674-87E0-A56D6B941238}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="e658002f-fdfe-4e4b-94aa-0526ee42a8ac"/>
-    <ds:schemaRef ds:uri="4ad8f8a2-17e7-49a9-8390-22f3c8f42b39"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BA99F9FA-472B-49CB-8CD8-32BE0FD0DC5E}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
working on zc boost, impementing ramp instruction
</commit_message>
<xml_diff>
--- a/IVM6311_Testing_scripts.xlsx
+++ b/IVM6311_Testing_scripts.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\invlab\Documents\IVM6311ATE\IVM6311ATE\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C800A2EA-36F5-4333-A658-3852D1CBAE92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{696A51F0-87F7-47F8-88C1-89377CAF7922}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="693" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -44990,7 +44990,7 @@
         <rFont val="Calibri"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve"> "inject"
+      <t xml:space="preserve">"inject"
 Wait__delay__0.1ms
 </t>
     </r>
@@ -45020,7 +45020,7 @@
         <family val="2"/>
       </rPr>
       <t xml:space="preserve">
-Ramp__SW__100mA__-100mA 
+Ramp__SW__100mA__-100mA
 </t>
     </r>
     <r>

</xml_diff>